<commit_message>
update whisp columns excel file
</commit_message>
<xml_diff>
--- a/whisp_columns.xlsx
+++ b/whisp_columns.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnell\Documents\GitHub\whisp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2CC6670-3A9C-4E9E-A550-7C0430EE1A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87BC43A7-E222-4A0F-9D82-753F6C558B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12420" xr2:uid="{FC85F32F-3F3C-476F-A445-BF878E774111}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1265" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1247" uniqueCount="314">
   <si>
     <t>Column name</t>
   </si>
@@ -281,12 +281,6 @@
     <t>Kalischek 2022</t>
   </si>
   <si>
-    <t>Cocoa_bnetd</t>
-  </si>
-  <si>
-    <t>BNETD 2024</t>
-  </si>
-  <si>
     <t>Rubber_FDaP</t>
   </si>
   <si>
@@ -758,15 +752,6 @@
     <t>RADD_after_2020</t>
   </si>
   <si>
-    <t>DIST_after_2020</t>
-  </si>
-  <si>
-    <t>2023-2025</t>
-  </si>
-  <si>
-    <t>Hansen 2025</t>
-  </si>
-  <si>
     <t>GFT_primary</t>
   </si>
   <si>
@@ -860,9 +845,6 @@
     <t>Various national sources combined, date can vary</t>
   </si>
   <si>
-    <t>geojson</t>
-  </si>
-  <si>
     <t>Coordinates of the geometry</t>
   </si>
   <si>
@@ -993,6 +975,9 @@
   </si>
   <si>
     <t>treecover_after_2020</t>
+  </si>
+  <si>
+    <t>geo</t>
   </si>
 </sst>
 </file>
@@ -1384,7 +1369,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36A90905-187C-4727-AD42-76516A57CDD0}">
-  <dimension ref="A1:N198"/>
+  <dimension ref="A1:N196"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.7265625" bestFit="1" customWidth="1"/>
@@ -2088,7 +2073,7 @@
         <v>2020</v>
       </c>
       <c r="F17" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="G17" t="s">
         <v>19</v>
@@ -2252,7 +2237,7 @@
         <v>2020</v>
       </c>
       <c r="F21" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="G21" t="s">
         <v>19</v>
@@ -2278,7 +2263,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="B22" t="s">
         <v>15</v>
@@ -2287,13 +2272,13 @@
         <v>50</v>
       </c>
       <c r="D22" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="E22">
         <v>2020</v>
       </c>
       <c r="F22" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="G22" t="s">
         <v>19</v>
@@ -2334,7 +2319,7 @@
         <v>2020</v>
       </c>
       <c r="F23" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="G23" t="s">
         <v>19</v>
@@ -2410,13 +2395,13 @@
         <v>50</v>
       </c>
       <c r="D25" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E25">
         <v>2020</v>
       </c>
       <c r="F25" t="s">
-        <v>82</v>
+        <v>301</v>
       </c>
       <c r="G25" t="s">
         <v>19</v>
@@ -2451,13 +2436,13 @@
         <v>50</v>
       </c>
       <c r="D26" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E26">
         <v>2020</v>
       </c>
       <c r="F26" t="s">
-        <v>307</v>
+        <v>84</v>
       </c>
       <c r="G26" t="s">
         <v>19</v>
@@ -2492,13 +2477,13 @@
         <v>50</v>
       </c>
       <c r="D27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E27">
         <v>2020</v>
       </c>
       <c r="F27" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G27" t="s">
         <v>19</v>
@@ -2524,7 +2509,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B28" t="s">
         <v>15</v>
@@ -2533,34 +2518,24 @@
         <v>50</v>
       </c>
       <c r="D28" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E28">
-        <v>2020</v>
+        <v>2000</v>
       </c>
       <c r="F28" t="s">
-        <v>89</v>
-      </c>
-      <c r="G28" t="s">
-        <v>19</v>
+        <v>62</v>
       </c>
       <c r="H28" s="2">
-        <v>1</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I28" s="2"/>
       <c r="J28" s="2">
-        <v>1</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K28" s="2"/>
       <c r="L28" s="2">
-        <v>1</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
@@ -2574,10 +2549,10 @@
         <v>50</v>
       </c>
       <c r="D29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E29">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="F29" t="s">
         <v>62</v>
@@ -2596,7 +2571,7 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B30" t="s">
         <v>15</v>
@@ -2605,10 +2580,10 @@
         <v>50</v>
       </c>
       <c r="D30" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E30">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="F30" t="s">
         <v>62</v>
@@ -2627,7 +2602,7 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B31" t="s">
         <v>15</v>
@@ -2636,10 +2611,10 @@
         <v>50</v>
       </c>
       <c r="D31" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E31">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="F31" t="s">
         <v>62</v>
@@ -2658,7 +2633,7 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B32" t="s">
         <v>15</v>
@@ -2667,10 +2642,10 @@
         <v>50</v>
       </c>
       <c r="D32" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E32">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="F32" t="s">
         <v>62</v>
@@ -2689,7 +2664,7 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B33" t="s">
         <v>15</v>
@@ -2698,10 +2673,10 @@
         <v>50</v>
       </c>
       <c r="D33" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E33">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="F33" t="s">
         <v>62</v>
@@ -2720,7 +2695,7 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B34" t="s">
         <v>15</v>
@@ -2729,10 +2704,10 @@
         <v>50</v>
       </c>
       <c r="D34" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E34">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="F34" t="s">
         <v>62</v>
@@ -2751,7 +2726,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B35" t="s">
         <v>15</v>
@@ -2760,10 +2735,10 @@
         <v>50</v>
       </c>
       <c r="D35" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E35">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="F35" t="s">
         <v>62</v>
@@ -2782,7 +2757,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B36" t="s">
         <v>15</v>
@@ -2791,10 +2766,10 @@
         <v>50</v>
       </c>
       <c r="D36" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E36">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="F36" t="s">
         <v>62</v>
@@ -2813,7 +2788,7 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B37" t="s">
         <v>15</v>
@@ -2822,10 +2797,10 @@
         <v>50</v>
       </c>
       <c r="D37" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E37">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="F37" t="s">
         <v>62</v>
@@ -2844,7 +2819,7 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B38" t="s">
         <v>15</v>
@@ -2853,10 +2828,10 @@
         <v>50</v>
       </c>
       <c r="D38" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E38">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="F38" t="s">
         <v>62</v>
@@ -2875,7 +2850,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B39" t="s">
         <v>15</v>
@@ -2884,10 +2859,10 @@
         <v>50</v>
       </c>
       <c r="D39" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E39">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="F39" t="s">
         <v>62</v>
@@ -2906,7 +2881,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B40" t="s">
         <v>15</v>
@@ -2915,10 +2890,10 @@
         <v>50</v>
       </c>
       <c r="D40" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E40">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="F40" t="s">
         <v>62</v>
@@ -2937,7 +2912,7 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B41" t="s">
         <v>15</v>
@@ -2946,10 +2921,10 @@
         <v>50</v>
       </c>
       <c r="D41" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E41">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="F41" t="s">
         <v>62</v>
@@ -2968,7 +2943,7 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B42" t="s">
         <v>15</v>
@@ -2977,10 +2952,10 @@
         <v>50</v>
       </c>
       <c r="D42" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E42">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="F42" t="s">
         <v>62</v>
@@ -2999,7 +2974,7 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B43" t="s">
         <v>15</v>
@@ -3008,10 +2983,10 @@
         <v>50</v>
       </c>
       <c r="D43" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E43">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="F43" t="s">
         <v>62</v>
@@ -3030,7 +3005,7 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B44" t="s">
         <v>15</v>
@@ -3039,10 +3014,10 @@
         <v>50</v>
       </c>
       <c r="D44" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E44">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F44" t="s">
         <v>62</v>
@@ -3061,7 +3036,7 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B45" t="s">
         <v>15</v>
@@ -3070,10 +3045,10 @@
         <v>50</v>
       </c>
       <c r="D45" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E45">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F45" t="s">
         <v>62</v>
@@ -3092,7 +3067,7 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B46" t="s">
         <v>15</v>
@@ -3101,10 +3076,10 @@
         <v>50</v>
       </c>
       <c r="D46" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E46">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="F46" t="s">
         <v>62</v>
@@ -3123,7 +3098,7 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B47" t="s">
         <v>15</v>
@@ -3132,10 +3107,10 @@
         <v>50</v>
       </c>
       <c r="D47" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E47">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="F47" t="s">
         <v>62</v>
@@ -3154,7 +3129,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B48" t="s">
         <v>15</v>
@@ -3163,10 +3138,10 @@
         <v>50</v>
       </c>
       <c r="D48" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E48">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="F48" t="s">
         <v>62</v>
@@ -3185,7 +3160,7 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B49" t="s">
         <v>15</v>
@@ -3194,10 +3169,10 @@
         <v>50</v>
       </c>
       <c r="D49" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E49">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F49" t="s">
         <v>62</v>
@@ -3216,7 +3191,7 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B50" t="s">
         <v>15</v>
@@ -3225,10 +3200,10 @@
         <v>50</v>
       </c>
       <c r="D50" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E50">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="F50" t="s">
         <v>62</v>
@@ -3247,7 +3222,7 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B51" t="s">
         <v>15</v>
@@ -3256,10 +3231,10 @@
         <v>50</v>
       </c>
       <c r="D51" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E51">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F51" t="s">
         <v>62</v>
@@ -3278,7 +3253,7 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>114</v>
+        <v>300</v>
       </c>
       <c r="B52" t="s">
         <v>15</v>
@@ -3287,10 +3262,10 @@
         <v>50</v>
       </c>
       <c r="D52" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E52">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F52" t="s">
         <v>62</v>
@@ -3309,7 +3284,7 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>306</v>
+        <v>113</v>
       </c>
       <c r="B53" t="s">
         <v>15</v>
@@ -3318,10 +3293,10 @@
         <v>50</v>
       </c>
       <c r="D53" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="E53">
-        <v>2024</v>
+        <v>2000</v>
       </c>
       <c r="F53" t="s">
         <v>62</v>
@@ -3349,10 +3324,10 @@
         <v>50</v>
       </c>
       <c r="D54" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E54">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="F54" t="s">
         <v>62</v>
@@ -3371,7 +3346,7 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B55" t="s">
         <v>15</v>
@@ -3380,10 +3355,10 @@
         <v>50</v>
       </c>
       <c r="D55" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E55">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="F55" t="s">
         <v>62</v>
@@ -3402,7 +3377,7 @@
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B56" t="s">
         <v>15</v>
@@ -3411,10 +3386,10 @@
         <v>50</v>
       </c>
       <c r="D56" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E56">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="F56" t="s">
         <v>62</v>
@@ -3433,7 +3408,7 @@
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B57" t="s">
         <v>15</v>
@@ -3442,10 +3417,10 @@
         <v>50</v>
       </c>
       <c r="D57" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E57">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="F57" t="s">
         <v>62</v>
@@ -3464,7 +3439,7 @@
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B58" t="s">
         <v>15</v>
@@ -3473,10 +3448,10 @@
         <v>50</v>
       </c>
       <c r="D58" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E58">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="F58" t="s">
         <v>62</v>
@@ -3495,7 +3470,7 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B59" t="s">
         <v>15</v>
@@ -3504,10 +3479,10 @@
         <v>50</v>
       </c>
       <c r="D59" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E59">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="F59" t="s">
         <v>62</v>
@@ -3526,7 +3501,7 @@
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B60" t="s">
         <v>15</v>
@@ -3535,10 +3510,10 @@
         <v>50</v>
       </c>
       <c r="D60" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E60">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="F60" t="s">
         <v>62</v>
@@ -3557,7 +3532,7 @@
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B61" t="s">
         <v>15</v>
@@ -3566,10 +3541,10 @@
         <v>50</v>
       </c>
       <c r="D61" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E61">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="F61" t="s">
         <v>62</v>
@@ -3588,7 +3563,7 @@
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B62" t="s">
         <v>15</v>
@@ -3597,10 +3572,10 @@
         <v>50</v>
       </c>
       <c r="D62" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E62">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="F62" t="s">
         <v>62</v>
@@ -3619,7 +3594,7 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B63" t="s">
         <v>15</v>
@@ -3628,10 +3603,10 @@
         <v>50</v>
       </c>
       <c r="D63" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E63">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="F63" t="s">
         <v>62</v>
@@ -3650,7 +3625,7 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B64" t="s">
         <v>15</v>
@@ -3659,10 +3634,10 @@
         <v>50</v>
       </c>
       <c r="D64" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E64">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="F64" t="s">
         <v>62</v>
@@ -3681,7 +3656,7 @@
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B65" t="s">
         <v>15</v>
@@ -3690,10 +3665,10 @@
         <v>50</v>
       </c>
       <c r="D65" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E65">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="F65" t="s">
         <v>62</v>
@@ -3712,7 +3687,7 @@
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B66" t="s">
         <v>15</v>
@@ -3721,10 +3696,10 @@
         <v>50</v>
       </c>
       <c r="D66" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E66">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="F66" t="s">
         <v>62</v>
@@ -3743,7 +3718,7 @@
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B67" t="s">
         <v>15</v>
@@ -3752,10 +3727,10 @@
         <v>50</v>
       </c>
       <c r="D67" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E67">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="F67" t="s">
         <v>62</v>
@@ -3774,7 +3749,7 @@
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B68" t="s">
         <v>15</v>
@@ -3783,10 +3758,10 @@
         <v>50</v>
       </c>
       <c r="D68" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E68">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="F68" t="s">
         <v>62</v>
@@ -3805,7 +3780,7 @@
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B69" t="s">
         <v>15</v>
@@ -3814,10 +3789,10 @@
         <v>50</v>
       </c>
       <c r="D69" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E69">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F69" t="s">
         <v>62</v>
@@ -3836,7 +3811,7 @@
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B70" t="s">
         <v>15</v>
@@ -3845,10 +3820,10 @@
         <v>50</v>
       </c>
       <c r="D70" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E70">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F70" t="s">
         <v>62</v>
@@ -3867,7 +3842,7 @@
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B71" t="s">
         <v>15</v>
@@ -3876,10 +3851,10 @@
         <v>50</v>
       </c>
       <c r="D71" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E71">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="F71" t="s">
         <v>62</v>
@@ -3898,7 +3873,7 @@
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B72" t="s">
         <v>15</v>
@@ -3907,10 +3882,10 @@
         <v>50</v>
       </c>
       <c r="D72" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E72">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="F72" t="s">
         <v>62</v>
@@ -3929,7 +3904,7 @@
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B73" t="s">
         <v>15</v>
@@ -3938,10 +3913,10 @@
         <v>50</v>
       </c>
       <c r="D73" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E73">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="F73" t="s">
         <v>62</v>
@@ -3960,7 +3935,7 @@
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B74" t="s">
         <v>15</v>
@@ -3969,10 +3944,10 @@
         <v>50</v>
       </c>
       <c r="D74" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E74">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F74" t="s">
         <v>62</v>
@@ -3991,7 +3966,7 @@
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B75" t="s">
         <v>15</v>
@@ -4000,10 +3975,10 @@
         <v>50</v>
       </c>
       <c r="D75" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E75">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="F75" t="s">
         <v>62</v>
@@ -4022,7 +3997,7 @@
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B76" t="s">
         <v>15</v>
@@ -4031,10 +4006,10 @@
         <v>50</v>
       </c>
       <c r="D76" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E76">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F76" t="s">
         <v>62</v>
@@ -4053,7 +4028,7 @@
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>139</v>
+        <v>299</v>
       </c>
       <c r="B77" t="s">
         <v>15</v>
@@ -4062,10 +4037,10 @@
         <v>50</v>
       </c>
       <c r="D77" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E77">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F77" t="s">
         <v>62</v>
@@ -4084,7 +4059,7 @@
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>305</v>
+        <v>138</v>
       </c>
       <c r="B78" t="s">
         <v>15</v>
@@ -4093,13 +4068,13 @@
         <v>50</v>
       </c>
       <c r="D78" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="E78">
-        <v>2024</v>
+        <v>2001</v>
       </c>
       <c r="F78" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H78" s="2">
         <v>0</v>
@@ -4124,10 +4099,10 @@
         <v>50</v>
       </c>
       <c r="D79" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E79">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="F79" t="s">
         <v>65</v>
@@ -4146,7 +4121,7 @@
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B80" t="s">
         <v>15</v>
@@ -4155,10 +4130,10 @@
         <v>50</v>
       </c>
       <c r="D80" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E80">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="F80" t="s">
         <v>65</v>
@@ -4177,7 +4152,7 @@
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B81" t="s">
         <v>15</v>
@@ -4186,10 +4161,10 @@
         <v>50</v>
       </c>
       <c r="D81" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E81">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="F81" t="s">
         <v>65</v>
@@ -4208,7 +4183,7 @@
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B82" t="s">
         <v>15</v>
@@ -4217,10 +4192,10 @@
         <v>50</v>
       </c>
       <c r="D82" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E82">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="F82" t="s">
         <v>65</v>
@@ -4239,7 +4214,7 @@
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B83" t="s">
         <v>15</v>
@@ -4248,10 +4223,10 @@
         <v>50</v>
       </c>
       <c r="D83" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E83">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="F83" t="s">
         <v>65</v>
@@ -4270,7 +4245,7 @@
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B84" t="s">
         <v>15</v>
@@ -4279,10 +4254,10 @@
         <v>50</v>
       </c>
       <c r="D84" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E84">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="F84" t="s">
         <v>65</v>
@@ -4301,7 +4276,7 @@
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B85" t="s">
         <v>15</v>
@@ -4310,10 +4285,10 @@
         <v>50</v>
       </c>
       <c r="D85" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E85">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="F85" t="s">
         <v>65</v>
@@ -4332,7 +4307,7 @@
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B86" t="s">
         <v>15</v>
@@ -4341,10 +4316,10 @@
         <v>50</v>
       </c>
       <c r="D86" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E86">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="F86" t="s">
         <v>65</v>
@@ -4363,7 +4338,7 @@
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B87" t="s">
         <v>15</v>
@@ -4372,10 +4347,10 @@
         <v>50</v>
       </c>
       <c r="D87" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E87">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="F87" t="s">
         <v>65</v>
@@ -4394,7 +4369,7 @@
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B88" t="s">
         <v>15</v>
@@ -4403,10 +4378,10 @@
         <v>50</v>
       </c>
       <c r="D88" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E88">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="F88" t="s">
         <v>65</v>
@@ -4425,7 +4400,7 @@
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B89" t="s">
         <v>15</v>
@@ -4434,10 +4409,10 @@
         <v>50</v>
       </c>
       <c r="D89" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E89">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="F89" t="s">
         <v>65</v>
@@ -4456,7 +4431,7 @@
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B90" t="s">
         <v>15</v>
@@ -4465,10 +4440,10 @@
         <v>50</v>
       </c>
       <c r="D90" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E90">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="F90" t="s">
         <v>65</v>
@@ -4487,7 +4462,7 @@
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B91" t="s">
         <v>15</v>
@@ -4496,10 +4471,10 @@
         <v>50</v>
       </c>
       <c r="D91" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E91">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="F91" t="s">
         <v>65</v>
@@ -4518,7 +4493,7 @@
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B92" t="s">
         <v>15</v>
@@ -4527,10 +4502,10 @@
         <v>50</v>
       </c>
       <c r="D92" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E92">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="F92" t="s">
         <v>65</v>
@@ -4549,7 +4524,7 @@
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B93" t="s">
         <v>15</v>
@@ -4558,10 +4533,10 @@
         <v>50</v>
       </c>
       <c r="D93" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E93">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F93" t="s">
         <v>65</v>
@@ -4580,7 +4555,7 @@
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B94" t="s">
         <v>15</v>
@@ -4589,10 +4564,10 @@
         <v>50</v>
       </c>
       <c r="D94" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E94">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F94" t="s">
         <v>65</v>
@@ -4611,7 +4586,7 @@
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B95" t="s">
         <v>15</v>
@@ -4620,10 +4595,10 @@
         <v>50</v>
       </c>
       <c r="D95" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E95">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="F95" t="s">
         <v>65</v>
@@ -4642,7 +4617,7 @@
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B96" t="s">
         <v>15</v>
@@ -4651,10 +4626,10 @@
         <v>50</v>
       </c>
       <c r="D96" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E96">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="F96" t="s">
         <v>65</v>
@@ -4673,7 +4648,7 @@
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B97" t="s">
         <v>15</v>
@@ -4682,10 +4657,10 @@
         <v>50</v>
       </c>
       <c r="D97" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E97">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="F97" t="s">
         <v>65</v>
@@ -4704,7 +4679,7 @@
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B98" t="s">
         <v>15</v>
@@ -4713,10 +4688,10 @@
         <v>50</v>
       </c>
       <c r="D98" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E98">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F98" t="s">
         <v>65</v>
@@ -4735,7 +4710,7 @@
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B99" t="s">
         <v>15</v>
@@ -4744,10 +4719,10 @@
         <v>50</v>
       </c>
       <c r="D99" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E99">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="F99" t="s">
         <v>65</v>
@@ -4766,7 +4741,7 @@
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B100" t="s">
         <v>15</v>
@@ -4775,10 +4750,10 @@
         <v>50</v>
       </c>
       <c r="D100" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E100">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F100" t="s">
         <v>65</v>
@@ -4797,7 +4772,7 @@
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>163</v>
+        <v>298</v>
       </c>
       <c r="B101" t="s">
         <v>15</v>
@@ -4806,10 +4781,10 @@
         <v>50</v>
       </c>
       <c r="D101" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E101">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F101" t="s">
         <v>65</v>
@@ -4828,7 +4803,7 @@
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>304</v>
+        <v>162</v>
       </c>
       <c r="B102" t="s">
         <v>15</v>
@@ -4837,13 +4812,13 @@
         <v>50</v>
       </c>
       <c r="D102" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E102">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="F102" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="H102" s="2">
         <v>0</v>
@@ -4868,13 +4843,13 @@
         <v>50</v>
       </c>
       <c r="D103" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E103">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="F103" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H103" s="2">
         <v>0</v>
@@ -4890,7 +4865,7 @@
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B104" t="s">
         <v>15</v>
@@ -4899,13 +4874,13 @@
         <v>50</v>
       </c>
       <c r="D104" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E104">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F104" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H104" s="2">
         <v>0</v>
@@ -4921,7 +4896,7 @@
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B105" t="s">
         <v>15</v>
@@ -4930,13 +4905,13 @@
         <v>50</v>
       </c>
       <c r="D105" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E105">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="F105" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H105" s="2">
         <v>0</v>
@@ -4952,7 +4927,7 @@
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B106" t="s">
         <v>15</v>
@@ -4961,13 +4936,13 @@
         <v>50</v>
       </c>
       <c r="D106" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E106">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F106" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H106" s="2">
         <v>0</v>
@@ -4983,7 +4958,7 @@
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B107" t="s">
         <v>15</v>
@@ -4992,13 +4967,13 @@
         <v>50</v>
       </c>
       <c r="D107" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E107">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F107" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H107" s="2">
         <v>0</v>
@@ -5014,7 +4989,7 @@
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B108" t="s">
         <v>15</v>
@@ -5023,13 +4998,13 @@
         <v>50</v>
       </c>
       <c r="D108" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E108">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="F108" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H108" s="2">
         <v>0</v>
@@ -5045,22 +5020,22 @@
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
+        <v>170</v>
+      </c>
+      <c r="B109" t="s">
+        <v>15</v>
+      </c>
+      <c r="C109" t="s">
+        <v>50</v>
+      </c>
+      <c r="D109" t="s">
         <v>171</v>
       </c>
-      <c r="B109" t="s">
-        <v>15</v>
-      </c>
-      <c r="C109" t="s">
-        <v>50</v>
-      </c>
-      <c r="D109" t="s">
-        <v>141</v>
-      </c>
       <c r="E109">
-        <v>2025</v>
+        <v>2001</v>
       </c>
       <c r="F109" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="H109" s="2">
         <v>0</v>
@@ -5076,22 +5051,22 @@
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
+        <v>173</v>
+      </c>
+      <c r="B110" t="s">
+        <v>15</v>
+      </c>
+      <c r="C110" t="s">
+        <v>50</v>
+      </c>
+      <c r="D110" t="s">
+        <v>171</v>
+      </c>
+      <c r="E110">
+        <v>2002</v>
+      </c>
+      <c r="F110" t="s">
         <v>172</v>
-      </c>
-      <c r="B110" t="s">
-        <v>15</v>
-      </c>
-      <c r="C110" t="s">
-        <v>50</v>
-      </c>
-      <c r="D110" t="s">
-        <v>173</v>
-      </c>
-      <c r="E110">
-        <v>2001</v>
-      </c>
-      <c r="F110" t="s">
-        <v>174</v>
       </c>
       <c r="H110" s="2">
         <v>0</v>
@@ -5107,7 +5082,7 @@
     </row>
     <row r="111" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B111" t="s">
         <v>15</v>
@@ -5116,13 +5091,13 @@
         <v>50</v>
       </c>
       <c r="D111" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E111">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="F111" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H111" s="2">
         <v>0</v>
@@ -5138,7 +5113,7 @@
     </row>
     <row r="112" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B112" t="s">
         <v>15</v>
@@ -5147,13 +5122,13 @@
         <v>50</v>
       </c>
       <c r="D112" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E112">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="F112" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H112" s="2">
         <v>0</v>
@@ -5169,7 +5144,7 @@
     </row>
     <row r="113" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B113" t="s">
         <v>15</v>
@@ -5178,13 +5153,13 @@
         <v>50</v>
       </c>
       <c r="D113" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E113">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="F113" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H113" s="2">
         <v>0</v>
@@ -5200,7 +5175,7 @@
     </row>
     <row r="114" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B114" t="s">
         <v>15</v>
@@ -5209,13 +5184,13 @@
         <v>50</v>
       </c>
       <c r="D114" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E114">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="F114" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H114" s="2">
         <v>0</v>
@@ -5231,7 +5206,7 @@
     </row>
     <row r="115" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B115" t="s">
         <v>15</v>
@@ -5240,13 +5215,13 @@
         <v>50</v>
       </c>
       <c r="D115" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E115">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="F115" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H115" s="2">
         <v>0</v>
@@ -5262,7 +5237,7 @@
     </row>
     <row r="116" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B116" t="s">
         <v>15</v>
@@ -5271,13 +5246,13 @@
         <v>50</v>
       </c>
       <c r="D116" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E116">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="F116" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H116" s="2">
         <v>0</v>
@@ -5293,7 +5268,7 @@
     </row>
     <row r="117" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B117" t="s">
         <v>15</v>
@@ -5302,13 +5277,13 @@
         <v>50</v>
       </c>
       <c r="D117" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E117">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="F117" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H117" s="2">
         <v>0</v>
@@ -5324,7 +5299,7 @@
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B118" t="s">
         <v>15</v>
@@ -5333,13 +5308,13 @@
         <v>50</v>
       </c>
       <c r="D118" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E118">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="F118" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H118" s="2">
         <v>0</v>
@@ -5355,7 +5330,7 @@
     </row>
     <row r="119" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B119" t="s">
         <v>15</v>
@@ -5364,13 +5339,13 @@
         <v>50</v>
       </c>
       <c r="D119" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E119">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="F119" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H119" s="2">
         <v>0</v>
@@ -5386,7 +5361,7 @@
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B120" t="s">
         <v>15</v>
@@ -5395,13 +5370,13 @@
         <v>50</v>
       </c>
       <c r="D120" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E120">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="F120" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H120" s="2">
         <v>0</v>
@@ -5417,7 +5392,7 @@
     </row>
     <row r="121" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B121" t="s">
         <v>15</v>
@@ -5426,13 +5401,13 @@
         <v>50</v>
       </c>
       <c r="D121" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E121">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="F121" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H121" s="2">
         <v>0</v>
@@ -5448,7 +5423,7 @@
     </row>
     <row r="122" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B122" t="s">
         <v>15</v>
@@ -5457,13 +5432,13 @@
         <v>50</v>
       </c>
       <c r="D122" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E122">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="F122" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H122" s="2">
         <v>0</v>
@@ -5479,7 +5454,7 @@
     </row>
     <row r="123" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B123" t="s">
         <v>15</v>
@@ -5488,13 +5463,13 @@
         <v>50</v>
       </c>
       <c r="D123" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E123">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="F123" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H123" s="2">
         <v>0</v>
@@ -5510,7 +5485,7 @@
     </row>
     <row r="124" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B124" t="s">
         <v>15</v>
@@ -5519,13 +5494,13 @@
         <v>50</v>
       </c>
       <c r="D124" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E124">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F124" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H124" s="2">
         <v>0</v>
@@ -5541,7 +5516,7 @@
     </row>
     <row r="125" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B125" t="s">
         <v>15</v>
@@ -5550,13 +5525,13 @@
         <v>50</v>
       </c>
       <c r="D125" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E125">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F125" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H125" s="2">
         <v>0</v>
@@ -5572,7 +5547,7 @@
     </row>
     <row r="126" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B126" t="s">
         <v>15</v>
@@ -5581,13 +5556,13 @@
         <v>50</v>
       </c>
       <c r="D126" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E126">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="F126" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H126" s="2">
         <v>0</v>
@@ -5603,7 +5578,7 @@
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B127" t="s">
         <v>15</v>
@@ -5612,13 +5587,13 @@
         <v>50</v>
       </c>
       <c r="D127" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E127">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="F127" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H127" s="2">
         <v>0</v>
@@ -5634,7 +5609,7 @@
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B128" t="s">
         <v>15</v>
@@ -5643,13 +5618,13 @@
         <v>50</v>
       </c>
       <c r="D128" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E128">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="F128" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H128" s="2">
         <v>0</v>
@@ -5665,22 +5640,22 @@
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
+        <v>192</v>
+      </c>
+      <c r="B129" t="s">
+        <v>15</v>
+      </c>
+      <c r="C129" t="s">
+        <v>50</v>
+      </c>
+      <c r="D129" t="s">
+        <v>171</v>
+      </c>
+      <c r="E129">
+        <v>2000</v>
+      </c>
+      <c r="F129" t="s">
         <v>193</v>
-      </c>
-      <c r="B129" t="s">
-        <v>15</v>
-      </c>
-      <c r="C129" t="s">
-        <v>50</v>
-      </c>
-      <c r="D129" t="s">
-        <v>173</v>
-      </c>
-      <c r="E129">
-        <v>2020</v>
-      </c>
-      <c r="F129" t="s">
-        <v>174</v>
       </c>
       <c r="H129" s="2">
         <v>0</v>
@@ -5705,13 +5680,13 @@
         <v>50</v>
       </c>
       <c r="D130" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E130">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="F130" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H130" s="2">
         <v>0</v>
@@ -5727,7 +5702,7 @@
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B131" t="s">
         <v>15</v>
@@ -5736,13 +5711,13 @@
         <v>50</v>
       </c>
       <c r="D131" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E131">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="F131" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H131" s="2">
         <v>0</v>
@@ -5758,7 +5733,7 @@
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B132" t="s">
         <v>15</v>
@@ -5767,13 +5742,13 @@
         <v>50</v>
       </c>
       <c r="D132" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E132">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="F132" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H132" s="2">
         <v>0</v>
@@ -5789,7 +5764,7 @@
     </row>
     <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B133" t="s">
         <v>15</v>
@@ -5798,13 +5773,13 @@
         <v>50</v>
       </c>
       <c r="D133" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E133">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="F133" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H133" s="2">
         <v>0</v>
@@ -5820,7 +5795,7 @@
     </row>
     <row r="134" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B134" t="s">
         <v>15</v>
@@ -5829,13 +5804,13 @@
         <v>50</v>
       </c>
       <c r="D134" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E134">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="F134" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H134" s="2">
         <v>0</v>
@@ -5851,7 +5826,7 @@
     </row>
     <row r="135" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B135" t="s">
         <v>15</v>
@@ -5860,13 +5835,13 @@
         <v>50</v>
       </c>
       <c r="D135" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E135">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="F135" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H135" s="2">
         <v>0</v>
@@ -5882,7 +5857,7 @@
     </row>
     <row r="136" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B136" t="s">
         <v>15</v>
@@ -5891,13 +5866,13 @@
         <v>50</v>
       </c>
       <c r="D136" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E136">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="F136" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H136" s="2">
         <v>0</v>
@@ -5913,7 +5888,7 @@
     </row>
     <row r="137" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B137" t="s">
         <v>15</v>
@@ -5922,13 +5897,13 @@
         <v>50</v>
       </c>
       <c r="D137" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E137">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="F137" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H137" s="2">
         <v>0</v>
@@ -5944,7 +5919,7 @@
     </row>
     <row r="138" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B138" t="s">
         <v>15</v>
@@ -5953,13 +5928,13 @@
         <v>50</v>
       </c>
       <c r="D138" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E138">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="F138" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H138" s="2">
         <v>0</v>
@@ -5975,7 +5950,7 @@
     </row>
     <row r="139" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B139" t="s">
         <v>15</v>
@@ -5984,13 +5959,13 @@
         <v>50</v>
       </c>
       <c r="D139" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E139">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="F139" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H139" s="2">
         <v>0</v>
@@ -6006,7 +5981,7 @@
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B140" t="s">
         <v>15</v>
@@ -6015,13 +5990,13 @@
         <v>50</v>
       </c>
       <c r="D140" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E140">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="F140" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H140" s="2">
         <v>0</v>
@@ -6037,7 +6012,7 @@
     </row>
     <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B141" t="s">
         <v>15</v>
@@ -6046,13 +6021,13 @@
         <v>50</v>
       </c>
       <c r="D141" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E141">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="F141" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H141" s="2">
         <v>0</v>
@@ -6068,7 +6043,7 @@
     </row>
     <row r="142" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B142" t="s">
         <v>15</v>
@@ -6077,13 +6052,13 @@
         <v>50</v>
       </c>
       <c r="D142" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E142">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="F142" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H142" s="2">
         <v>0</v>
@@ -6099,7 +6074,7 @@
     </row>
     <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B143" t="s">
         <v>15</v>
@@ -6108,13 +6083,13 @@
         <v>50</v>
       </c>
       <c r="D143" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E143">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="F143" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H143" s="2">
         <v>0</v>
@@ -6130,7 +6105,7 @@
     </row>
     <row r="144" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B144" t="s">
         <v>15</v>
@@ -6139,13 +6114,13 @@
         <v>50</v>
       </c>
       <c r="D144" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E144">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="F144" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H144" s="2">
         <v>0</v>
@@ -6161,7 +6136,7 @@
     </row>
     <row r="145" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B145" t="s">
         <v>15</v>
@@ -6170,13 +6145,13 @@
         <v>50</v>
       </c>
       <c r="D145" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E145">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F145" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H145" s="2">
         <v>0</v>
@@ -6192,7 +6167,7 @@
     </row>
     <row r="146" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B146" t="s">
         <v>15</v>
@@ -6201,13 +6176,13 @@
         <v>50</v>
       </c>
       <c r="D146" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E146">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F146" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H146" s="2">
         <v>0</v>
@@ -6223,7 +6198,7 @@
     </row>
     <row r="147" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B147" t="s">
         <v>15</v>
@@ -6232,13 +6207,13 @@
         <v>50</v>
       </c>
       <c r="D147" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E147">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="F147" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H147" s="2">
         <v>0</v>
@@ -6254,7 +6229,7 @@
     </row>
     <row r="148" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B148" t="s">
         <v>15</v>
@@ -6263,13 +6238,13 @@
         <v>50</v>
       </c>
       <c r="D148" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E148">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="F148" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H148" s="2">
         <v>0</v>
@@ -6285,7 +6260,7 @@
     </row>
     <row r="149" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B149" t="s">
         <v>15</v>
@@ -6294,13 +6269,13 @@
         <v>50</v>
       </c>
       <c r="D149" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E149">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="F149" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H149" s="2">
         <v>0</v>
@@ -6316,7 +6291,7 @@
     </row>
     <row r="150" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B150" t="s">
         <v>15</v>
@@ -6325,13 +6300,13 @@
         <v>50</v>
       </c>
       <c r="D150" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E150">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F150" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H150" s="2">
         <v>0</v>
@@ -6347,7 +6322,7 @@
     </row>
     <row r="151" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B151" t="s">
         <v>15</v>
@@ -6356,13 +6331,13 @@
         <v>50</v>
       </c>
       <c r="D151" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E151">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="F151" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H151" s="2">
         <v>0</v>
@@ -6378,7 +6353,7 @@
     </row>
     <row r="152" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B152" t="s">
         <v>15</v>
@@ -6387,13 +6362,13 @@
         <v>50</v>
       </c>
       <c r="D152" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E152">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F152" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H152" s="2">
         <v>0</v>
@@ -6409,7 +6384,7 @@
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B153" t="s">
         <v>15</v>
@@ -6418,13 +6393,13 @@
         <v>50</v>
       </c>
       <c r="D153" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E153">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F153" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H153" s="2">
         <v>0</v>
@@ -6440,7 +6415,7 @@
     </row>
     <row r="154" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B154" t="s">
         <v>15</v>
@@ -6449,13 +6424,13 @@
         <v>50</v>
       </c>
       <c r="D154" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E154">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="F154" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H154" s="2">
         <v>0</v>
@@ -6471,27 +6446,32 @@
     </row>
     <row r="155" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
+        <v>219</v>
+      </c>
+      <c r="B155" t="s">
+        <v>15</v>
+      </c>
+      <c r="C155" t="s">
+        <v>50</v>
+      </c>
+      <c r="D155" t="s">
+        <v>114</v>
+      </c>
+      <c r="E155" t="s">
         <v>220</v>
       </c>
-      <c r="B155" t="s">
-        <v>15</v>
-      </c>
-      <c r="C155" t="s">
-        <v>50</v>
-      </c>
-      <c r="D155" t="s">
-        <v>173</v>
-      </c>
-      <c r="E155">
-        <v>2025</v>
-      </c>
       <c r="F155" t="s">
-        <v>195</v>
+        <v>62</v>
+      </c>
+      <c r="G155" t="s">
+        <v>19</v>
       </c>
       <c r="H155" s="2">
-        <v>0</v>
-      </c>
-      <c r="I155" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="I155" s="2" t="s">
+        <v>221</v>
+      </c>
       <c r="J155" s="2">
         <v>0</v>
       </c>
@@ -6502,7 +6482,7 @@
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B156" t="s">
         <v>15</v>
@@ -6511,10 +6491,10 @@
         <v>50</v>
       </c>
       <c r="D156" t="s">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="E156" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F156" t="s">
         <v>62</v>
@@ -6526,7 +6506,7 @@
         <v>1</v>
       </c>
       <c r="I156" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J156" s="2">
         <v>0</v>
@@ -6538,7 +6518,7 @@
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B157" t="s">
         <v>15</v>
@@ -6547,13 +6527,13 @@
         <v>50</v>
       </c>
       <c r="D157" t="s">
-        <v>91</v>
+        <v>139</v>
       </c>
       <c r="E157" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F157" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G157" t="s">
         <v>19</v>
@@ -6562,7 +6542,7 @@
         <v>1</v>
       </c>
       <c r="I157" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J157" s="2">
         <v>0</v>
@@ -6574,22 +6554,22 @@
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
+        <v>224</v>
+      </c>
+      <c r="B158" t="s">
+        <v>15</v>
+      </c>
+      <c r="C158" t="s">
+        <v>50</v>
+      </c>
+      <c r="D158" t="s">
         <v>225</v>
       </c>
-      <c r="B158" t="s">
-        <v>15</v>
-      </c>
-      <c r="C158" t="s">
-        <v>50</v>
-      </c>
-      <c r="D158" t="s">
-        <v>141</v>
-      </c>
       <c r="E158" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F158" t="s">
-        <v>65</v>
+        <v>172</v>
       </c>
       <c r="G158" t="s">
         <v>19</v>
@@ -6598,7 +6578,7 @@
         <v>1</v>
       </c>
       <c r="I158" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J158" s="2">
         <v>0</v>
@@ -6619,13 +6599,13 @@
         <v>50</v>
       </c>
       <c r="D159" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E159" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F159" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="G159" t="s">
         <v>19</v>
@@ -6634,7 +6614,7 @@
         <v>1</v>
       </c>
       <c r="I159" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J159" s="2">
         <v>0</v>
@@ -6646,22 +6626,22 @@
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
+        <v>227</v>
+      </c>
+      <c r="B160" t="s">
+        <v>15</v>
+      </c>
+      <c r="C160" t="s">
+        <v>50</v>
+      </c>
+      <c r="D160" t="s">
+        <v>139</v>
+      </c>
+      <c r="E160" t="s">
         <v>228</v>
       </c>
-      <c r="B160" t="s">
-        <v>15</v>
-      </c>
-      <c r="C160" t="s">
-        <v>50</v>
-      </c>
-      <c r="D160" t="s">
-        <v>227</v>
-      </c>
-      <c r="E160" t="s">
-        <v>222</v>
-      </c>
       <c r="F160" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
       <c r="G160" t="s">
         <v>19</v>
@@ -6670,7 +6650,7 @@
         <v>1</v>
       </c>
       <c r="I160" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J160" s="2">
         <v>0</v>
@@ -6691,13 +6671,13 @@
         <v>50</v>
       </c>
       <c r="D161" t="s">
-        <v>141</v>
+        <v>114</v>
       </c>
       <c r="E161" t="s">
         <v>230</v>
       </c>
       <c r="F161" t="s">
-        <v>165</v>
+        <v>62</v>
       </c>
       <c r="G161" t="s">
         <v>19</v>
@@ -6706,19 +6686,21 @@
         <v>1</v>
       </c>
       <c r="I161" s="2" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="J161" s="2">
-        <v>0</v>
-      </c>
-      <c r="K161" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="K161" s="2" t="s">
+        <v>231</v>
+      </c>
       <c r="L161" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="162" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B162" t="s">
         <v>15</v>
@@ -6727,10 +6709,10 @@
         <v>50</v>
       </c>
       <c r="D162" t="s">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="E162" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="F162" t="s">
         <v>62</v>
@@ -6742,13 +6724,13 @@
         <v>1</v>
       </c>
       <c r="I162" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="J162" s="2">
         <v>1</v>
       </c>
       <c r="K162" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="L162" s="2">
         <v>0</v>
@@ -6756,7 +6738,7 @@
     </row>
     <row r="163" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B163" t="s">
         <v>15</v>
@@ -6765,13 +6747,13 @@
         <v>50</v>
       </c>
       <c r="D163" t="s">
-        <v>91</v>
+        <v>139</v>
       </c>
       <c r="E163" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="F163" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G163" t="s">
         <v>19</v>
@@ -6780,13 +6762,13 @@
         <v>1</v>
       </c>
       <c r="I163" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="J163" s="2">
         <v>1</v>
       </c>
       <c r="K163" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="L163" s="2">
         <v>0</v>
@@ -6794,22 +6776,22 @@
     </row>
     <row r="164" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
+        <v>234</v>
+      </c>
+      <c r="B164" t="s">
+        <v>15</v>
+      </c>
+      <c r="C164" t="s">
+        <v>50</v>
+      </c>
+      <c r="D164" t="s">
         <v>235</v>
       </c>
-      <c r="B164" t="s">
-        <v>15</v>
-      </c>
-      <c r="C164" t="s">
-        <v>50</v>
-      </c>
-      <c r="D164" t="s">
-        <v>141</v>
-      </c>
       <c r="E164" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="F164" t="s">
-        <v>65</v>
+        <v>172</v>
       </c>
       <c r="G164" t="s">
         <v>19</v>
@@ -6818,13 +6800,13 @@
         <v>1</v>
       </c>
       <c r="I164" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="J164" s="2">
         <v>1</v>
       </c>
       <c r="K164" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="L164" s="2">
         <v>0</v>
@@ -6832,7 +6814,7 @@
     </row>
     <row r="165" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B165" t="s">
         <v>15</v>
@@ -6841,13 +6823,13 @@
         <v>50</v>
       </c>
       <c r="D165" t="s">
-        <v>237</v>
+        <v>139</v>
       </c>
       <c r="E165" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="F165" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="G165" t="s">
         <v>19</v>
@@ -6856,13 +6838,13 @@
         <v>1</v>
       </c>
       <c r="I165" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="J165" s="2">
         <v>1</v>
       </c>
       <c r="K165" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="L165" s="2">
         <v>0</v>
@@ -6870,7 +6852,7 @@
     </row>
     <row r="166" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B166" t="s">
         <v>15</v>
@@ -6879,74 +6861,72 @@
         <v>50</v>
       </c>
       <c r="D166" t="s">
-        <v>141</v>
-      </c>
-      <c r="E166" t="s">
-        <v>232</v>
+        <v>56</v>
+      </c>
+      <c r="E166">
+        <v>2020</v>
       </c>
       <c r="F166" t="s">
-        <v>195</v>
+        <v>52</v>
       </c>
       <c r="G166" t="s">
         <v>19</v>
       </c>
       <c r="H166" s="2">
+        <v>0</v>
+      </c>
+      <c r="I166" s="2"/>
+      <c r="J166" s="2">
+        <v>0</v>
+      </c>
+      <c r="K166" s="2"/>
+      <c r="L166" s="2">
         <v>1</v>
       </c>
-      <c r="I166" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="J166" s="2">
-        <v>1</v>
-      </c>
-      <c r="K166" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="L166" s="2">
-        <v>0</v>
+      <c r="M166" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="167" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
+        <v>239</v>
+      </c>
+      <c r="B167" t="s">
+        <v>15</v>
+      </c>
+      <c r="C167" t="s">
+        <v>50</v>
+      </c>
+      <c r="D167" t="s">
         <v>240</v>
       </c>
-      <c r="B167" t="s">
-        <v>15</v>
-      </c>
-      <c r="C167" t="s">
-        <v>50</v>
-      </c>
-      <c r="D167" t="s">
-        <v>141</v>
-      </c>
-      <c r="E167" t="s">
+      <c r="E167">
+        <v>2020</v>
+      </c>
+      <c r="F167" t="s">
         <v>241</v>
-      </c>
-      <c r="F167" t="s">
-        <v>242</v>
       </c>
       <c r="G167" t="s">
         <v>19</v>
       </c>
       <c r="H167" s="2">
+        <v>0</v>
+      </c>
+      <c r="I167" s="2"/>
+      <c r="J167" s="2">
+        <v>0</v>
+      </c>
+      <c r="K167" s="2"/>
+      <c r="L167" s="2">
         <v>1</v>
       </c>
-      <c r="I167" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="J167" s="2">
-        <v>1</v>
-      </c>
-      <c r="K167" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="L167" s="2">
-        <v>0</v>
+      <c r="M167" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="168" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B168" t="s">
         <v>15</v>
@@ -6961,7 +6941,7 @@
         <v>2020</v>
       </c>
       <c r="F168" t="s">
-        <v>52</v>
+        <v>243</v>
       </c>
       <c r="G168" t="s">
         <v>19</v>
@@ -6998,7 +6978,7 @@
         <v>2020</v>
       </c>
       <c r="F169" t="s">
-        <v>246</v>
+        <v>52</v>
       </c>
       <c r="G169" t="s">
         <v>19</v>
@@ -7015,27 +6995,27 @@
         <v>1</v>
       </c>
       <c r="M169" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="170" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
+        <v>246</v>
+      </c>
+      <c r="B170" t="s">
+        <v>15</v>
+      </c>
+      <c r="C170" t="s">
+        <v>50</v>
+      </c>
+      <c r="D170" t="s">
         <v>247</v>
-      </c>
-      <c r="B170" t="s">
-        <v>15</v>
-      </c>
-      <c r="C170" t="s">
-        <v>50</v>
-      </c>
-      <c r="D170" t="s">
-        <v>56</v>
       </c>
       <c r="E170">
         <v>2020</v>
       </c>
       <c r="F170" t="s">
-        <v>248</v>
+        <v>52</v>
       </c>
       <c r="G170" t="s">
         <v>19</v>
@@ -7052,7 +7032,7 @@
         <v>1</v>
       </c>
       <c r="M170" s="2" t="s">
-        <v>58</v>
+        <v>248</v>
       </c>
     </row>
     <row r="171" spans="1:14" x14ac:dyDescent="0.35">
@@ -7069,13 +7049,10 @@
         <v>250</v>
       </c>
       <c r="E171">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="F171" t="s">
-        <v>52</v>
-      </c>
-      <c r="G171" t="s">
-        <v>19</v>
+        <v>251</v>
       </c>
       <c r="H171" s="2">
         <v>0</v>
@@ -7089,12 +7066,15 @@
         <v>1</v>
       </c>
       <c r="M171" s="2" t="s">
-        <v>54</v>
+        <v>248</v>
+      </c>
+      <c r="N171" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="172" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B172" t="s">
         <v>15</v>
@@ -7103,13 +7083,13 @@
         <v>50</v>
       </c>
       <c r="D172" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E172">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="F172" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="G172" t="s">
         <v>19</v>
@@ -7126,12 +7106,12 @@
         <v>1</v>
       </c>
       <c r="M172" s="2" t="s">
-        <v>253</v>
+        <v>312</v>
       </c>
     </row>
     <row r="173" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B173" t="s">
         <v>15</v>
@@ -7140,13 +7120,13 @@
         <v>50</v>
       </c>
       <c r="D173" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E173">
-        <v>2015</v>
+        <v>2023</v>
       </c>
       <c r="F173" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H173" s="2">
         <v>0</v>
@@ -7160,10 +7140,7 @@
         <v>1</v>
       </c>
       <c r="M173" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="N173" t="s">
-        <v>257</v>
+        <v>312</v>
       </c>
     </row>
     <row r="174" spans="1:14" x14ac:dyDescent="0.35">
@@ -7177,16 +7154,13 @@
         <v>50</v>
       </c>
       <c r="D174" t="s">
+        <v>256</v>
+      </c>
+      <c r="E174">
+        <v>2022</v>
+      </c>
+      <c r="F174" t="s">
         <v>259</v>
-      </c>
-      <c r="E174">
-        <v>2023</v>
-      </c>
-      <c r="F174" t="s">
-        <v>62</v>
-      </c>
-      <c r="G174" t="s">
-        <v>19</v>
       </c>
       <c r="H174" s="2">
         <v>0</v>
@@ -7200,7 +7174,7 @@
         <v>1</v>
       </c>
       <c r="M174" s="2" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
     </row>
     <row r="175" spans="1:14" x14ac:dyDescent="0.35">
@@ -7214,13 +7188,16 @@
         <v>50</v>
       </c>
       <c r="D175" t="s">
-        <v>261</v>
+        <v>74</v>
       </c>
       <c r="E175">
         <v>2023</v>
       </c>
       <c r="F175" t="s">
-        <v>262</v>
+        <v>301</v>
+      </c>
+      <c r="G175" t="s">
+        <v>19</v>
       </c>
       <c r="H175" s="2">
         <v>0</v>
@@ -7234,12 +7211,12 @@
         <v>1</v>
       </c>
       <c r="M175" s="2" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
     </row>
     <row r="176" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B176" t="s">
         <v>15</v>
@@ -7248,13 +7225,16 @@
         <v>50</v>
       </c>
       <c r="D176" t="s">
-        <v>261</v>
+        <v>82</v>
       </c>
       <c r="E176">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F176" t="s">
-        <v>264</v>
+        <v>301</v>
+      </c>
+      <c r="G176" t="s">
+        <v>19</v>
       </c>
       <c r="H176" s="2">
         <v>0</v>
@@ -7268,12 +7248,12 @@
         <v>1</v>
       </c>
       <c r="M176" s="2" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
     </row>
     <row r="177" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
-        <v>265</v>
+        <v>302</v>
       </c>
       <c r="B177" t="s">
         <v>15</v>
@@ -7282,13 +7262,13 @@
         <v>50</v>
       </c>
       <c r="D177" t="s">
-        <v>74</v>
+        <v>303</v>
       </c>
       <c r="E177">
         <v>2023</v>
       </c>
       <c r="F177" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="G177" t="s">
         <v>19</v>
@@ -7305,12 +7285,12 @@
         <v>1</v>
       </c>
       <c r="M177" s="2" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
     </row>
     <row r="178" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="B178" t="s">
         <v>15</v>
@@ -7319,13 +7299,13 @@
         <v>50</v>
       </c>
       <c r="D178" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E178">
         <v>2023</v>
       </c>
       <c r="F178" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="G178" t="s">
         <v>19</v>
@@ -7342,12 +7322,12 @@
         <v>1</v>
       </c>
       <c r="M178" s="2" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
     </row>
     <row r="179" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
-        <v>308</v>
+        <v>263</v>
       </c>
       <c r="B179" t="s">
         <v>15</v>
@@ -7356,13 +7336,13 @@
         <v>50</v>
       </c>
       <c r="D179" t="s">
-        <v>309</v>
+        <v>264</v>
       </c>
       <c r="E179">
         <v>2023</v>
       </c>
       <c r="F179" t="s">
-        <v>307</v>
+        <v>257</v>
       </c>
       <c r="G179" t="s">
         <v>19</v>
@@ -7379,12 +7359,12 @@
         <v>1</v>
       </c>
       <c r="M179" s="2" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
     </row>
     <row r="180" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B180" t="s">
         <v>15</v>
@@ -7393,13 +7373,13 @@
         <v>50</v>
       </c>
       <c r="D180" t="s">
-        <v>78</v>
+        <v>264</v>
       </c>
       <c r="E180">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="F180" t="s">
-        <v>307</v>
+        <v>259</v>
       </c>
       <c r="G180" t="s">
         <v>19</v>
@@ -7416,12 +7396,12 @@
         <v>1</v>
       </c>
       <c r="M180" s="2" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
     </row>
     <row r="181" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>268</v>
+        <v>307</v>
       </c>
       <c r="B181" t="s">
         <v>15</v>
@@ -7430,13 +7410,13 @@
         <v>50</v>
       </c>
       <c r="D181" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E181">
-        <v>2023</v>
+        <v>2015</v>
       </c>
       <c r="F181" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="G181" t="s">
         <v>19</v>
@@ -7453,81 +7433,59 @@
         <v>1</v>
       </c>
       <c r="M181" s="2" t="s">
-        <v>314</v>
+        <v>305</v>
+      </c>
+      <c r="N181" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="182" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
-        <v>270</v>
+        <v>313</v>
       </c>
       <c r="B182" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C182" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="D182" t="s">
         <v>269</v>
       </c>
-      <c r="E182">
-        <v>2022</v>
+      <c r="E182" t="s">
+        <v>16</v>
       </c>
       <c r="F182" t="s">
-        <v>264</v>
+        <v>18</v>
       </c>
       <c r="G182" t="s">
         <v>19</v>
       </c>
-      <c r="H182" s="2">
-        <v>0</v>
-      </c>
-      <c r="I182" s="2"/>
-      <c r="J182" s="2">
-        <v>0</v>
-      </c>
-      <c r="K182" s="2"/>
-      <c r="L182" s="2">
-        <v>1</v>
-      </c>
-      <c r="M182" s="2" t="s">
-        <v>314</v>
+      <c r="N182" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="183" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
-        <v>313</v>
+        <v>270</v>
       </c>
       <c r="B183" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C183" t="s">
-        <v>50</v>
+        <v>271</v>
       </c>
       <c r="D183" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E183">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="F183" t="s">
-        <v>272</v>
+        <v>18</v>
       </c>
       <c r="G183" t="s">
         <v>19</v>
-      </c>
-      <c r="H183" s="2">
-        <v>0</v>
-      </c>
-      <c r="I183" s="2"/>
-      <c r="J183" s="2">
-        <v>0</v>
-      </c>
-      <c r="K183" s="2"/>
-      <c r="L183" s="2">
-        <v>1</v>
-      </c>
-      <c r="M183" s="2" t="s">
-        <v>311</v>
       </c>
       <c r="N183" t="s">
         <v>273</v>
@@ -7541,13 +7499,13 @@
         <v>21</v>
       </c>
       <c r="C184" t="s">
-        <v>16</v>
+        <v>271</v>
       </c>
       <c r="D184" t="s">
         <v>275</v>
       </c>
-      <c r="E184" t="s">
-        <v>16</v>
+      <c r="E184">
+        <v>2020</v>
       </c>
       <c r="F184" t="s">
         <v>18</v>
@@ -7556,7 +7514,7 @@
         <v>19</v>
       </c>
       <c r="N184" t="s">
-        <v>38</v>
+        <v>273</v>
       </c>
     </row>
     <row r="185" spans="1:14" x14ac:dyDescent="0.35">
@@ -7567,13 +7525,13 @@
         <v>21</v>
       </c>
       <c r="C185" t="s">
+        <v>271</v>
+      </c>
+      <c r="D185" t="s">
         <v>277</v>
       </c>
-      <c r="D185" t="s">
-        <v>278</v>
-      </c>
-      <c r="E185">
-        <v>2020</v>
+      <c r="E185" t="s">
+        <v>220</v>
       </c>
       <c r="F185" t="s">
         <v>18</v>
@@ -7582,24 +7540,24 @@
         <v>19</v>
       </c>
       <c r="N185" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="186" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B186" t="s">
         <v>21</v>
       </c>
       <c r="C186" t="s">
+        <v>271</v>
+      </c>
+      <c r="D186" t="s">
         <v>277</v>
       </c>
-      <c r="D186" t="s">
-        <v>281</v>
-      </c>
-      <c r="E186">
-        <v>2020</v>
+      <c r="E186" t="s">
+        <v>279</v>
       </c>
       <c r="F186" t="s">
         <v>18</v>
@@ -7608,24 +7566,24 @@
         <v>19</v>
       </c>
       <c r="N186" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="187" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B187" t="s">
         <v>21</v>
       </c>
       <c r="C187" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="D187" t="s">
-        <v>283</v>
-      </c>
-      <c r="E187" t="s">
-        <v>222</v>
+        <v>281</v>
+      </c>
+      <c r="E187">
+        <v>2020</v>
       </c>
       <c r="F187" t="s">
         <v>18</v>
@@ -7634,24 +7592,24 @@
         <v>19</v>
       </c>
       <c r="N187" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="188" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B188" t="s">
         <v>21</v>
       </c>
       <c r="C188" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="D188" t="s">
         <v>283</v>
       </c>
-      <c r="E188" t="s">
-        <v>285</v>
+      <c r="E188">
+        <v>2020</v>
       </c>
       <c r="F188" t="s">
         <v>18</v>
@@ -7660,21 +7618,21 @@
         <v>19</v>
       </c>
       <c r="N188" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="189" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B189" t="s">
         <v>21</v>
       </c>
       <c r="C189" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="D189" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="E189">
         <v>2020</v>
@@ -7686,24 +7644,24 @@
         <v>19</v>
       </c>
       <c r="N189" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="190" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>288</v>
+        <v>309</v>
       </c>
       <c r="B190" t="s">
         <v>21</v>
       </c>
       <c r="C190" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="D190" t="s">
-        <v>289</v>
-      </c>
-      <c r="E190">
-        <v>2020</v>
+        <v>285</v>
+      </c>
+      <c r="E190" t="s">
+        <v>279</v>
       </c>
       <c r="F190" t="s">
         <v>18</v>
@@ -7712,24 +7670,24 @@
         <v>19</v>
       </c>
       <c r="N190" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="191" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>290</v>
+        <v>310</v>
       </c>
       <c r="B191" t="s">
         <v>21</v>
       </c>
       <c r="C191" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="D191" t="s">
-        <v>291</v>
-      </c>
-      <c r="E191">
-        <v>2020</v>
+        <v>272</v>
+      </c>
+      <c r="E191" t="s">
+        <v>279</v>
       </c>
       <c r="F191" t="s">
         <v>18</v>
@@ -7738,24 +7696,24 @@
         <v>19</v>
       </c>
       <c r="N191" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="192" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B192" t="s">
         <v>21</v>
       </c>
       <c r="C192" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="D192" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="E192" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="F192" t="s">
         <v>18</v>
@@ -7764,24 +7722,24 @@
         <v>19</v>
       </c>
       <c r="N192" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="193" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="B193" t="s">
         <v>21</v>
       </c>
       <c r="C193" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="D193" t="s">
-        <v>278</v>
-      </c>
-      <c r="E193" t="s">
-        <v>285</v>
+        <v>287</v>
+      </c>
+      <c r="E193">
+        <v>2015</v>
       </c>
       <c r="F193" t="s">
         <v>18</v>
@@ -7790,24 +7748,24 @@
         <v>19</v>
       </c>
       <c r="N193" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
     </row>
     <row r="194" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
-        <v>317</v>
+        <v>288</v>
       </c>
       <c r="B194" t="s">
         <v>21</v>
       </c>
       <c r="C194" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="D194" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="E194" t="s">
-        <v>285</v>
+        <v>16</v>
       </c>
       <c r="F194" t="s">
         <v>18</v>
@@ -7816,24 +7774,24 @@
         <v>19</v>
       </c>
       <c r="N194" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
     </row>
     <row r="195" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
-        <v>312</v>
+        <v>292</v>
       </c>
       <c r="B195" t="s">
         <v>21</v>
       </c>
       <c r="C195" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="D195" t="s">
         <v>293</v>
       </c>
-      <c r="E195">
-        <v>2015</v>
+      <c r="E195" t="s">
+        <v>16</v>
       </c>
       <c r="F195" t="s">
         <v>18</v>
@@ -7842,18 +7800,18 @@
         <v>19</v>
       </c>
       <c r="N195" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="196" spans="1:14" x14ac:dyDescent="0.35">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="196" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B196" t="s">
         <v>21</v>
       </c>
       <c r="C196" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="D196" t="s">
         <v>296</v>
@@ -7869,58 +7827,6 @@
       </c>
       <c r="N196" t="s">
         <v>297</v>
-      </c>
-    </row>
-    <row r="197" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A197" t="s">
-        <v>298</v>
-      </c>
-      <c r="B197" t="s">
-        <v>21</v>
-      </c>
-      <c r="C197" t="s">
-        <v>295</v>
-      </c>
-      <c r="D197" t="s">
-        <v>299</v>
-      </c>
-      <c r="E197" t="s">
-        <v>16</v>
-      </c>
-      <c r="F197" t="s">
-        <v>18</v>
-      </c>
-      <c r="G197" t="s">
-        <v>19</v>
-      </c>
-      <c r="N197" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="198" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A198" t="s">
-        <v>301</v>
-      </c>
-      <c r="B198" t="s">
-        <v>21</v>
-      </c>
-      <c r="C198" t="s">
-        <v>295</v>
-      </c>
-      <c r="D198" t="s">
-        <v>302</v>
-      </c>
-      <c r="E198" t="s">
-        <v>16</v>
-      </c>
-      <c r="F198" t="s">
-        <v>18</v>
-      </c>
-      <c r="G198" t="s">
-        <v>19</v>
-      </c>
-      <c r="N198" t="s">
-        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -7931,33 +7837,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <kae7f6409c1a45b5af70ba169c41da0e xmlns="82302deb-32b0-442b-bedc-ba64a9aa8ccd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </kae7f6409c1a45b5af70ba169c41da0e>
-    <REDD_x002f_NFM_x0020_category xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="82302deb-32b0-442b-bedc-ba64a9aa8ccd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003082C08FD3D0614AAB94B75C024070A7" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1a4b61487ffa532d49c6719891dd0d2e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="82302deb-32b0-442b-bedc-ba64a9aa8ccd" xmlns:ns3="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cea40d1c5f6ee0e5ae997cf8704aff88" ns2:_="" ns3:_="">
     <xsd:import namespace="82302deb-32b0-442b-bedc-ba64a9aa8ccd"/>
@@ -8246,26 +8125,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63A60D8A-7D1B-403D-BB2C-B10CCD11CB4B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="82302deb-32b0-442b-bedc-ba64a9aa8ccd"/>
-    <ds:schemaRef ds:uri="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5DBDC3B9-24A5-4D52-9DEE-E1BAF29BA53E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <kae7f6409c1a45b5af70ba169c41da0e xmlns="82302deb-32b0-442b-bedc-ba64a9aa8ccd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </kae7f6409c1a45b5af70ba169c41da0e>
+    <REDD_x002f_NFM_x0020_category xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="82302deb-32b0-442b-bedc-ba64a9aa8ccd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE6D2EE7-47BC-4B0F-B98D-543F5E3F8F03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8282,4 +8169,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5DBDC3B9-24A5-4D52-9DEE-E1BAF29BA53E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63A60D8A-7D1B-403D-BB2C-B10CCD11CB4B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="82302deb-32b0-442b-bedc-ba64a9aa8ccd"/>
+    <ds:schemaRef ds:uri="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
added national data to whisp columns: a new tab as not strictly default/core whisp datasets
</commit_message>
<xml_diff>
--- a/whisp_columns.xlsx
+++ b/whisp_columns.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnell\Documents\GitHub\whisp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87BC43A7-E222-4A0F-9D82-753F6C558B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D28990-C9B1-4A71-96CF-8FE5A8DEDD0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12420" xr2:uid="{FC85F32F-3F3C-476F-A445-BF878E774111}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12420" activeTab="1" xr2:uid="{FC85F32F-3F3C-476F-A445-BF878E774111}"/>
   </bookViews>
   <sheets>
     <sheet name="Whisp outputs" sheetId="1" r:id="rId1"/>
+    <sheet name="Whisp outputs national" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1247" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1489" uniqueCount="357">
   <si>
     <t>Column name</t>
   </si>
@@ -978,6 +979,135 @@
   </si>
   <si>
     <t>geo</t>
+  </si>
+  <si>
+    <t>nCO_ideam_forest_2020</t>
+  </si>
+  <si>
+    <t>IDEAM 2020</t>
+  </si>
+  <si>
+    <t>nCO_ideam_agroforest_2020</t>
+  </si>
+  <si>
+    <t>Area of agroforestry</t>
+  </si>
+  <si>
+    <t>nBR_INPE_TC_primary_forest_Amazon_2020</t>
+  </si>
+  <si>
+    <t>Assis et al,. 2019</t>
+  </si>
+  <si>
+    <t>nBR_INPE_TC_secondary_forest_Amazon_2020</t>
+  </si>
+  <si>
+    <t>nBR_BFS_primary_forest_Pantanal_2020</t>
+  </si>
+  <si>
+    <t>Serviço Florestal Brasileiro, 2024</t>
+  </si>
+  <si>
+    <t>nBR_BFS_primary_forest_Caatinga_2020</t>
+  </si>
+  <si>
+    <t>nBR_BFS_primary_forest_AtlanticForest_2020</t>
+  </si>
+  <si>
+    <t>nBR_BFS_primary_forest_Pampa_2020</t>
+  </si>
+  <si>
+    <t>nBR_BFS_primary&amp;secondary_forest_Cerrado_2020</t>
+  </si>
+  <si>
+    <t>nBR_MapBiomas_col9_forest_Brazil_2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Souza et al., 2020</t>
+  </si>
+  <si>
+    <t>nBR_INPE_TCsilviculture_Amazon_2020</t>
+  </si>
+  <si>
+    <t>TERRACLASS (EMBRAPA) (2023)</t>
+  </si>
+  <si>
+    <t>nBR_INPE_TCsilviculture_Cerrado_2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TERRACLASS (INPE/EMBRAPA). </t>
+  </si>
+  <si>
+    <t>nBR_MapBiomas_col9_silviculture_Brazil_2020</t>
+  </si>
+  <si>
+    <t>nBR_PRODES_deforestation_Brazil_before_2020</t>
+  </si>
+  <si>
+    <t>1988-2000</t>
+  </si>
+  <si>
+    <t>nBR_DETER_forestdegradation_Amazon_before_2020</t>
+  </si>
+  <si>
+    <t>2016-2000</t>
+  </si>
+  <si>
+    <t>Doblas 2022</t>
+  </si>
+  <si>
+    <t>nBR_PRODES_deforestation_Brazil_after_2020</t>
+  </si>
+  <si>
+    <t>2000-present</t>
+  </si>
+  <si>
+    <t>nBR_DETER_forestdegradation_Amazon_after_2020</t>
+  </si>
+  <si>
+    <t>nBR_INPE_TCamz_cer_perennial_2020</t>
+  </si>
+  <si>
+    <t>Area of Perennial Crops</t>
+  </si>
+  <si>
+    <t>nBR_MapBiomas_col9_coffee_2020</t>
+  </si>
+  <si>
+    <t>nBR_MapBiomas_col9_palmoil_2020</t>
+  </si>
+  <si>
+    <t>nBR_MapBiomas_col9_pc_2020</t>
+  </si>
+  <si>
+    <t>nBR_INPE_TCamz_cer_annual_2020</t>
+  </si>
+  <si>
+    <t>Area of Annual Crops</t>
+  </si>
+  <si>
+    <t>nBR_MapBiomas_col9_soy_2020</t>
+  </si>
+  <si>
+    <t>nBR_MapBiomas_col9_annual_crops_2020</t>
+  </si>
+  <si>
+    <t>nBR_INPE_TCamz_pasture_2020</t>
+  </si>
+  <si>
+    <t>Area of Pasture</t>
+  </si>
+  <si>
+    <t>nBR_INPE_TCcer_pasture_2020</t>
+  </si>
+  <si>
+    <t>nBR_MapBiomas_col9_pasture_2020</t>
+  </si>
+  <si>
+    <t>nCI_Cocoa_bnetd</t>
+  </si>
+  <si>
+    <t>BNETD 2020.</t>
   </si>
 </sst>
 </file>
@@ -1005,7 +1135,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1015,6 +1145,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1031,10 +1167,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7777,7 +7914,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="195" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>292</v>
       </c>
@@ -7836,7 +7973,1152 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD3BA78D-4BAA-453B-B2F4-F30CD56DAD59}">
+  <dimension ref="A1:N29"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2">
+        <v>2020</v>
+      </c>
+      <c r="F2" t="s">
+        <v>315</v>
+      </c>
+      <c r="H2" s="2">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J2" s="2">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>316</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" t="s">
+        <v>317</v>
+      </c>
+      <c r="E3">
+        <v>2020</v>
+      </c>
+      <c r="F3" t="s">
+        <v>315</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J3" s="2">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>318</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4">
+        <v>2020</v>
+      </c>
+      <c r="F4" t="s">
+        <v>319</v>
+      </c>
+      <c r="H4" s="2">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J4" s="2">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L4" s="2">
+        <v>1</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>320</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5">
+        <v>2020</v>
+      </c>
+      <c r="F5" t="s">
+        <v>319</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J5" s="2">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L5" s="2">
+        <v>1</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>321</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6">
+        <v>2020</v>
+      </c>
+      <c r="F6" t="s">
+        <v>322</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J6" s="2">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L6" s="2">
+        <v>1</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>323</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7">
+        <v>2020</v>
+      </c>
+      <c r="F7" t="s">
+        <v>322</v>
+      </c>
+      <c r="H7" s="2">
+        <v>1</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J7" s="2">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L7" s="2">
+        <v>1</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>324</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8">
+        <v>2020</v>
+      </c>
+      <c r="F8" t="s">
+        <v>322</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J8" s="2">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L8" s="2">
+        <v>1</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>325</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9">
+        <v>2020</v>
+      </c>
+      <c r="F9" t="s">
+        <v>322</v>
+      </c>
+      <c r="H9" s="2">
+        <v>1</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J9" s="2">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L9" s="2">
+        <v>1</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>326</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10">
+        <v>2020</v>
+      </c>
+      <c r="F10" t="s">
+        <v>322</v>
+      </c>
+      <c r="H10" s="2">
+        <v>1</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J10" s="2">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L10" s="2">
+        <v>1</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>327</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11">
+        <v>2020</v>
+      </c>
+      <c r="F11" t="s">
+        <v>328</v>
+      </c>
+      <c r="H11" s="2">
+        <v>1</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J11" s="2">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L11" s="2">
+        <v>1</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>329</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12">
+        <v>2020</v>
+      </c>
+      <c r="F12" t="s">
+        <v>330</v>
+      </c>
+      <c r="H12" s="2">
+        <v>1</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J12" s="2">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" s="2">
+        <v>1</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>331</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13">
+        <v>2020</v>
+      </c>
+      <c r="F13" t="s">
+        <v>332</v>
+      </c>
+      <c r="H13" s="2">
+        <v>1</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" s="2">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L13" s="2">
+        <v>1</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>333</v>
+      </c>
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E14">
+        <v>2020</v>
+      </c>
+      <c r="F14" t="s">
+        <v>328</v>
+      </c>
+      <c r="H14" s="2">
+        <v>1</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J14" s="2">
+        <v>1</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L14" s="2">
+        <v>1</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>334</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" t="s">
+        <v>89</v>
+      </c>
+      <c r="E15" t="s">
+        <v>335</v>
+      </c>
+      <c r="F15" t="s">
+        <v>319</v>
+      </c>
+      <c r="H15" s="2">
+        <v>1</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="J15" s="2">
+        <v>1</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="L15" s="2">
+        <v>1</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>336</v>
+      </c>
+      <c r="B16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" t="s">
+        <v>114</v>
+      </c>
+      <c r="E16" t="s">
+        <v>337</v>
+      </c>
+      <c r="F16" t="s">
+        <v>338</v>
+      </c>
+      <c r="H16" s="2">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="J16" s="2">
+        <v>1</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="L16" s="2">
+        <v>1</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>339</v>
+      </c>
+      <c r="B17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" t="s">
+        <v>89</v>
+      </c>
+      <c r="E17" t="s">
+        <v>340</v>
+      </c>
+      <c r="F17" t="s">
+        <v>319</v>
+      </c>
+      <c r="H17" s="2">
+        <v>1</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="J17" s="2">
+        <v>1</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="L17" s="2">
+        <v>1</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>341</v>
+      </c>
+      <c r="B18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>114</v>
+      </c>
+      <c r="E18" t="s">
+        <v>340</v>
+      </c>
+      <c r="F18" t="s">
+        <v>338</v>
+      </c>
+      <c r="H18" s="2">
+        <v>1</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="J18" s="2">
+        <v>1</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="L18" s="2">
+        <v>1</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>342</v>
+      </c>
+      <c r="B19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" t="s">
+        <v>343</v>
+      </c>
+      <c r="E19">
+        <v>2020</v>
+      </c>
+      <c r="F19" t="s">
+        <v>330</v>
+      </c>
+      <c r="H19" s="2">
+        <v>1</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J19" s="2">
+        <v>1</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L19" s="2">
+        <v>1</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>344</v>
+      </c>
+      <c r="B20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" t="s">
+        <v>303</v>
+      </c>
+      <c r="E20">
+        <v>2020</v>
+      </c>
+      <c r="F20" t="s">
+        <v>328</v>
+      </c>
+      <c r="H20" s="2">
+        <v>1</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J20" s="2">
+        <v>1</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L20" s="2">
+        <v>1</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>345</v>
+      </c>
+      <c r="B21" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" t="s">
+        <v>74</v>
+      </c>
+      <c r="E21">
+        <v>2020</v>
+      </c>
+      <c r="F21" t="s">
+        <v>328</v>
+      </c>
+      <c r="H21" s="2">
+        <v>1</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J21" s="2">
+        <v>1</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L21" s="2">
+        <v>1</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>346</v>
+      </c>
+      <c r="B22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" t="s">
+        <v>343</v>
+      </c>
+      <c r="E22">
+        <v>2020</v>
+      </c>
+      <c r="F22" t="s">
+        <v>328</v>
+      </c>
+      <c r="H22" s="2">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J22" s="2">
+        <v>1</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L22" s="2">
+        <v>1</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>347</v>
+      </c>
+      <c r="B23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" t="s">
+        <v>348</v>
+      </c>
+      <c r="E23">
+        <v>2020</v>
+      </c>
+      <c r="F23" t="s">
+        <v>330</v>
+      </c>
+      <c r="H23" s="2">
+        <v>1</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J23" s="2">
+        <v>1</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L23" s="2">
+        <v>1</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>349</v>
+      </c>
+      <c r="B24" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" t="s">
+        <v>86</v>
+      </c>
+      <c r="E24">
+        <v>2020</v>
+      </c>
+      <c r="F24" t="s">
+        <v>328</v>
+      </c>
+      <c r="H24" s="2">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J24" s="2">
+        <v>1</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L24" s="2">
+        <v>1</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>350</v>
+      </c>
+      <c r="B25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" t="s">
+        <v>348</v>
+      </c>
+      <c r="E25">
+        <v>2020</v>
+      </c>
+      <c r="F25" t="s">
+        <v>328</v>
+      </c>
+      <c r="H25" s="2">
+        <v>1</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J25" s="2">
+        <v>1</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L25" s="2">
+        <v>1</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>351</v>
+      </c>
+      <c r="B26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" t="s">
+        <v>352</v>
+      </c>
+      <c r="E26">
+        <v>2020</v>
+      </c>
+      <c r="F26" t="s">
+        <v>330</v>
+      </c>
+      <c r="H26" s="2">
+        <v>1</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J26" s="2">
+        <v>1</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L26" s="2">
+        <v>1</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>353</v>
+      </c>
+      <c r="B27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" t="s">
+        <v>352</v>
+      </c>
+      <c r="E27">
+        <v>2020</v>
+      </c>
+      <c r="F27" t="s">
+        <v>332</v>
+      </c>
+      <c r="H27" s="2">
+        <v>1</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J27" s="2">
+        <v>1</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L27" s="2">
+        <v>1</v>
+      </c>
+      <c r="M27" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>354</v>
+      </c>
+      <c r="B28" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" t="s">
+        <v>352</v>
+      </c>
+      <c r="E28">
+        <v>2020</v>
+      </c>
+      <c r="F28" t="s">
+        <v>328</v>
+      </c>
+      <c r="H28" s="2">
+        <v>1</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J28" s="2">
+        <v>1</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L28" s="2">
+        <v>1</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>355</v>
+      </c>
+      <c r="B29" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" t="s">
+        <v>78</v>
+      </c>
+      <c r="E29">
+        <v>2020</v>
+      </c>
+      <c r="F29" t="s">
+        <v>356</v>
+      </c>
+      <c r="H29" s="2">
+        <v>1</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J29" s="2">
+        <v>1</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="L29" s="2">
+        <v>1</v>
+      </c>
+      <c r="M29" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <kae7f6409c1a45b5af70ba169c41da0e xmlns="82302deb-32b0-442b-bedc-ba64a9aa8ccd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </kae7f6409c1a45b5af70ba169c41da0e>
+    <REDD_x002f_NFM_x0020_category xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="82302deb-32b0-442b-bedc-ba64a9aa8ccd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003082C08FD3D0614AAB94B75C024070A7" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1a4b61487ffa532d49c6719891dd0d2e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="82302deb-32b0-442b-bedc-ba64a9aa8ccd" xmlns:ns3="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cea40d1c5f6ee0e5ae997cf8704aff88" ns2:_="" ns3:_="">
     <xsd:import namespace="82302deb-32b0-442b-bedc-ba64a9aa8ccd"/>
@@ -8125,34 +9407,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63A60D8A-7D1B-403D-BB2C-B10CCD11CB4B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="82302deb-32b0-442b-bedc-ba64a9aa8ccd"/>
+    <ds:schemaRef ds:uri="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <kae7f6409c1a45b5af70ba169c41da0e xmlns="82302deb-32b0-442b-bedc-ba64a9aa8ccd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </kae7f6409c1a45b5af70ba169c41da0e>
-    <REDD_x002f_NFM_x0020_category xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="82302deb-32b0-442b-bedc-ba64a9aa8ccd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5DBDC3B9-24A5-4D52-9DEE-E1BAF29BA53E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE6D2EE7-47BC-4B0F-B98D-543F5E3F8F03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8169,23 +9443,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5DBDC3B9-24A5-4D52-9DEE-E1BAF29BA53E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63A60D8A-7D1B-403D-BB2C-B10CCD11CB4B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="82302deb-32b0-442b-bedc-ba64a9aa8ccd"/>
-    <ds:schemaRef ds:uri="cc7ce8ca-8f52-44ec-9496-3c41d0f5ad18"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
keep ESRI only and gain 2020-2023 crop
</commit_message>
<xml_diff>
--- a/whisp_columns.xlsx
+++ b/whisp_columns.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnell\Documents\GitHub\whisp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\astri\Documents\FAO\test_degrad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07598504-323B-44EF-9C81-1DB66198FEFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F13A04-E6F9-4BB6-B53D-204FFC390426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Whisp outputs" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1490" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1478" uniqueCount="356">
   <si>
     <t>Column name</t>
   </si>
@@ -944,12 +944,6 @@
     <t>Karra 2021</t>
   </si>
   <si>
-    <t>GLC_FCS30D_TC_2022</t>
-  </si>
-  <si>
-    <t>Liangyun 2023</t>
-  </si>
-  <si>
     <t>Oil_palm_2023_FDaP</t>
   </si>
   <si>
@@ -965,15 +959,9 @@
     <t>Cocoa_2023_FDaP</t>
   </si>
   <si>
-    <t>ESRI_2023_crop</t>
-  </si>
-  <si>
     <t>Area of Crop</t>
   </si>
   <si>
-    <t>GLC_FCS30D_crop_2022</t>
-  </si>
-  <si>
     <t>GFW_logging_before_2020</t>
   </si>
   <si>
@@ -1095,6 +1083,12 @@
   </si>
   <si>
     <t>To maintain a consistent output format, numeric values will be converted to strings. Note: any multipolygons in the input will be split into individual parts, which may result in duplicate attribute values in the output.</t>
+  </si>
+  <si>
+    <t>ESRI_crop_gain_2020_2023</t>
+  </si>
+  <si>
+    <t>2020 and 2023</t>
   </si>
 </sst>
 </file>
@@ -1174,7 +1168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1195,16 +1189,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1510,14 +1500,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:N196"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:N194"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="33.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.453125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.26953125" style="7" bestFit="1" customWidth="1"/>
@@ -1542,7 +1532,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -1586,7 +1576,7 @@
       <c r="D2" t="s">
         <v>77</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" t="s">
         <v>76</v>
       </c>
       <c r="F2" t="s">
@@ -1627,7 +1617,7 @@
       <c r="D3" t="s">
         <v>77</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" t="s">
         <v>76</v>
       </c>
       <c r="F3" t="s">
@@ -1655,7 +1645,7 @@
         <v>76</v>
       </c>
       <c r="N3" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1671,7 +1661,7 @@
       <c r="D4" t="s">
         <v>85</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" t="s">
         <v>76</v>
       </c>
       <c r="F4" t="s">
@@ -1712,7 +1702,7 @@
       <c r="D5" t="s">
         <v>87</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" t="s">
         <v>76</v>
       </c>
       <c r="F5" t="s">
@@ -1753,7 +1743,7 @@
       <c r="D6" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" t="s">
         <v>76</v>
       </c>
       <c r="F6" t="s">
@@ -1794,7 +1784,7 @@
       <c r="D7" t="s">
         <v>92</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" t="s">
         <v>76</v>
       </c>
       <c r="F7" t="s">
@@ -1835,7 +1825,7 @@
       <c r="D8" t="s">
         <v>94</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" t="s">
         <v>76</v>
       </c>
       <c r="F8" t="s">
@@ -1876,7 +1866,7 @@
       <c r="D9" t="s">
         <v>97</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" t="s">
         <v>76</v>
       </c>
       <c r="F9" t="s">
@@ -1920,7 +1910,7 @@
       <c r="D10" t="s">
         <v>100</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" t="s">
         <v>76</v>
       </c>
       <c r="F10" t="s">
@@ -1964,7 +1954,7 @@
       <c r="D11" t="s">
         <v>103</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" t="s">
         <v>76</v>
       </c>
       <c r="F11" t="s">
@@ -2005,7 +1995,7 @@
       <c r="D12" t="s">
         <v>107</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="8">
         <v>2020</v>
       </c>
       <c r="F12" t="s">
@@ -2046,7 +2036,7 @@
       <c r="D13" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="8">
         <v>2020</v>
       </c>
       <c r="F13" t="s">
@@ -2087,7 +2077,7 @@
       <c r="D14" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="8">
         <v>2000</v>
       </c>
       <c r="F14" t="s">
@@ -2131,7 +2121,7 @@
       <c r="D15" t="s">
         <v>115</v>
       </c>
-      <c r="E15" s="9">
+      <c r="E15" s="8">
         <v>2020</v>
       </c>
       <c r="F15" t="s">
@@ -2172,7 +2162,7 @@
       <c r="D16" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16" s="8">
         <v>2020</v>
       </c>
       <c r="F16" t="s">
@@ -2213,7 +2203,7 @@
       <c r="D17" t="s">
         <v>120</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="8">
         <v>2020</v>
       </c>
       <c r="F17" t="s">
@@ -2254,7 +2244,7 @@
       <c r="D18" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="8">
         <v>2020</v>
       </c>
       <c r="F18" t="s">
@@ -2295,7 +2285,7 @@
       <c r="D19" t="s">
         <v>38</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="8">
         <v>2020</v>
       </c>
       <c r="F19" t="s">
@@ -2336,7 +2326,7 @@
       <c r="D20" t="s">
         <v>61</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="8">
         <v>2020</v>
       </c>
       <c r="F20" t="s">
@@ -2377,7 +2367,7 @@
       <c r="D21" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="9">
+      <c r="E21" s="8">
         <v>2020</v>
       </c>
       <c r="F21" t="s">
@@ -2418,7 +2408,7 @@
       <c r="D22" t="s">
         <v>59</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="8">
         <v>2020</v>
       </c>
       <c r="F22" t="s">
@@ -2459,7 +2449,7 @@
       <c r="D23" t="s">
         <v>73</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="8">
         <v>2020</v>
       </c>
       <c r="F23" t="s">
@@ -2500,7 +2490,7 @@
       <c r="D24" t="s">
         <v>73</v>
       </c>
-      <c r="E24" s="9">
+      <c r="E24" s="8">
         <v>2020</v>
       </c>
       <c r="F24" t="s">
@@ -2541,7 +2531,7 @@
       <c r="D25" t="s">
         <v>133</v>
       </c>
-      <c r="E25" s="9">
+      <c r="E25" s="8">
         <v>2020</v>
       </c>
       <c r="F25" t="s">
@@ -2582,7 +2572,7 @@
       <c r="D26" t="s">
         <v>133</v>
       </c>
-      <c r="E26" s="9">
+      <c r="E26" s="8">
         <v>2020</v>
       </c>
       <c r="F26" t="s">
@@ -2623,7 +2613,7 @@
       <c r="D27" t="s">
         <v>66</v>
       </c>
-      <c r="E27" s="9">
+      <c r="E27" s="8">
         <v>2020</v>
       </c>
       <c r="F27" t="s">
@@ -2664,7 +2654,7 @@
       <c r="D28" t="s">
         <v>45</v>
       </c>
-      <c r="E28" s="9">
+      <c r="E28" s="8">
         <v>2000</v>
       </c>
       <c r="F28" t="s">
@@ -2695,7 +2685,7 @@
       <c r="D29" t="s">
         <v>45</v>
       </c>
-      <c r="E29" s="9">
+      <c r="E29" s="8">
         <v>2001</v>
       </c>
       <c r="F29" t="s">
@@ -2726,7 +2716,7 @@
       <c r="D30" t="s">
         <v>45</v>
       </c>
-      <c r="E30" s="9">
+      <c r="E30" s="8">
         <v>2002</v>
       </c>
       <c r="F30" t="s">
@@ -2757,7 +2747,7 @@
       <c r="D31" t="s">
         <v>45</v>
       </c>
-      <c r="E31" s="9">
+      <c r="E31" s="8">
         <v>2003</v>
       </c>
       <c r="F31" t="s">
@@ -2788,7 +2778,7 @@
       <c r="D32" t="s">
         <v>45</v>
       </c>
-      <c r="E32" s="9">
+      <c r="E32" s="8">
         <v>2004</v>
       </c>
       <c r="F32" t="s">
@@ -2819,7 +2809,7 @@
       <c r="D33" t="s">
         <v>45</v>
       </c>
-      <c r="E33" s="9">
+      <c r="E33" s="8">
         <v>2005</v>
       </c>
       <c r="F33" t="s">
@@ -2850,7 +2840,7 @@
       <c r="D34" t="s">
         <v>45</v>
       </c>
-      <c r="E34" s="9">
+      <c r="E34" s="8">
         <v>2006</v>
       </c>
       <c r="F34" t="s">
@@ -2881,7 +2871,7 @@
       <c r="D35" t="s">
         <v>45</v>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="8">
         <v>2007</v>
       </c>
       <c r="F35" t="s">
@@ -2912,7 +2902,7 @@
       <c r="D36" t="s">
         <v>45</v>
       </c>
-      <c r="E36" s="9">
+      <c r="E36" s="8">
         <v>2008</v>
       </c>
       <c r="F36" t="s">
@@ -2943,7 +2933,7 @@
       <c r="D37" t="s">
         <v>45</v>
       </c>
-      <c r="E37" s="9">
+      <c r="E37" s="8">
         <v>2009</v>
       </c>
       <c r="F37" t="s">
@@ -2974,7 +2964,7 @@
       <c r="D38" t="s">
         <v>45</v>
       </c>
-      <c r="E38" s="9">
+      <c r="E38" s="8">
         <v>2010</v>
       </c>
       <c r="F38" t="s">
@@ -3005,7 +2995,7 @@
       <c r="D39" t="s">
         <v>45</v>
       </c>
-      <c r="E39" s="9">
+      <c r="E39" s="8">
         <v>2011</v>
       </c>
       <c r="F39" t="s">
@@ -3036,7 +3026,7 @@
       <c r="D40" t="s">
         <v>45</v>
       </c>
-      <c r="E40" s="9">
+      <c r="E40" s="8">
         <v>2012</v>
       </c>
       <c r="F40" t="s">
@@ -3067,7 +3057,7 @@
       <c r="D41" t="s">
         <v>45</v>
       </c>
-      <c r="E41" s="9">
+      <c r="E41" s="8">
         <v>2013</v>
       </c>
       <c r="F41" t="s">
@@ -3098,7 +3088,7 @@
       <c r="D42" t="s">
         <v>45</v>
       </c>
-      <c r="E42" s="9">
+      <c r="E42" s="8">
         <v>2014</v>
       </c>
       <c r="F42" t="s">
@@ -3129,7 +3119,7 @@
       <c r="D43" t="s">
         <v>45</v>
       </c>
-      <c r="E43" s="9">
+      <c r="E43" s="8">
         <v>2015</v>
       </c>
       <c r="F43" t="s">
@@ -3160,7 +3150,7 @@
       <c r="D44" t="s">
         <v>45</v>
       </c>
-      <c r="E44" s="9">
+      <c r="E44" s="8">
         <v>2016</v>
       </c>
       <c r="F44" t="s">
@@ -3191,7 +3181,7 @@
       <c r="D45" t="s">
         <v>45</v>
       </c>
-      <c r="E45" s="9">
+      <c r="E45" s="8">
         <v>2017</v>
       </c>
       <c r="F45" t="s">
@@ -3222,7 +3212,7 @@
       <c r="D46" t="s">
         <v>45</v>
       </c>
-      <c r="E46" s="9">
+      <c r="E46" s="8">
         <v>2018</v>
       </c>
       <c r="F46" t="s">
@@ -3253,7 +3243,7 @@
       <c r="D47" t="s">
         <v>45</v>
       </c>
-      <c r="E47" s="9">
+      <c r="E47" s="8">
         <v>2019</v>
       </c>
       <c r="F47" t="s">
@@ -3284,7 +3274,7 @@
       <c r="D48" t="s">
         <v>45</v>
       </c>
-      <c r="E48" s="9">
+      <c r="E48" s="8">
         <v>2020</v>
       </c>
       <c r="F48" t="s">
@@ -3315,7 +3305,7 @@
       <c r="D49" t="s">
         <v>45</v>
       </c>
-      <c r="E49" s="9">
+      <c r="E49" s="8">
         <v>2021</v>
       </c>
       <c r="F49" t="s">
@@ -3346,7 +3336,7 @@
       <c r="D50" t="s">
         <v>45</v>
       </c>
-      <c r="E50" s="9">
+      <c r="E50" s="8">
         <v>2022</v>
       </c>
       <c r="F50" t="s">
@@ -3377,7 +3367,7 @@
       <c r="D51" t="s">
         <v>45</v>
       </c>
-      <c r="E51" s="9">
+      <c r="E51" s="8">
         <v>2023</v>
       </c>
       <c r="F51" t="s">
@@ -3408,7 +3398,7 @@
       <c r="D52" t="s">
         <v>45</v>
       </c>
-      <c r="E52" s="9">
+      <c r="E52" s="8">
         <v>2024</v>
       </c>
       <c r="F52" t="s">
@@ -3439,7 +3429,7 @@
       <c r="D53" t="s">
         <v>49</v>
       </c>
-      <c r="E53" s="9">
+      <c r="E53" s="8">
         <v>2000</v>
       </c>
       <c r="F53" t="s">
@@ -3470,7 +3460,7 @@
       <c r="D54" t="s">
         <v>49</v>
       </c>
-      <c r="E54" s="9">
+      <c r="E54" s="8">
         <v>2001</v>
       </c>
       <c r="F54" t="s">
@@ -3501,7 +3491,7 @@
       <c r="D55" t="s">
         <v>49</v>
       </c>
-      <c r="E55" s="9">
+      <c r="E55" s="8">
         <v>2002</v>
       </c>
       <c r="F55" t="s">
@@ -3532,7 +3522,7 @@
       <c r="D56" t="s">
         <v>49</v>
       </c>
-      <c r="E56" s="9">
+      <c r="E56" s="8">
         <v>2003</v>
       </c>
       <c r="F56" t="s">
@@ -3563,7 +3553,7 @@
       <c r="D57" t="s">
         <v>49</v>
       </c>
-      <c r="E57" s="9">
+      <c r="E57" s="8">
         <v>2004</v>
       </c>
       <c r="F57" t="s">
@@ -3594,7 +3584,7 @@
       <c r="D58" t="s">
         <v>49</v>
       </c>
-      <c r="E58" s="9">
+      <c r="E58" s="8">
         <v>2005</v>
       </c>
       <c r="F58" t="s">
@@ -3625,7 +3615,7 @@
       <c r="D59" t="s">
         <v>49</v>
       </c>
-      <c r="E59" s="9">
+      <c r="E59" s="8">
         <v>2006</v>
       </c>
       <c r="F59" t="s">
@@ -3656,7 +3646,7 @@
       <c r="D60" t="s">
         <v>49</v>
       </c>
-      <c r="E60" s="9">
+      <c r="E60" s="8">
         <v>2007</v>
       </c>
       <c r="F60" t="s">
@@ -3687,7 +3677,7 @@
       <c r="D61" t="s">
         <v>49</v>
       </c>
-      <c r="E61" s="9">
+      <c r="E61" s="8">
         <v>2008</v>
       </c>
       <c r="F61" t="s">
@@ -3718,7 +3708,7 @@
       <c r="D62" t="s">
         <v>49</v>
       </c>
-      <c r="E62" s="9">
+      <c r="E62" s="8">
         <v>2009</v>
       </c>
       <c r="F62" t="s">
@@ -3749,7 +3739,7 @@
       <c r="D63" t="s">
         <v>49</v>
       </c>
-      <c r="E63" s="9">
+      <c r="E63" s="8">
         <v>2010</v>
       </c>
       <c r="F63" t="s">
@@ -3780,7 +3770,7 @@
       <c r="D64" t="s">
         <v>49</v>
       </c>
-      <c r="E64" s="9">
+      <c r="E64" s="8">
         <v>2011</v>
       </c>
       <c r="F64" t="s">
@@ -3811,7 +3801,7 @@
       <c r="D65" t="s">
         <v>49</v>
       </c>
-      <c r="E65" s="9">
+      <c r="E65" s="8">
         <v>2012</v>
       </c>
       <c r="F65" t="s">
@@ -3842,7 +3832,7 @@
       <c r="D66" t="s">
         <v>49</v>
       </c>
-      <c r="E66" s="9">
+      <c r="E66" s="8">
         <v>2013</v>
       </c>
       <c r="F66" t="s">
@@ -3873,7 +3863,7 @@
       <c r="D67" t="s">
         <v>49</v>
       </c>
-      <c r="E67" s="9">
+      <c r="E67" s="8">
         <v>2014</v>
       </c>
       <c r="F67" t="s">
@@ -3904,7 +3894,7 @@
       <c r="D68" t="s">
         <v>49</v>
       </c>
-      <c r="E68" s="9">
+      <c r="E68" s="8">
         <v>2015</v>
       </c>
       <c r="F68" t="s">
@@ -3935,7 +3925,7 @@
       <c r="D69" t="s">
         <v>49</v>
       </c>
-      <c r="E69" s="9">
+      <c r="E69" s="8">
         <v>2016</v>
       </c>
       <c r="F69" t="s">
@@ -3966,7 +3956,7 @@
       <c r="D70" t="s">
         <v>49</v>
       </c>
-      <c r="E70" s="9">
+      <c r="E70" s="8">
         <v>2017</v>
       </c>
       <c r="F70" t="s">
@@ -3997,7 +3987,7 @@
       <c r="D71" t="s">
         <v>49</v>
       </c>
-      <c r="E71" s="9">
+      <c r="E71" s="8">
         <v>2018</v>
       </c>
       <c r="F71" t="s">
@@ -4028,7 +4018,7 @@
       <c r="D72" t="s">
         <v>49</v>
       </c>
-      <c r="E72" s="9">
+      <c r="E72" s="8">
         <v>2019</v>
       </c>
       <c r="F72" t="s">
@@ -4059,7 +4049,7 @@
       <c r="D73" t="s">
         <v>49</v>
       </c>
-      <c r="E73" s="9">
+      <c r="E73" s="8">
         <v>2020</v>
       </c>
       <c r="F73" t="s">
@@ -4090,7 +4080,7 @@
       <c r="D74" t="s">
         <v>49</v>
       </c>
-      <c r="E74" s="9">
+      <c r="E74" s="8">
         <v>2021</v>
       </c>
       <c r="F74" t="s">
@@ -4121,7 +4111,7 @@
       <c r="D75" t="s">
         <v>49</v>
       </c>
-      <c r="E75" s="9">
+      <c r="E75" s="8">
         <v>2022</v>
       </c>
       <c r="F75" t="s">
@@ -4152,7 +4142,7 @@
       <c r="D76" t="s">
         <v>49</v>
       </c>
-      <c r="E76" s="9">
+      <c r="E76" s="8">
         <v>2023</v>
       </c>
       <c r="F76" t="s">
@@ -4183,7 +4173,7 @@
       <c r="D77" t="s">
         <v>49</v>
       </c>
-      <c r="E77" s="9">
+      <c r="E77" s="8">
         <v>2024</v>
       </c>
       <c r="F77" t="s">
@@ -4214,7 +4204,7 @@
       <c r="D78" t="s">
         <v>189</v>
       </c>
-      <c r="E78" s="9">
+      <c r="E78" s="8">
         <v>2001</v>
       </c>
       <c r="F78" t="s">
@@ -4245,7 +4235,7 @@
       <c r="D79" t="s">
         <v>189</v>
       </c>
-      <c r="E79" s="9">
+      <c r="E79" s="8">
         <v>2002</v>
       </c>
       <c r="F79" t="s">
@@ -4276,7 +4266,7 @@
       <c r="D80" t="s">
         <v>189</v>
       </c>
-      <c r="E80" s="9">
+      <c r="E80" s="8">
         <v>2003</v>
       </c>
       <c r="F80" t="s">
@@ -4307,7 +4297,7 @@
       <c r="D81" t="s">
         <v>189</v>
       </c>
-      <c r="E81" s="9">
+      <c r="E81" s="8">
         <v>2004</v>
       </c>
       <c r="F81" t="s">
@@ -4338,7 +4328,7 @@
       <c r="D82" t="s">
         <v>189</v>
       </c>
-      <c r="E82" s="9">
+      <c r="E82" s="8">
         <v>2005</v>
       </c>
       <c r="F82" t="s">
@@ -4369,7 +4359,7 @@
       <c r="D83" t="s">
         <v>189</v>
       </c>
-      <c r="E83" s="9">
+      <c r="E83" s="8">
         <v>2006</v>
       </c>
       <c r="F83" t="s">
@@ -4400,7 +4390,7 @@
       <c r="D84" t="s">
         <v>189</v>
       </c>
-      <c r="E84" s="9">
+      <c r="E84" s="8">
         <v>2007</v>
       </c>
       <c r="F84" t="s">
@@ -4431,7 +4421,7 @@
       <c r="D85" t="s">
         <v>189</v>
       </c>
-      <c r="E85" s="9">
+      <c r="E85" s="8">
         <v>2008</v>
       </c>
       <c r="F85" t="s">
@@ -4462,7 +4452,7 @@
       <c r="D86" t="s">
         <v>189</v>
       </c>
-      <c r="E86" s="9">
+      <c r="E86" s="8">
         <v>2009</v>
       </c>
       <c r="F86" t="s">
@@ -4493,7 +4483,7 @@
       <c r="D87" t="s">
         <v>189</v>
       </c>
-      <c r="E87" s="9">
+      <c r="E87" s="8">
         <v>2010</v>
       </c>
       <c r="F87" t="s">
@@ -4524,7 +4514,7 @@
       <c r="D88" t="s">
         <v>189</v>
       </c>
-      <c r="E88" s="9">
+      <c r="E88" s="8">
         <v>2011</v>
       </c>
       <c r="F88" t="s">
@@ -4555,7 +4545,7 @@
       <c r="D89" t="s">
         <v>189</v>
       </c>
-      <c r="E89" s="9">
+      <c r="E89" s="8">
         <v>2012</v>
       </c>
       <c r="F89" t="s">
@@ -4586,7 +4576,7 @@
       <c r="D90" t="s">
         <v>189</v>
       </c>
-      <c r="E90" s="9">
+      <c r="E90" s="8">
         <v>2013</v>
       </c>
       <c r="F90" t="s">
@@ -4617,7 +4607,7 @@
       <c r="D91" t="s">
         <v>189</v>
       </c>
-      <c r="E91" s="9">
+      <c r="E91" s="8">
         <v>2014</v>
       </c>
       <c r="F91" t="s">
@@ -4648,7 +4638,7 @@
       <c r="D92" t="s">
         <v>189</v>
       </c>
-      <c r="E92" s="9">
+      <c r="E92" s="8">
         <v>2015</v>
       </c>
       <c r="F92" t="s">
@@ -4679,7 +4669,7 @@
       <c r="D93" t="s">
         <v>189</v>
       </c>
-      <c r="E93" s="9">
+      <c r="E93" s="8">
         <v>2016</v>
       </c>
       <c r="F93" t="s">
@@ -4710,7 +4700,7 @@
       <c r="D94" t="s">
         <v>189</v>
       </c>
-      <c r="E94" s="9">
+      <c r="E94" s="8">
         <v>2017</v>
       </c>
       <c r="F94" t="s">
@@ -4741,7 +4731,7 @@
       <c r="D95" t="s">
         <v>189</v>
       </c>
-      <c r="E95" s="9">
+      <c r="E95" s="8">
         <v>2018</v>
       </c>
       <c r="F95" t="s">
@@ -4772,7 +4762,7 @@
       <c r="D96" t="s">
         <v>189</v>
       </c>
-      <c r="E96" s="9">
+      <c r="E96" s="8">
         <v>2019</v>
       </c>
       <c r="F96" t="s">
@@ -4803,7 +4793,7 @@
       <c r="D97" t="s">
         <v>189</v>
       </c>
-      <c r="E97" s="9">
+      <c r="E97" s="8">
         <v>2020</v>
       </c>
       <c r="F97" t="s">
@@ -4834,7 +4824,7 @@
       <c r="D98" t="s">
         <v>189</v>
       </c>
-      <c r="E98" s="9">
+      <c r="E98" s="8">
         <v>2021</v>
       </c>
       <c r="F98" t="s">
@@ -4865,7 +4855,7 @@
       <c r="D99" t="s">
         <v>189</v>
       </c>
-      <c r="E99" s="9">
+      <c r="E99" s="8">
         <v>2022</v>
       </c>
       <c r="F99" t="s">
@@ -4896,7 +4886,7 @@
       <c r="D100" t="s">
         <v>189</v>
       </c>
-      <c r="E100" s="9">
+      <c r="E100" s="8">
         <v>2023</v>
       </c>
       <c r="F100" t="s">
@@ -4927,7 +4917,7 @@
       <c r="D101" t="s">
         <v>189</v>
       </c>
-      <c r="E101" s="9">
+      <c r="E101" s="8">
         <v>2024</v>
       </c>
       <c r="F101" t="s">
@@ -4958,7 +4948,7 @@
       <c r="D102" t="s">
         <v>189</v>
       </c>
-      <c r="E102" s="9">
+      <c r="E102" s="8">
         <v>2019</v>
       </c>
       <c r="F102" t="s">
@@ -4989,7 +4979,7 @@
       <c r="D103" t="s">
         <v>189</v>
       </c>
-      <c r="E103" s="9">
+      <c r="E103" s="8">
         <v>2020</v>
       </c>
       <c r="F103" t="s">
@@ -5020,7 +5010,7 @@
       <c r="D104" t="s">
         <v>189</v>
       </c>
-      <c r="E104" s="9">
+      <c r="E104" s="8">
         <v>2021</v>
       </c>
       <c r="F104" t="s">
@@ -5051,7 +5041,7 @@
       <c r="D105" t="s">
         <v>189</v>
       </c>
-      <c r="E105" s="9">
+      <c r="E105" s="8">
         <v>2022</v>
       </c>
       <c r="F105" t="s">
@@ -5082,7 +5072,7 @@
       <c r="D106" t="s">
         <v>189</v>
       </c>
-      <c r="E106" s="9">
+      <c r="E106" s="8">
         <v>2023</v>
       </c>
       <c r="F106" t="s">
@@ -5113,7 +5103,7 @@
       <c r="D107" t="s">
         <v>189</v>
       </c>
-      <c r="E107" s="9">
+      <c r="E107" s="8">
         <v>2024</v>
       </c>
       <c r="F107" t="s">
@@ -5144,7 +5134,7 @@
       <c r="D108" t="s">
         <v>189</v>
       </c>
-      <c r="E108" s="9">
+      <c r="E108" s="8">
         <v>2025</v>
       </c>
       <c r="F108" t="s">
@@ -5175,7 +5165,7 @@
       <c r="D109" t="s">
         <v>222</v>
       </c>
-      <c r="E109" s="9">
+      <c r="E109" s="8">
         <v>2001</v>
       </c>
       <c r="F109" t="s">
@@ -5206,7 +5196,7 @@
       <c r="D110" t="s">
         <v>222</v>
       </c>
-      <c r="E110" s="9">
+      <c r="E110" s="8">
         <v>2002</v>
       </c>
       <c r="F110" t="s">
@@ -5237,7 +5227,7 @@
       <c r="D111" t="s">
         <v>222</v>
       </c>
-      <c r="E111" s="9">
+      <c r="E111" s="8">
         <v>2003</v>
       </c>
       <c r="F111" t="s">
@@ -5268,7 +5258,7 @@
       <c r="D112" t="s">
         <v>222</v>
       </c>
-      <c r="E112" s="9">
+      <c r="E112" s="8">
         <v>2004</v>
       </c>
       <c r="F112" t="s">
@@ -5299,7 +5289,7 @@
       <c r="D113" t="s">
         <v>222</v>
       </c>
-      <c r="E113" s="9">
+      <c r="E113" s="8">
         <v>2005</v>
       </c>
       <c r="F113" t="s">
@@ -5330,7 +5320,7 @@
       <c r="D114" t="s">
         <v>222</v>
       </c>
-      <c r="E114" s="9">
+      <c r="E114" s="8">
         <v>2006</v>
       </c>
       <c r="F114" t="s">
@@ -5361,7 +5351,7 @@
       <c r="D115" t="s">
         <v>222</v>
       </c>
-      <c r="E115" s="9">
+      <c r="E115" s="8">
         <v>2007</v>
       </c>
       <c r="F115" t="s">
@@ -5392,7 +5382,7 @@
       <c r="D116" t="s">
         <v>222</v>
       </c>
-      <c r="E116" s="9">
+      <c r="E116" s="8">
         <v>2008</v>
       </c>
       <c r="F116" t="s">
@@ -5423,7 +5413,7 @@
       <c r="D117" t="s">
         <v>222</v>
       </c>
-      <c r="E117" s="9">
+      <c r="E117" s="8">
         <v>2009</v>
       </c>
       <c r="F117" t="s">
@@ -5454,7 +5444,7 @@
       <c r="D118" t="s">
         <v>222</v>
       </c>
-      <c r="E118" s="9">
+      <c r="E118" s="8">
         <v>2010</v>
       </c>
       <c r="F118" t="s">
@@ -5485,7 +5475,7 @@
       <c r="D119" t="s">
         <v>222</v>
       </c>
-      <c r="E119" s="9">
+      <c r="E119" s="8">
         <v>2011</v>
       </c>
       <c r="F119" t="s">
@@ -5516,7 +5506,7 @@
       <c r="D120" t="s">
         <v>222</v>
       </c>
-      <c r="E120" s="9">
+      <c r="E120" s="8">
         <v>2012</v>
       </c>
       <c r="F120" t="s">
@@ -5547,7 +5537,7 @@
       <c r="D121" t="s">
         <v>222</v>
       </c>
-      <c r="E121" s="9">
+      <c r="E121" s="8">
         <v>2013</v>
       </c>
       <c r="F121" t="s">
@@ -5578,7 +5568,7 @@
       <c r="D122" t="s">
         <v>222</v>
       </c>
-      <c r="E122" s="9">
+      <c r="E122" s="8">
         <v>2014</v>
       </c>
       <c r="F122" t="s">
@@ -5609,7 +5599,7 @@
       <c r="D123" t="s">
         <v>222</v>
       </c>
-      <c r="E123" s="9">
+      <c r="E123" s="8">
         <v>2015</v>
       </c>
       <c r="F123" t="s">
@@ -5640,7 +5630,7 @@
       <c r="D124" t="s">
         <v>222</v>
       </c>
-      <c r="E124" s="9">
+      <c r="E124" s="8">
         <v>2016</v>
       </c>
       <c r="F124" t="s">
@@ -5671,7 +5661,7 @@
       <c r="D125" t="s">
         <v>222</v>
       </c>
-      <c r="E125" s="9">
+      <c r="E125" s="8">
         <v>2017</v>
       </c>
       <c r="F125" t="s">
@@ -5702,7 +5692,7 @@
       <c r="D126" t="s">
         <v>222</v>
       </c>
-      <c r="E126" s="9">
+      <c r="E126" s="8">
         <v>2018</v>
       </c>
       <c r="F126" t="s">
@@ -5733,7 +5723,7 @@
       <c r="D127" t="s">
         <v>222</v>
       </c>
-      <c r="E127" s="9">
+      <c r="E127" s="8">
         <v>2019</v>
       </c>
       <c r="F127" t="s">
@@ -5764,7 +5754,7 @@
       <c r="D128" t="s">
         <v>222</v>
       </c>
-      <c r="E128" s="9">
+      <c r="E128" s="8">
         <v>2020</v>
       </c>
       <c r="F128" t="s">
@@ -5795,7 +5785,7 @@
       <c r="D129" t="s">
         <v>222</v>
       </c>
-      <c r="E129" s="9">
+      <c r="E129" s="8">
         <v>2000</v>
       </c>
       <c r="F129" t="s">
@@ -5826,7 +5816,7 @@
       <c r="D130" t="s">
         <v>222</v>
       </c>
-      <c r="E130" s="9">
+      <c r="E130" s="8">
         <v>2001</v>
       </c>
       <c r="F130" t="s">
@@ -5857,7 +5847,7 @@
       <c r="D131" t="s">
         <v>222</v>
       </c>
-      <c r="E131" s="9">
+      <c r="E131" s="8">
         <v>2002</v>
       </c>
       <c r="F131" t="s">
@@ -5888,7 +5878,7 @@
       <c r="D132" t="s">
         <v>222</v>
       </c>
-      <c r="E132" s="9">
+      <c r="E132" s="8">
         <v>2003</v>
       </c>
       <c r="F132" t="s">
@@ -5919,7 +5909,7 @@
       <c r="D133" t="s">
         <v>222</v>
       </c>
-      <c r="E133" s="9">
+      <c r="E133" s="8">
         <v>2004</v>
       </c>
       <c r="F133" t="s">
@@ -5950,7 +5940,7 @@
       <c r="D134" t="s">
         <v>222</v>
       </c>
-      <c r="E134" s="9">
+      <c r="E134" s="8">
         <v>2005</v>
       </c>
       <c r="F134" t="s">
@@ -5981,7 +5971,7 @@
       <c r="D135" t="s">
         <v>222</v>
       </c>
-      <c r="E135" s="9">
+      <c r="E135" s="8">
         <v>2006</v>
       </c>
       <c r="F135" t="s">
@@ -6012,7 +6002,7 @@
       <c r="D136" t="s">
         <v>222</v>
       </c>
-      <c r="E136" s="9">
+      <c r="E136" s="8">
         <v>2007</v>
       </c>
       <c r="F136" t="s">
@@ -6043,7 +6033,7 @@
       <c r="D137" t="s">
         <v>222</v>
       </c>
-      <c r="E137" s="9">
+      <c r="E137" s="8">
         <v>2008</v>
       </c>
       <c r="F137" t="s">
@@ -6074,7 +6064,7 @@
       <c r="D138" t="s">
         <v>222</v>
       </c>
-      <c r="E138" s="9">
+      <c r="E138" s="8">
         <v>2009</v>
       </c>
       <c r="F138" t="s">
@@ -6105,7 +6095,7 @@
       <c r="D139" t="s">
         <v>222</v>
       </c>
-      <c r="E139" s="9">
+      <c r="E139" s="8">
         <v>2010</v>
       </c>
       <c r="F139" t="s">
@@ -6136,7 +6126,7 @@
       <c r="D140" t="s">
         <v>222</v>
       </c>
-      <c r="E140" s="9">
+      <c r="E140" s="8">
         <v>2011</v>
       </c>
       <c r="F140" t="s">
@@ -6167,7 +6157,7 @@
       <c r="D141" t="s">
         <v>222</v>
       </c>
-      <c r="E141" s="9">
+      <c r="E141" s="8">
         <v>2012</v>
       </c>
       <c r="F141" t="s">
@@ -6198,7 +6188,7 @@
       <c r="D142" t="s">
         <v>222</v>
       </c>
-      <c r="E142" s="9">
+      <c r="E142" s="8">
         <v>2013</v>
       </c>
       <c r="F142" t="s">
@@ -6229,7 +6219,7 @@
       <c r="D143" t="s">
         <v>222</v>
       </c>
-      <c r="E143" s="9">
+      <c r="E143" s="8">
         <v>2014</v>
       </c>
       <c r="F143" t="s">
@@ -6260,7 +6250,7 @@
       <c r="D144" t="s">
         <v>222</v>
       </c>
-      <c r="E144" s="9">
+      <c r="E144" s="8">
         <v>2015</v>
       </c>
       <c r="F144" t="s">
@@ -6291,7 +6281,7 @@
       <c r="D145" t="s">
         <v>222</v>
       </c>
-      <c r="E145" s="9">
+      <c r="E145" s="8">
         <v>2016</v>
       </c>
       <c r="F145" t="s">
@@ -6322,7 +6312,7 @@
       <c r="D146" t="s">
         <v>222</v>
       </c>
-      <c r="E146" s="9">
+      <c r="E146" s="8">
         <v>2017</v>
       </c>
       <c r="F146" t="s">
@@ -6353,7 +6343,7 @@
       <c r="D147" t="s">
         <v>222</v>
       </c>
-      <c r="E147" s="9">
+      <c r="E147" s="8">
         <v>2018</v>
       </c>
       <c r="F147" t="s">
@@ -6384,7 +6374,7 @@
       <c r="D148" t="s">
         <v>222</v>
       </c>
-      <c r="E148" s="9">
+      <c r="E148" s="8">
         <v>2019</v>
       </c>
       <c r="F148" t="s">
@@ -6415,7 +6405,7 @@
       <c r="D149" t="s">
         <v>222</v>
       </c>
-      <c r="E149" s="9">
+      <c r="E149" s="8">
         <v>2020</v>
       </c>
       <c r="F149" t="s">
@@ -6446,7 +6436,7 @@
       <c r="D150" t="s">
         <v>222</v>
       </c>
-      <c r="E150" s="9">
+      <c r="E150" s="8">
         <v>2021</v>
       </c>
       <c r="F150" t="s">
@@ -6477,7 +6467,7 @@
       <c r="D151" t="s">
         <v>222</v>
       </c>
-      <c r="E151" s="9">
+      <c r="E151" s="8">
         <v>2022</v>
       </c>
       <c r="F151" t="s">
@@ -6508,7 +6498,7 @@
       <c r="D152" t="s">
         <v>222</v>
       </c>
-      <c r="E152" s="9">
+      <c r="E152" s="8">
         <v>2023</v>
       </c>
       <c r="F152" t="s">
@@ -6539,7 +6529,7 @@
       <c r="D153" t="s">
         <v>222</v>
       </c>
-      <c r="E153" s="9">
+      <c r="E153" s="8">
         <v>2024</v>
       </c>
       <c r="F153" t="s">
@@ -6570,7 +6560,7 @@
       <c r="D154" t="s">
         <v>222</v>
       </c>
-      <c r="E154" s="9">
+      <c r="E154" s="8">
         <v>2025</v>
       </c>
       <c r="F154" t="s">
@@ -6601,7 +6591,7 @@
       <c r="D155" t="s">
         <v>49</v>
       </c>
-      <c r="E155" s="11" t="s">
+      <c r="E155" t="s">
         <v>271</v>
       </c>
       <c r="F155" t="s">
@@ -6637,7 +6627,7 @@
       <c r="D156" t="s">
         <v>45</v>
       </c>
-      <c r="E156" s="11" t="s">
+      <c r="E156" t="s">
         <v>271</v>
       </c>
       <c r="F156" t="s">
@@ -6673,7 +6663,7 @@
       <c r="D157" t="s">
         <v>189</v>
       </c>
-      <c r="E157" s="11" t="s">
+      <c r="E157" t="s">
         <v>271</v>
       </c>
       <c r="F157" t="s">
@@ -6709,7 +6699,7 @@
       <c r="D158" t="s">
         <v>275</v>
       </c>
-      <c r="E158" s="11" t="s">
+      <c r="E158" t="s">
         <v>271</v>
       </c>
       <c r="F158" t="s">
@@ -6745,7 +6735,7 @@
       <c r="D159" t="s">
         <v>275</v>
       </c>
-      <c r="E159" s="11" t="s">
+      <c r="E159" t="s">
         <v>271</v>
       </c>
       <c r="F159" t="s">
@@ -6781,7 +6771,7 @@
       <c r="D160" t="s">
         <v>189</v>
       </c>
-      <c r="E160" s="11" t="s">
+      <c r="E160" t="s">
         <v>278</v>
       </c>
       <c r="F160" t="s">
@@ -6817,7 +6807,7 @@
       <c r="D161" t="s">
         <v>49</v>
       </c>
-      <c r="E161" s="11" t="s">
+      <c r="E161" t="s">
         <v>280</v>
       </c>
       <c r="F161" t="s">
@@ -6855,7 +6845,7 @@
       <c r="D162" t="s">
         <v>45</v>
       </c>
-      <c r="E162" s="11" t="s">
+      <c r="E162" t="s">
         <v>280</v>
       </c>
       <c r="F162" t="s">
@@ -6893,7 +6883,7 @@
       <c r="D163" t="s">
         <v>189</v>
       </c>
-      <c r="E163" s="11" t="s">
+      <c r="E163" t="s">
         <v>280</v>
       </c>
       <c r="F163" t="s">
@@ -6931,7 +6921,7 @@
       <c r="D164" t="s">
         <v>284</v>
       </c>
-      <c r="E164" s="11" t="s">
+      <c r="E164" t="s">
         <v>285</v>
       </c>
       <c r="F164" t="s">
@@ -6969,7 +6959,7 @@
       <c r="D165" t="s">
         <v>189</v>
       </c>
-      <c r="E165" s="11" t="s">
+      <c r="E165" t="s">
         <v>280</v>
       </c>
       <c r="F165" t="s">
@@ -7007,7 +6997,7 @@
       <c r="D166" t="s">
         <v>23</v>
       </c>
-      <c r="E166" s="9">
+      <c r="E166" s="8">
         <v>2020</v>
       </c>
       <c r="F166" t="s">
@@ -7044,7 +7034,7 @@
       <c r="D167" t="s">
         <v>289</v>
       </c>
-      <c r="E167" s="9">
+      <c r="E167" s="8">
         <v>2020</v>
       </c>
       <c r="F167" t="s">
@@ -7081,7 +7071,7 @@
       <c r="D168" t="s">
         <v>23</v>
       </c>
-      <c r="E168" s="9">
+      <c r="E168" s="8">
         <v>2020</v>
       </c>
       <c r="F168" t="s">
@@ -7118,7 +7108,7 @@
       <c r="D169" t="s">
         <v>294</v>
       </c>
-      <c r="E169" s="9">
+      <c r="E169" s="8">
         <v>2020</v>
       </c>
       <c r="F169" t="s">
@@ -7155,7 +7145,7 @@
       <c r="D170" t="s">
         <v>296</v>
       </c>
-      <c r="E170" s="9">
+      <c r="E170" s="8">
         <v>2020</v>
       </c>
       <c r="F170" t="s">
@@ -7192,7 +7182,7 @@
       <c r="D171" t="s">
         <v>298</v>
       </c>
-      <c r="E171" s="9">
+      <c r="E171" s="8">
         <v>2015</v>
       </c>
       <c r="F171" t="s">
@@ -7229,7 +7219,7 @@
       <c r="D172" t="s">
         <v>302</v>
       </c>
-      <c r="E172" s="9">
+      <c r="E172" s="8">
         <v>2023</v>
       </c>
       <c r="F172" t="s">
@@ -7266,7 +7256,7 @@
       <c r="D173" t="s">
         <v>305</v>
       </c>
-      <c r="E173" s="9">
+      <c r="E173" s="8">
         <v>2023</v>
       </c>
       <c r="F173" t="s">
@@ -7298,13 +7288,16 @@
         <v>16</v>
       </c>
       <c r="D174" t="s">
-        <v>305</v>
-      </c>
-      <c r="E174" s="9">
-        <v>2022</v>
+        <v>61</v>
+      </c>
+      <c r="E174" s="8">
+        <v>2023</v>
       </c>
       <c r="F174" t="s">
-        <v>308</v>
+        <v>121</v>
+      </c>
+      <c r="G174" t="s">
+        <v>79</v>
       </c>
       <c r="H174" s="3">
         <v>0</v>
@@ -7318,7 +7311,7 @@
         <v>1</v>
       </c>
       <c r="M174" s="4" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
     </row>
     <row r="175" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -7332,9 +7325,9 @@
         <v>16</v>
       </c>
       <c r="D175" t="s">
-        <v>61</v>
-      </c>
-      <c r="E175" s="9">
+        <v>133</v>
+      </c>
+      <c r="E175" s="8">
         <v>2023</v>
       </c>
       <c r="F175" t="s">
@@ -7355,12 +7348,12 @@
         <v>1</v>
       </c>
       <c r="M175" s="4" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="176" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B176" t="s">
         <v>15</v>
@@ -7369,9 +7362,9 @@
         <v>16</v>
       </c>
       <c r="D176" t="s">
-        <v>133</v>
-      </c>
-      <c r="E176" s="9">
+        <v>59</v>
+      </c>
+      <c r="E176" s="8">
         <v>2023</v>
       </c>
       <c r="F176" t="s">
@@ -7392,12 +7385,12 @@
         <v>1</v>
       </c>
       <c r="M176" s="4" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="177" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B177" t="s">
         <v>15</v>
@@ -7406,9 +7399,9 @@
         <v>16</v>
       </c>
       <c r="D177" t="s">
-        <v>59</v>
-      </c>
-      <c r="E177" s="9">
+        <v>73</v>
+      </c>
+      <c r="E177" s="8">
         <v>2023</v>
       </c>
       <c r="F177" t="s">
@@ -7429,12 +7422,12 @@
         <v>1</v>
       </c>
       <c r="M177" s="4" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="178" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
-        <v>313</v>
+        <v>354</v>
       </c>
       <c r="B178" t="s">
         <v>15</v>
@@ -7443,13 +7436,13 @@
         <v>16</v>
       </c>
       <c r="D178" t="s">
-        <v>73</v>
-      </c>
-      <c r="E178" s="9">
-        <v>2023</v>
+        <v>312</v>
+      </c>
+      <c r="E178" s="8" t="s">
+        <v>355</v>
       </c>
       <c r="F178" t="s">
-        <v>121</v>
+        <v>306</v>
       </c>
       <c r="G178" t="s">
         <v>79</v>
@@ -7466,27 +7459,27 @@
         <v>1</v>
       </c>
       <c r="M178" s="4" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="179" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
+        <v>313</v>
+      </c>
+      <c r="B179" t="s">
+        <v>15</v>
+      </c>
+      <c r="C179" t="s">
+        <v>16</v>
+      </c>
+      <c r="D179" t="s">
         <v>314</v>
       </c>
-      <c r="B179" t="s">
-        <v>15</v>
-      </c>
-      <c r="C179" t="s">
-        <v>16</v>
-      </c>
-      <c r="D179" t="s">
+      <c r="E179" s="8">
+        <v>2015</v>
+      </c>
+      <c r="F179" t="s">
         <v>315</v>
-      </c>
-      <c r="E179" s="9">
-        <v>2023</v>
-      </c>
-      <c r="F179" t="s">
-        <v>306</v>
       </c>
       <c r="G179" t="s">
         <v>79</v>
@@ -7503,101 +7496,79 @@
         <v>1</v>
       </c>
       <c r="M179" s="4" t="s">
-        <v>310</v>
+        <v>316</v>
+      </c>
+      <c r="N179" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="180" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B180" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="C180" t="s">
-        <v>16</v>
+        <v>76</v>
       </c>
       <c r="D180" t="s">
-        <v>315</v>
-      </c>
-      <c r="E180" s="9">
-        <v>2022</v>
+        <v>319</v>
+      </c>
+      <c r="E180" t="s">
+        <v>76</v>
       </c>
       <c r="F180" t="s">
-        <v>308</v>
+        <v>78</v>
       </c>
       <c r="G180" t="s">
         <v>79</v>
       </c>
-      <c r="H180" s="3">
-        <v>0</v>
-      </c>
-      <c r="I180" s="4"/>
-      <c r="J180" s="3">
-        <v>0</v>
-      </c>
-      <c r="K180" s="4"/>
-      <c r="L180" s="3">
-        <v>1</v>
-      </c>
-      <c r="M180" s="4" t="s">
-        <v>310</v>
+      <c r="N180" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="181" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B181" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="C181" t="s">
-        <v>16</v>
+        <v>321</v>
       </c>
       <c r="D181" t="s">
-        <v>318</v>
-      </c>
-      <c r="E181" s="9">
-        <v>2015</v>
+        <v>322</v>
+      </c>
+      <c r="E181" s="8">
+        <v>2020</v>
       </c>
       <c r="F181" t="s">
-        <v>319</v>
+        <v>78</v>
       </c>
       <c r="G181" t="s">
         <v>79</v>
       </c>
-      <c r="H181" s="3">
-        <v>0</v>
-      </c>
-      <c r="I181" s="4"/>
-      <c r="J181" s="3">
-        <v>0</v>
-      </c>
-      <c r="K181" s="4"/>
-      <c r="L181" s="3">
-        <v>1</v>
-      </c>
-      <c r="M181" s="4" t="s">
-        <v>320</v>
-      </c>
       <c r="N181" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="182" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B182" t="s">
         <v>81</v>
       </c>
       <c r="C182" t="s">
-        <v>76</v>
+        <v>321</v>
       </c>
       <c r="D182" t="s">
-        <v>323</v>
-      </c>
-      <c r="E182" s="11" t="s">
-        <v>76</v>
+        <v>325</v>
+      </c>
+      <c r="E182" s="8">
+        <v>2020</v>
       </c>
       <c r="F182" t="s">
         <v>78</v>
@@ -7606,24 +7577,24 @@
         <v>79</v>
       </c>
       <c r="N182" t="s">
-        <v>98</v>
+        <v>323</v>
       </c>
     </row>
     <row r="183" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B183" t="s">
         <v>81</v>
       </c>
       <c r="C183" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D183" t="s">
-        <v>326</v>
-      </c>
-      <c r="E183" s="9">
-        <v>2020</v>
+        <v>327</v>
+      </c>
+      <c r="E183" t="s">
+        <v>271</v>
       </c>
       <c r="F183" t="s">
         <v>78</v>
@@ -7632,7 +7603,7 @@
         <v>79</v>
       </c>
       <c r="N183" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="184" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -7643,13 +7614,13 @@
         <v>81</v>
       </c>
       <c r="C184" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D184" t="s">
+        <v>327</v>
+      </c>
+      <c r="E184" t="s">
         <v>329</v>
-      </c>
-      <c r="E184" s="9">
-        <v>2020</v>
       </c>
       <c r="F184" t="s">
         <v>78</v>
@@ -7658,7 +7629,7 @@
         <v>79</v>
       </c>
       <c r="N184" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="185" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -7669,13 +7640,13 @@
         <v>81</v>
       </c>
       <c r="C185" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D185" t="s">
         <v>331</v>
       </c>
-      <c r="E185" s="11" t="s">
-        <v>271</v>
+      <c r="E185" s="8">
+        <v>2020</v>
       </c>
       <c r="F185" t="s">
         <v>78</v>
@@ -7684,7 +7655,7 @@
         <v>79</v>
       </c>
       <c r="N185" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="186" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -7695,13 +7666,13 @@
         <v>81</v>
       </c>
       <c r="C186" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D186" t="s">
-        <v>331</v>
-      </c>
-      <c r="E186" s="11" t="s">
         <v>333</v>
+      </c>
+      <c r="E186" s="8">
+        <v>2020</v>
       </c>
       <c r="F186" t="s">
         <v>78</v>
@@ -7710,7 +7681,7 @@
         <v>79</v>
       </c>
       <c r="N186" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="187" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -7721,12 +7692,12 @@
         <v>81</v>
       </c>
       <c r="C187" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D187" t="s">
         <v>335</v>
       </c>
-      <c r="E187" s="9">
+      <c r="E187" s="8">
         <v>2020</v>
       </c>
       <c r="F187" t="s">
@@ -7736,7 +7707,7 @@
         <v>79</v>
       </c>
       <c r="N187" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="188" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -7747,13 +7718,13 @@
         <v>81</v>
       </c>
       <c r="C188" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D188" t="s">
-        <v>337</v>
-      </c>
-      <c r="E188" s="9">
-        <v>2020</v>
+        <v>335</v>
+      </c>
+      <c r="E188" t="s">
+        <v>329</v>
       </c>
       <c r="F188" t="s">
         <v>78</v>
@@ -7762,24 +7733,24 @@
         <v>79</v>
       </c>
       <c r="N188" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="189" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B189" t="s">
         <v>81</v>
       </c>
       <c r="C189" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D189" t="s">
-        <v>339</v>
-      </c>
-      <c r="E189" s="9">
-        <v>2020</v>
+        <v>322</v>
+      </c>
+      <c r="E189" t="s">
+        <v>329</v>
       </c>
       <c r="F189" t="s">
         <v>78</v>
@@ -7788,24 +7759,24 @@
         <v>79</v>
       </c>
       <c r="N189" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="190" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B190" t="s">
         <v>81</v>
       </c>
       <c r="C190" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D190" t="s">
         <v>339</v>
       </c>
-      <c r="E190" s="11" t="s">
-        <v>333</v>
+      <c r="E190" t="s">
+        <v>329</v>
       </c>
       <c r="F190" t="s">
         <v>78</v>
@@ -7814,24 +7785,24 @@
         <v>79</v>
       </c>
       <c r="N190" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="191" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B191" t="s">
         <v>81</v>
       </c>
       <c r="C191" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D191" t="s">
-        <v>326</v>
-      </c>
-      <c r="E191" s="11" t="s">
-        <v>333</v>
+        <v>341</v>
+      </c>
+      <c r="E191" s="8">
+        <v>2015</v>
       </c>
       <c r="F191" t="s">
         <v>78</v>
@@ -7840,7 +7811,7 @@
         <v>79</v>
       </c>
       <c r="N191" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="192" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -7851,13 +7822,13 @@
         <v>81</v>
       </c>
       <c r="C192" t="s">
-        <v>325</v>
+        <v>343</v>
       </c>
       <c r="D192" t="s">
-        <v>343</v>
-      </c>
-      <c r="E192" s="11" t="s">
-        <v>333</v>
+        <v>344</v>
+      </c>
+      <c r="E192" t="s">
+        <v>76</v>
       </c>
       <c r="F192" t="s">
         <v>78</v>
@@ -7866,24 +7837,24 @@
         <v>79</v>
       </c>
       <c r="N192" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
     </row>
     <row r="193" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B193" t="s">
         <v>81</v>
       </c>
       <c r="C193" t="s">
-        <v>325</v>
+        <v>343</v>
       </c>
       <c r="D193" t="s">
-        <v>345</v>
-      </c>
-      <c r="E193" s="9">
-        <v>2015</v>
+        <v>347</v>
+      </c>
+      <c r="E193" t="s">
+        <v>76</v>
       </c>
       <c r="F193" t="s">
         <v>78</v>
@@ -7892,23 +7863,23 @@
         <v>79</v>
       </c>
       <c r="N193" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="194" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="194" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B194" t="s">
         <v>81</v>
       </c>
       <c r="C194" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="D194" t="s">
-        <v>348</v>
-      </c>
-      <c r="E194" s="11" t="s">
+        <v>350</v>
+      </c>
+      <c r="E194" t="s">
         <v>76</v>
       </c>
       <c r="F194" t="s">
@@ -7918,59 +7889,7 @@
         <v>79</v>
       </c>
       <c r="N194" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="195" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A195" t="s">
-        <v>350</v>
-      </c>
-      <c r="B195" t="s">
-        <v>81</v>
-      </c>
-      <c r="C195" t="s">
-        <v>347</v>
-      </c>
-      <c r="D195" t="s">
         <v>351</v>
-      </c>
-      <c r="E195" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="F195" t="s">
-        <v>78</v>
-      </c>
-      <c r="G195" t="s">
-        <v>79</v>
-      </c>
-      <c r="N195" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="196" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A196" t="s">
-        <v>353</v>
-      </c>
-      <c r="B196" t="s">
-        <v>81</v>
-      </c>
-      <c r="C196" t="s">
-        <v>347</v>
-      </c>
-      <c r="D196" t="s">
-        <v>354</v>
-      </c>
-      <c r="E196" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="F196" t="s">
-        <v>78</v>
-      </c>
-      <c r="G196" t="s">
-        <v>79</v>
-      </c>
-      <c r="N196" t="s">
-        <v>355</v>
       </c>
     </row>
   </sheetData>
@@ -7984,10 +7903,10 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:N29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="4" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.54296875" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" style="9" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="13.54296875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.54296875" style="6" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.54296875" bestFit="1" customWidth="1"/>
@@ -8010,7 +7929,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -8054,7 +7973,7 @@
       <c r="D2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="8">
         <v>2020</v>
       </c>
       <c r="F2" t="s">
@@ -8092,7 +8011,7 @@
       <c r="D3" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="8">
         <v>2020</v>
       </c>
       <c r="F3" t="s">
@@ -8130,7 +8049,7 @@
       <c r="D4" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="8">
         <v>2020</v>
       </c>
       <c r="F4" t="s">
@@ -8168,7 +8087,7 @@
       <c r="D5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="8">
         <v>2020</v>
       </c>
       <c r="F5" t="s">
@@ -8206,7 +8125,7 @@
       <c r="D6" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="8">
         <v>2020</v>
       </c>
       <c r="F6" t="s">
@@ -8244,7 +8163,7 @@
       <c r="D7" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="8">
         <v>2020</v>
       </c>
       <c r="F7" t="s">
@@ -8282,7 +8201,7 @@
       <c r="D8" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="8">
         <v>2020</v>
       </c>
       <c r="F8" t="s">
@@ -8320,7 +8239,7 @@
       <c r="D9" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="8">
         <v>2020</v>
       </c>
       <c r="F9" t="s">
@@ -8347,7 +8266,7 @@
     </row>
     <row r="10" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="B10" t="s">
         <v>15</v>
@@ -8358,7 +8277,7 @@
       <c r="D10" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="8">
         <v>2020</v>
       </c>
       <c r="F10" t="s">
@@ -8396,7 +8315,7 @@
       <c r="D11" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="8">
         <v>2020</v>
       </c>
       <c r="F11" t="s">
@@ -8434,7 +8353,7 @@
       <c r="D12" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="8">
         <v>2020</v>
       </c>
       <c r="F12" t="s">
@@ -8472,7 +8391,7 @@
       <c r="D13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="8">
         <v>2020</v>
       </c>
       <c r="F13" t="s">
@@ -8510,7 +8429,7 @@
       <c r="D14" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="8">
         <v>2020</v>
       </c>
       <c r="F14" t="s">
@@ -8548,7 +8467,7 @@
       <c r="D15" t="s">
         <v>45</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>46</v>
       </c>
       <c r="F15" t="s">
@@ -8586,7 +8505,7 @@
       <c r="D16" t="s">
         <v>49</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="9" t="s">
         <v>50</v>
       </c>
       <c r="F16" t="s">
@@ -8624,7 +8543,7 @@
       <c r="D17" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F17" t="s">
@@ -8662,7 +8581,7 @@
       <c r="D18" t="s">
         <v>49</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" s="9" t="s">
         <v>53</v>
       </c>
       <c r="F18" t="s">
@@ -8700,7 +8619,7 @@
       <c r="D19" t="s">
         <v>57</v>
       </c>
-      <c r="E19" s="9">
+      <c r="E19" s="8">
         <v>2020</v>
       </c>
       <c r="F19" t="s">
@@ -8738,7 +8657,7 @@
       <c r="D20" t="s">
         <v>59</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="8">
         <v>2020</v>
       </c>
       <c r="F20" t="s">
@@ -8776,7 +8695,7 @@
       <c r="D21" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="9">
+      <c r="E21" s="8">
         <v>2020</v>
       </c>
       <c r="F21" t="s">
@@ -8814,7 +8733,7 @@
       <c r="D22" t="s">
         <v>57</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="8">
         <v>2020</v>
       </c>
       <c r="F22" t="s">
@@ -8852,7 +8771,7 @@
       <c r="D23" t="s">
         <v>64</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="8">
         <v>2020</v>
       </c>
       <c r="F23" t="s">
@@ -8890,7 +8809,7 @@
       <c r="D24" t="s">
         <v>66</v>
       </c>
-      <c r="E24" s="9">
+      <c r="E24" s="8">
         <v>2020</v>
       </c>
       <c r="F24" t="s">
@@ -8928,7 +8847,7 @@
       <c r="D25" t="s">
         <v>64</v>
       </c>
-      <c r="E25" s="9">
+      <c r="E25" s="8">
         <v>2020</v>
       </c>
       <c r="F25" t="s">
@@ -8966,7 +8885,7 @@
       <c r="D26" t="s">
         <v>69</v>
       </c>
-      <c r="E26" s="9">
+      <c r="E26" s="8">
         <v>2020</v>
       </c>
       <c r="F26" t="s">
@@ -9004,7 +8923,7 @@
       <c r="D27" t="s">
         <v>69</v>
       </c>
-      <c r="E27" s="9">
+      <c r="E27" s="8">
         <v>2020</v>
       </c>
       <c r="F27" t="s">
@@ -9042,7 +8961,7 @@
       <c r="D28" t="s">
         <v>69</v>
       </c>
-      <c r="E28" s="9">
+      <c r="E28" s="8">
         <v>2020</v>
       </c>
       <c r="F28" t="s">
@@ -9080,7 +8999,7 @@
       <c r="D29" t="s">
         <v>73</v>
       </c>
-      <c r="E29" s="9">
+      <c r="E29" s="8">
         <v>2020</v>
       </c>
       <c r="F29" t="s">

</xml_diff>

<commit_message>
updated risk metrics to not use ESA and GFC (GLAD) treeecover for 2020. Removal rational due to high commission errors for indicator 1 when comparing to 21,752 reference points from JRC (as used in testing the EUFO 2020 map)
</commit_message>
<xml_diff>
--- a/whisp_columns.xlsx
+++ b/whisp_columns.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1478" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1480" uniqueCount="357">
   <si>
     <t>Column name</t>
   </si>
@@ -378,6 +378,9 @@
   </si>
   <si>
     <t>Hansen 2013</t>
+  </si>
+  <si>
+    <t>Removed from standard risk metrics due to commission errors</t>
   </si>
   <si>
     <t>Forest_FDaP</t>
@@ -1192,9 +1195,6 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
@@ -1204,11 +1204,14 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -1518,20 +1521,20 @@
   <dimension ref="A1:N194"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="34.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="9" width="15.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="31.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="33.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="8" width="34.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="8" width="15.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="31.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="33.43357142857143" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="14" width="12.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="9" width="24.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="9" width="14.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="8" width="24.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="8" width="14.43357142857143" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="14" width="18.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="9" width="18.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="8" width="18.576428571428572" customWidth="1" bestFit="1"/>
     <col min="10" max="10" style="14" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="9" width="18.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="8" width="18.14785714285714" customWidth="1" bestFit="1"/>
     <col min="12" max="12" style="14" width="17.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="9" width="19.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="9" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="8" width="19.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="8" width="20.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -1591,7 +1594,7 @@
       <c r="D2" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F2" s="3" t="s">
@@ -1600,19 +1603,19 @@
       <c r="G2" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="L2" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M2" s="3" t="s">
@@ -1620,7 +1623,7 @@
       </c>
       <c r="N2" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="3" t="s">
         <v>81</v>
       </c>
@@ -1633,7 +1636,7 @@
       <c r="D3" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F3" s="3" t="s">
@@ -1642,19 +1645,19 @@
       <c r="G3" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="J3" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L3" s="13" t="s">
+      <c r="L3" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M3" s="3" t="s">
@@ -1664,7 +1667,7 @@
         <v>84</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="3" t="s">
         <v>85</v>
       </c>
@@ -1677,7 +1680,7 @@
       <c r="D4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -1686,19 +1689,19 @@
       <c r="G4" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="J4" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L4" s="13" t="s">
+      <c r="L4" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M4" s="3" t="s">
@@ -1706,7 +1709,7 @@
       </c>
       <c r="N4" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="3" t="s">
         <v>88</v>
       </c>
@@ -1719,7 +1722,7 @@
       <c r="D5" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F5" s="3" t="s">
@@ -1728,19 +1731,19 @@
       <c r="G5" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="J5" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="L5" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M5" s="3" t="s">
@@ -1748,7 +1751,7 @@
       </c>
       <c r="N5" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="3" t="s">
         <v>90</v>
       </c>
@@ -1761,7 +1764,7 @@
       <c r="D6" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F6" s="3" t="s">
@@ -1770,19 +1773,19 @@
       <c r="G6" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J6" s="13" t="s">
+      <c r="J6" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L6" s="13" t="s">
+      <c r="L6" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M6" s="3" t="s">
@@ -1790,7 +1793,7 @@
       </c>
       <c r="N6" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="3" t="s">
         <v>93</v>
       </c>
@@ -1803,7 +1806,7 @@
       <c r="D7" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F7" s="3" t="s">
@@ -1812,19 +1815,19 @@
       <c r="G7" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H7" s="13" t="s">
+      <c r="H7" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="J7" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L7" s="13" t="s">
+      <c r="L7" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M7" s="3" t="s">
@@ -1832,7 +1835,7 @@
       </c>
       <c r="N7" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="3" t="s">
         <v>95</v>
       </c>
@@ -1845,7 +1848,7 @@
       <c r="D8" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F8" s="3" t="s">
@@ -1854,19 +1857,19 @@
       <c r="G8" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J8" s="13" t="s">
+      <c r="J8" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L8" s="13" t="s">
+      <c r="L8" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M8" s="3" t="s">
@@ -1874,7 +1877,7 @@
       </c>
       <c r="N8" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="3" t="s">
         <v>97</v>
       </c>
@@ -1887,7 +1890,7 @@
       <c r="D9" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F9" s="3" t="s">
@@ -1896,19 +1899,19 @@
       <c r="G9" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="J9" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="L9" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M9" s="3" t="s">
@@ -1918,7 +1921,7 @@
         <v>100</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="3" t="s">
         <v>101</v>
       </c>
@@ -1931,7 +1934,7 @@
       <c r="D10" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F10" s="3" t="s">
@@ -1940,19 +1943,19 @@
       <c r="G10" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J10" s="13" t="s">
+      <c r="J10" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L10" s="13" t="s">
+      <c r="L10" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M10" s="3" t="s">
@@ -1962,7 +1965,7 @@
         <v>100</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="3" t="s">
         <v>103</v>
       </c>
@@ -1975,7 +1978,7 @@
       <c r="D11" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F11" s="3" t="s">
@@ -1984,19 +1987,19 @@
       <c r="G11" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J11" s="13" t="s">
+      <c r="J11" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L11" s="13" t="s">
+      <c r="L11" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M11" s="3" t="s">
@@ -2004,7 +2007,7 @@
       </c>
       <c r="N11" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="3" t="s">
         <v>106</v>
       </c>
@@ -2026,19 +2029,19 @@
       <c r="G12" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="12" t="s">
         <v>77</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="J12" s="13" t="s">
+      <c r="J12" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L12" s="13" t="s">
+      <c r="L12" s="12" t="s">
         <v>77</v>
       </c>
       <c r="M12" s="3" t="s">
@@ -2046,7 +2049,7 @@
       </c>
       <c r="N12" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="3" t="s">
         <v>111</v>
       </c>
@@ -2088,7 +2091,7 @@
       </c>
       <c r="N13" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="3" t="s">
         <v>113</v>
       </c>
@@ -2132,7 +2135,7 @@
         <v>115</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="3" t="s">
         <v>116</v>
       </c>
@@ -2197,28 +2200,30 @@
         <v>80</v>
       </c>
       <c r="H16" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J16" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L16" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="N16" s="3"/>
+      <c r="N16" s="3" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>15</v>
@@ -2227,13 +2232,13 @@
         <v>16</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E17" s="4">
         <v>2020</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>80</v>
@@ -2260,7 +2265,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>15</v>
@@ -2275,34 +2280,36 @@
         <v>2020</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>80</v>
       </c>
       <c r="H18" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18" s="6" t="s">
         <v>25</v>
       </c>
       <c r="J18" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" s="6" t="s">
         <v>25</v>
       </c>
       <c r="L18" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="N18" s="3"/>
+      <c r="N18" s="3" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>15</v>
@@ -2344,7 +2351,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>15</v>
@@ -2359,7 +2366,7 @@
         <v>2020</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>80</v>
@@ -2386,7 +2393,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>15</v>
@@ -2401,7 +2408,7 @@
         <v>2020</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>80</v>
@@ -2428,7 +2435,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>15</v>
@@ -2443,7 +2450,7 @@
         <v>2020</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>80</v>
@@ -2470,7 +2477,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>15</v>
@@ -2485,7 +2492,7 @@
         <v>2020</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>80</v>
@@ -2512,7 +2519,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>15</v>
@@ -2527,7 +2534,7 @@
         <v>2020</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>80</v>
@@ -2554,7 +2561,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
       <c r="A25" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>15</v>
@@ -2563,13 +2570,13 @@
         <v>16</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E25" s="4">
         <v>2020</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>80</v>
@@ -2596,22 +2603,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>136</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>135</v>
       </c>
       <c r="E26" s="4">
         <v>2020</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>80</v>
@@ -2638,7 +2645,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
       <c r="A27" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>15</v>
@@ -2653,7 +2660,7 @@
         <v>2020</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>80</v>
@@ -2680,7 +2687,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
       <c r="A28" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>15</v>
@@ -2714,7 +2721,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
       <c r="A29" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>15</v>
@@ -2748,7 +2755,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
       <c r="A30" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>15</v>
@@ -2782,7 +2789,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
       <c r="A31" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>15</v>
@@ -2816,7 +2823,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
       <c r="A32" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>15</v>
@@ -2850,7 +2857,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
       <c r="A33" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>15</v>
@@ -2884,7 +2891,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>15</v>
@@ -2918,7 +2925,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>15</v>
@@ -2952,7 +2959,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>15</v>
@@ -2986,7 +2993,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>15</v>
@@ -3020,7 +3027,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>15</v>
@@ -3054,7 +3061,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
       <c r="A39" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>15</v>
@@ -3088,7 +3095,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>15</v>
@@ -3122,7 +3129,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
       <c r="A41" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>15</v>
@@ -3156,7 +3163,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
       <c r="A42" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>15</v>
@@ -3190,7 +3197,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
       <c r="A43" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>15</v>
@@ -3224,7 +3231,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
       <c r="A44" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>15</v>
@@ -3258,7 +3265,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
       <c r="A45" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>15</v>
@@ -3292,7 +3299,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
       <c r="A46" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>15</v>
@@ -3326,7 +3333,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
       <c r="A47" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>15</v>
@@ -3360,7 +3367,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
       <c r="A48" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>15</v>
@@ -3394,7 +3401,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
       <c r="A49" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>15</v>
@@ -3428,7 +3435,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
       <c r="A50" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>15</v>
@@ -3462,7 +3469,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
       <c r="A51" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>15</v>
@@ -3496,7 +3503,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
       <c r="A52" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>15</v>
@@ -3530,7 +3537,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
       <c r="A53" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>15</v>
@@ -3564,7 +3571,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
       <c r="A54" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>15</v>
@@ -3598,7 +3605,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
       <c r="A55" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>15</v>
@@ -3632,7 +3639,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
       <c r="A56" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>15</v>
@@ -3666,7 +3673,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
       <c r="A57" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>15</v>
@@ -3700,7 +3707,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
       <c r="A58" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>15</v>
@@ -3734,7 +3741,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
       <c r="A59" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>15</v>
@@ -3768,7 +3775,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
       <c r="A60" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>15</v>
@@ -3802,7 +3809,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
       <c r="A61" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>15</v>
@@ -3836,7 +3843,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
       <c r="A62" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>15</v>
@@ -3870,7 +3877,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
       <c r="A63" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>15</v>
@@ -3904,7 +3911,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
       <c r="A64" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>15</v>
@@ -3938,7 +3945,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
       <c r="A65" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>15</v>
@@ -3972,7 +3979,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
       <c r="A66" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>15</v>
@@ -4006,7 +4013,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
       <c r="A67" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>15</v>
@@ -4040,7 +4047,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
       <c r="A68" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>15</v>
@@ -4074,7 +4081,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
       <c r="A69" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>15</v>
@@ -4108,7 +4115,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
       <c r="A70" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>15</v>
@@ -4142,7 +4149,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
       <c r="A71" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>15</v>
@@ -4176,7 +4183,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
       <c r="A72" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>15</v>
@@ -4210,7 +4217,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
       <c r="A73" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>15</v>
@@ -4244,7 +4251,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
       <c r="A74" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>15</v>
@@ -4278,7 +4285,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
       <c r="A75" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>15</v>
@@ -4312,7 +4319,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
       <c r="A76" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>15</v>
@@ -4346,7 +4353,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
       <c r="A77" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>15</v>
@@ -4380,7 +4387,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
       <c r="A78" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>15</v>
@@ -4389,7 +4396,7 @@
         <v>16</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E78" s="4">
         <v>2001</v>
@@ -4414,16 +4421,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
       <c r="A79" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D79" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C79" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D79" s="3" t="s">
-        <v>191</v>
       </c>
       <c r="E79" s="4">
         <v>2002</v>
@@ -4448,7 +4455,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
       <c r="A80" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>15</v>
@@ -4457,7 +4464,7 @@
         <v>16</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E80" s="4">
         <v>2003</v>
@@ -4482,7 +4489,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
       <c r="A81" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>15</v>
@@ -4491,7 +4498,7 @@
         <v>16</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E81" s="4">
         <v>2004</v>
@@ -4516,7 +4523,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
       <c r="A82" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B82" s="3" t="s">
         <v>15</v>
@@ -4525,7 +4532,7 @@
         <v>16</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E82" s="4">
         <v>2005</v>
@@ -4550,7 +4557,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
       <c r="A83" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B83" s="3" t="s">
         <v>15</v>
@@ -4559,7 +4566,7 @@
         <v>16</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E83" s="4">
         <v>2006</v>
@@ -4584,7 +4591,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
       <c r="A84" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B84" s="3" t="s">
         <v>15</v>
@@ -4593,7 +4600,7 @@
         <v>16</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E84" s="4">
         <v>2007</v>
@@ -4618,7 +4625,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
       <c r="A85" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B85" s="3" t="s">
         <v>15</v>
@@ -4627,7 +4634,7 @@
         <v>16</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E85" s="4">
         <v>2008</v>
@@ -4652,7 +4659,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
       <c r="A86" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B86" s="3" t="s">
         <v>15</v>
@@ -4661,7 +4668,7 @@
         <v>16</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E86" s="4">
         <v>2009</v>
@@ -4686,7 +4693,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
       <c r="A87" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>15</v>
@@ -4695,7 +4702,7 @@
         <v>16</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E87" s="4">
         <v>2010</v>
@@ -4720,7 +4727,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
       <c r="A88" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B88" s="3" t="s">
         <v>15</v>
@@ -4729,7 +4736,7 @@
         <v>16</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E88" s="4">
         <v>2011</v>
@@ -4754,7 +4761,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
       <c r="A89" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B89" s="3" t="s">
         <v>15</v>
@@ -4763,7 +4770,7 @@
         <v>16</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E89" s="4">
         <v>2012</v>
@@ -4788,7 +4795,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
       <c r="A90" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B90" s="3" t="s">
         <v>15</v>
@@ -4797,7 +4804,7 @@
         <v>16</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E90" s="4">
         <v>2013</v>
@@ -4822,7 +4829,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
       <c r="A91" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B91" s="3" t="s">
         <v>15</v>
@@ -4831,7 +4838,7 @@
         <v>16</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E91" s="4">
         <v>2014</v>
@@ -4856,7 +4863,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
       <c r="A92" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B92" s="3" t="s">
         <v>15</v>
@@ -4865,7 +4872,7 @@
         <v>16</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E92" s="4">
         <v>2015</v>
@@ -4890,7 +4897,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
       <c r="A93" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B93" s="3" t="s">
         <v>15</v>
@@ -4899,7 +4906,7 @@
         <v>16</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E93" s="4">
         <v>2016</v>
@@ -4924,7 +4931,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
       <c r="A94" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B94" s="3" t="s">
         <v>15</v>
@@ -4933,7 +4940,7 @@
         <v>16</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E94" s="4">
         <v>2017</v>
@@ -4958,7 +4965,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
       <c r="A95" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B95" s="3" t="s">
         <v>15</v>
@@ -4967,7 +4974,7 @@
         <v>16</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E95" s="4">
         <v>2018</v>
@@ -4992,7 +4999,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
       <c r="A96" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B96" s="3" t="s">
         <v>15</v>
@@ -5001,7 +5008,7 @@
         <v>16</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E96" s="4">
         <v>2019</v>
@@ -5026,7 +5033,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
       <c r="A97" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B97" s="3" t="s">
         <v>15</v>
@@ -5035,7 +5042,7 @@
         <v>16</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E97" s="4">
         <v>2020</v>
@@ -5060,7 +5067,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
       <c r="A98" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B98" s="3" t="s">
         <v>15</v>
@@ -5069,7 +5076,7 @@
         <v>16</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E98" s="4">
         <v>2021</v>
@@ -5094,7 +5101,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
       <c r="A99" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B99" s="3" t="s">
         <v>15</v>
@@ -5103,7 +5110,7 @@
         <v>16</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E99" s="4">
         <v>2022</v>
@@ -5128,7 +5135,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
       <c r="A100" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B100" s="3" t="s">
         <v>15</v>
@@ -5137,7 +5144,7 @@
         <v>16</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E100" s="4">
         <v>2023</v>
@@ -5162,7 +5169,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
       <c r="A101" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B101" s="3" t="s">
         <v>15</v>
@@ -5171,7 +5178,7 @@
         <v>16</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E101" s="4">
         <v>2024</v>
@@ -5196,7 +5203,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
       <c r="A102" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B102" s="3" t="s">
         <v>15</v>
@@ -5205,13 +5212,13 @@
         <v>16</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E102" s="4">
         <v>2019</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G102" s="3"/>
       <c r="H102" s="5">
@@ -5230,7 +5237,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
       <c r="A103" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B103" s="3" t="s">
         <v>15</v>
@@ -5239,13 +5246,13 @@
         <v>16</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E103" s="4">
         <v>2020</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G103" s="3"/>
       <c r="H103" s="5">
@@ -5264,7 +5271,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
       <c r="A104" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B104" s="3" t="s">
         <v>15</v>
@@ -5273,13 +5280,13 @@
         <v>16</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E104" s="4">
         <v>2021</v>
       </c>
       <c r="F104" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G104" s="3"/>
       <c r="H104" s="5">
@@ -5298,7 +5305,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
       <c r="A105" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B105" s="3" t="s">
         <v>15</v>
@@ -5307,13 +5314,13 @@
         <v>16</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E105" s="4">
         <v>2022</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G105" s="3"/>
       <c r="H105" s="5">
@@ -5332,7 +5339,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
       <c r="A106" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>15</v>
@@ -5341,13 +5348,13 @@
         <v>16</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E106" s="4">
         <v>2023</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G106" s="3"/>
       <c r="H106" s="5">
@@ -5366,7 +5373,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
       <c r="A107" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B107" s="3" t="s">
         <v>15</v>
@@ -5375,13 +5382,13 @@
         <v>16</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E107" s="4">
         <v>2024</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G107" s="3"/>
       <c r="H107" s="5">
@@ -5400,7 +5407,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
       <c r="A108" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B108" s="3" t="s">
         <v>15</v>
@@ -5409,13 +5416,13 @@
         <v>16</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E108" s="4">
         <v>2025</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G108" s="3"/>
       <c r="H108" s="5">
@@ -5434,7 +5441,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
       <c r="A109" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B109" s="3" t="s">
         <v>15</v>
@@ -5443,13 +5450,13 @@
         <v>16</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E109" s="4">
         <v>2001</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G109" s="3"/>
       <c r="H109" s="5">
@@ -5468,7 +5475,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
       <c r="A110" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B110" s="3" t="s">
         <v>15</v>
@@ -5477,13 +5484,13 @@
         <v>16</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E110" s="4">
         <v>2002</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G110" s="3"/>
       <c r="H110" s="5">
@@ -5502,7 +5509,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
       <c r="A111" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B111" s="3" t="s">
         <v>15</v>
@@ -5511,13 +5518,13 @@
         <v>16</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E111" s="4">
         <v>2003</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G111" s="3"/>
       <c r="H111" s="5">
@@ -5536,7 +5543,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
       <c r="A112" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B112" s="3" t="s">
         <v>15</v>
@@ -5545,13 +5552,13 @@
         <v>16</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E112" s="4">
         <v>2004</v>
       </c>
       <c r="F112" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G112" s="3"/>
       <c r="H112" s="5">
@@ -5570,7 +5577,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
       <c r="A113" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B113" s="3" t="s">
         <v>15</v>
@@ -5579,13 +5586,13 @@
         <v>16</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E113" s="4">
         <v>2005</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G113" s="3"/>
       <c r="H113" s="5">
@@ -5604,7 +5611,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
       <c r="A114" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B114" s="3" t="s">
         <v>15</v>
@@ -5613,13 +5620,13 @@
         <v>16</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E114" s="4">
         <v>2006</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G114" s="3"/>
       <c r="H114" s="5">
@@ -5638,7 +5645,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
       <c r="A115" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B115" s="3" t="s">
         <v>15</v>
@@ -5647,13 +5654,13 @@
         <v>16</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E115" s="4">
         <v>2007</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G115" s="3"/>
       <c r="H115" s="5">
@@ -5672,7 +5679,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
       <c r="A116" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B116" s="3" t="s">
         <v>15</v>
@@ -5681,13 +5688,13 @@
         <v>16</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E116" s="4">
         <v>2008</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G116" s="3"/>
       <c r="H116" s="5">
@@ -5706,7 +5713,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
       <c r="A117" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B117" s="3" t="s">
         <v>15</v>
@@ -5715,13 +5722,13 @@
         <v>16</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E117" s="4">
         <v>2009</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G117" s="3"/>
       <c r="H117" s="5">
@@ -5740,7 +5747,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
       <c r="A118" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B118" s="3" t="s">
         <v>15</v>
@@ -5749,13 +5756,13 @@
         <v>16</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E118" s="4">
         <v>2010</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G118" s="3"/>
       <c r="H118" s="5">
@@ -5774,7 +5781,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
       <c r="A119" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B119" s="3" t="s">
         <v>15</v>
@@ -5783,13 +5790,13 @@
         <v>16</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E119" s="4">
         <v>2011</v>
       </c>
       <c r="F119" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G119" s="3"/>
       <c r="H119" s="5">
@@ -5808,7 +5815,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
       <c r="A120" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B120" s="3" t="s">
         <v>15</v>
@@ -5817,13 +5824,13 @@
         <v>16</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E120" s="4">
         <v>2012</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G120" s="3"/>
       <c r="H120" s="5">
@@ -5842,7 +5849,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
       <c r="A121" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B121" s="3" t="s">
         <v>15</v>
@@ -5851,13 +5858,13 @@
         <v>16</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E121" s="4">
         <v>2013</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G121" s="3"/>
       <c r="H121" s="5">
@@ -5876,7 +5883,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
       <c r="A122" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B122" s="3" t="s">
         <v>15</v>
@@ -5885,13 +5892,13 @@
         <v>16</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E122" s="4">
         <v>2014</v>
       </c>
       <c r="F122" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G122" s="3"/>
       <c r="H122" s="5">
@@ -5910,7 +5917,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
       <c r="A123" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B123" s="3" t="s">
         <v>15</v>
@@ -5919,13 +5926,13 @@
         <v>16</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E123" s="4">
         <v>2015</v>
       </c>
       <c r="F123" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G123" s="3"/>
       <c r="H123" s="5">
@@ -5944,7 +5951,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
       <c r="A124" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B124" s="3" t="s">
         <v>15</v>
@@ -5953,13 +5960,13 @@
         <v>16</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E124" s="4">
         <v>2016</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G124" s="3"/>
       <c r="H124" s="5">
@@ -5978,7 +5985,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
       <c r="A125" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B125" s="3" t="s">
         <v>15</v>
@@ -5987,13 +5994,13 @@
         <v>16</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E125" s="4">
         <v>2017</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G125" s="3"/>
       <c r="H125" s="5">
@@ -6012,7 +6019,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
       <c r="A126" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B126" s="3" t="s">
         <v>15</v>
@@ -6021,13 +6028,13 @@
         <v>16</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E126" s="4">
         <v>2018</v>
       </c>
       <c r="F126" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G126" s="3"/>
       <c r="H126" s="5">
@@ -6046,7 +6053,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
       <c r="A127" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B127" s="3" t="s">
         <v>15</v>
@@ -6055,13 +6062,13 @@
         <v>16</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E127" s="4">
         <v>2019</v>
       </c>
       <c r="F127" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G127" s="3"/>
       <c r="H127" s="5">
@@ -6080,7 +6087,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
       <c r="A128" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B128" s="3" t="s">
         <v>15</v>
@@ -6089,13 +6096,13 @@
         <v>16</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E128" s="4">
         <v>2020</v>
       </c>
       <c r="F128" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G128" s="3"/>
       <c r="H128" s="5">
@@ -6114,7 +6121,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
       <c r="A129" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B129" s="3" t="s">
         <v>15</v>
@@ -6123,13 +6130,13 @@
         <v>16</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E129" s="4">
         <v>2000</v>
       </c>
       <c r="F129" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G129" s="3"/>
       <c r="H129" s="5">
@@ -6148,7 +6155,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
       <c r="A130" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B130" s="3" t="s">
         <v>15</v>
@@ -6157,13 +6164,13 @@
         <v>16</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E130" s="4">
         <v>2001</v>
       </c>
       <c r="F130" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G130" s="3"/>
       <c r="H130" s="5">
@@ -6182,7 +6189,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
       <c r="A131" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B131" s="3" t="s">
         <v>15</v>
@@ -6191,13 +6198,13 @@
         <v>16</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E131" s="4">
         <v>2002</v>
       </c>
       <c r="F131" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G131" s="3"/>
       <c r="H131" s="5">
@@ -6216,7 +6223,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
       <c r="A132" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B132" s="3" t="s">
         <v>15</v>
@@ -6225,13 +6232,13 @@
         <v>16</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E132" s="4">
         <v>2003</v>
       </c>
       <c r="F132" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G132" s="3"/>
       <c r="H132" s="5">
@@ -6250,7 +6257,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18.75">
       <c r="A133" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B133" s="3" t="s">
         <v>15</v>
@@ -6259,13 +6266,13 @@
         <v>16</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E133" s="4">
         <v>2004</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G133" s="3"/>
       <c r="H133" s="5">
@@ -6284,7 +6291,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
       <c r="A134" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B134" s="3" t="s">
         <v>15</v>
@@ -6293,13 +6300,13 @@
         <v>16</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E134" s="4">
         <v>2005</v>
       </c>
       <c r="F134" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G134" s="3"/>
       <c r="H134" s="5">
@@ -6318,7 +6325,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
       <c r="A135" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B135" s="3" t="s">
         <v>15</v>
@@ -6327,13 +6334,13 @@
         <v>16</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E135" s="4">
         <v>2006</v>
       </c>
       <c r="F135" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G135" s="3"/>
       <c r="H135" s="5">
@@ -6352,7 +6359,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
       <c r="A136" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B136" s="3" t="s">
         <v>15</v>
@@ -6361,13 +6368,13 @@
         <v>16</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E136" s="4">
         <v>2007</v>
       </c>
       <c r="F136" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G136" s="3"/>
       <c r="H136" s="5">
@@ -6386,7 +6393,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
       <c r="A137" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B137" s="3" t="s">
         <v>15</v>
@@ -6395,13 +6402,13 @@
         <v>16</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E137" s="4">
         <v>2008</v>
       </c>
       <c r="F137" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G137" s="3"/>
       <c r="H137" s="5">
@@ -6420,7 +6427,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
       <c r="A138" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B138" s="3" t="s">
         <v>15</v>
@@ -6429,13 +6436,13 @@
         <v>16</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E138" s="4">
         <v>2009</v>
       </c>
       <c r="F138" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G138" s="3"/>
       <c r="H138" s="5">
@@ -6454,7 +6461,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
       <c r="A139" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B139" s="3" t="s">
         <v>15</v>
@@ -6463,13 +6470,13 @@
         <v>16</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E139" s="4">
         <v>2010</v>
       </c>
       <c r="F139" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G139" s="3"/>
       <c r="H139" s="5">
@@ -6488,7 +6495,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
       <c r="A140" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B140" s="3" t="s">
         <v>15</v>
@@ -6497,13 +6504,13 @@
         <v>16</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E140" s="4">
         <v>2011</v>
       </c>
       <c r="F140" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G140" s="3"/>
       <c r="H140" s="5">
@@ -6522,7 +6529,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
       <c r="A141" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B141" s="3" t="s">
         <v>15</v>
@@ -6531,13 +6538,13 @@
         <v>16</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E141" s="4">
         <v>2012</v>
       </c>
       <c r="F141" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G141" s="3"/>
       <c r="H141" s="5">
@@ -6556,7 +6563,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
       <c r="A142" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B142" s="3" t="s">
         <v>15</v>
@@ -6565,13 +6572,13 @@
         <v>16</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E142" s="4">
         <v>2013</v>
       </c>
       <c r="F142" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G142" s="3"/>
       <c r="H142" s="5">
@@ -6590,7 +6597,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18.75">
       <c r="A143" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B143" s="3" t="s">
         <v>15</v>
@@ -6599,13 +6606,13 @@
         <v>16</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E143" s="4">
         <v>2014</v>
       </c>
       <c r="F143" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G143" s="3"/>
       <c r="H143" s="5">
@@ -6624,7 +6631,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18.75">
       <c r="A144" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B144" s="3" t="s">
         <v>15</v>
@@ -6633,13 +6640,13 @@
         <v>16</v>
       </c>
       <c r="D144" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E144" s="4">
         <v>2015</v>
       </c>
       <c r="F144" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G144" s="3"/>
       <c r="H144" s="5">
@@ -6658,7 +6665,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18.75">
       <c r="A145" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B145" s="3" t="s">
         <v>15</v>
@@ -6667,13 +6674,13 @@
         <v>16</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E145" s="4">
         <v>2016</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G145" s="3"/>
       <c r="H145" s="5">
@@ -6692,7 +6699,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18.75">
       <c r="A146" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B146" s="3" t="s">
         <v>15</v>
@@ -6701,13 +6708,13 @@
         <v>16</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E146" s="4">
         <v>2017</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G146" s="3"/>
       <c r="H146" s="5">
@@ -6726,7 +6733,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18.75">
       <c r="A147" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B147" s="3" t="s">
         <v>15</v>
@@ -6735,13 +6742,13 @@
         <v>16</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E147" s="4">
         <v>2018</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G147" s="3"/>
       <c r="H147" s="5">
@@ -6760,7 +6767,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18.75">
       <c r="A148" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B148" s="3" t="s">
         <v>15</v>
@@ -6769,13 +6776,13 @@
         <v>16</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E148" s="4">
         <v>2019</v>
       </c>
       <c r="F148" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G148" s="3"/>
       <c r="H148" s="5">
@@ -6794,7 +6801,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18.75">
       <c r="A149" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B149" s="3" t="s">
         <v>15</v>
@@ -6803,13 +6810,13 @@
         <v>16</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E149" s="4">
         <v>2020</v>
       </c>
       <c r="F149" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G149" s="3"/>
       <c r="H149" s="5">
@@ -6828,7 +6835,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75">
       <c r="A150" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B150" s="3" t="s">
         <v>15</v>
@@ -6837,13 +6844,13 @@
         <v>16</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E150" s="4">
         <v>2021</v>
       </c>
       <c r="F150" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G150" s="3"/>
       <c r="H150" s="5">
@@ -6862,7 +6869,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75">
       <c r="A151" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B151" s="3" t="s">
         <v>15</v>
@@ -6871,13 +6878,13 @@
         <v>16</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E151" s="4">
         <v>2022</v>
       </c>
       <c r="F151" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G151" s="3"/>
       <c r="H151" s="5">
@@ -6896,7 +6903,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75">
       <c r="A152" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B152" s="3" t="s">
         <v>15</v>
@@ -6905,13 +6912,13 @@
         <v>16</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E152" s="4">
         <v>2023</v>
       </c>
       <c r="F152" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G152" s="3"/>
       <c r="H152" s="5">
@@ -6930,7 +6937,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18.75">
       <c r="A153" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B153" s="3" t="s">
         <v>15</v>
@@ -6939,13 +6946,13 @@
         <v>16</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E153" s="4">
         <v>2024</v>
       </c>
       <c r="F153" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G153" s="3"/>
       <c r="H153" s="5">
@@ -6964,7 +6971,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18.75">
       <c r="A154" s="3" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B154" s="3" t="s">
         <v>15</v>
@@ -6973,13 +6980,13 @@
         <v>16</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E154" s="4">
         <v>2025</v>
       </c>
       <c r="F154" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G154" s="3"/>
       <c r="H154" s="5">
@@ -6998,7 +7005,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75">
       <c r="A155" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B155" s="3" t="s">
         <v>15</v>
@@ -7009,8 +7016,8 @@
       <c r="D155" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E155" s="12" t="s">
-        <v>273</v>
+      <c r="E155" s="11" t="s">
+        <v>274</v>
       </c>
       <c r="F155" s="3" t="s">
         <v>118</v>
@@ -7036,7 +7043,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75">
       <c r="A156" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B156" s="3" t="s">
         <v>15</v>
@@ -7047,8 +7054,8 @@
       <c r="D156" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E156" s="12" t="s">
-        <v>273</v>
+      <c r="E156" s="11" t="s">
+        <v>274</v>
       </c>
       <c r="F156" s="3" t="s">
         <v>118</v>
@@ -7074,7 +7081,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75">
       <c r="A157" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B157" s="3" t="s">
         <v>15</v>
@@ -7083,10 +7090,10 @@
         <v>16</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="E157" s="12" t="s">
-        <v>273</v>
+        <v>192</v>
+      </c>
+      <c r="E157" s="11" t="s">
+        <v>274</v>
       </c>
       <c r="F157" s="3" t="s">
         <v>120</v>
@@ -7112,7 +7119,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
       <c r="A158" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B158" s="3" t="s">
         <v>15</v>
@@ -7121,13 +7128,13 @@
         <v>16</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="E158" s="12" t="s">
-        <v>273</v>
+        <v>278</v>
+      </c>
+      <c r="E158" s="11" t="s">
+        <v>274</v>
       </c>
       <c r="F158" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G158" s="3" t="s">
         <v>80</v>
@@ -7150,22 +7157,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
       <c r="A159" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B159" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C159" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D159" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="B159" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C159" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D159" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="E159" s="12" t="s">
-        <v>273</v>
+      <c r="E159" s="11" t="s">
+        <v>274</v>
       </c>
       <c r="F159" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G159" s="3" t="s">
         <v>80</v>
@@ -7188,7 +7195,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
       <c r="A160" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B160" s="3" t="s">
         <v>15</v>
@@ -7197,13 +7204,13 @@
         <v>16</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="E160" s="12" t="s">
-        <v>280</v>
+        <v>192</v>
+      </c>
+      <c r="E160" s="11" t="s">
+        <v>281</v>
       </c>
       <c r="F160" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G160" s="3" t="s">
         <v>80</v>
@@ -7226,7 +7233,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75">
       <c r="A161" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B161" s="3" t="s">
         <v>15</v>
@@ -7237,8 +7244,8 @@
       <c r="D161" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E161" s="12" t="s">
-        <v>282</v>
+      <c r="E161" s="11" t="s">
+        <v>283</v>
       </c>
       <c r="F161" s="3" t="s">
         <v>118</v>
@@ -7266,7 +7273,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75">
       <c r="A162" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B162" s="3" t="s">
         <v>15</v>
@@ -7277,8 +7284,8 @@
       <c r="D162" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E162" s="12" t="s">
-        <v>282</v>
+      <c r="E162" s="11" t="s">
+        <v>283</v>
       </c>
       <c r="F162" s="3" t="s">
         <v>118</v>
@@ -7306,7 +7313,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75">
       <c r="A163" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B163" s="3" t="s">
         <v>15</v>
@@ -7315,10 +7322,10 @@
         <v>16</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="E163" s="12" t="s">
-        <v>282</v>
+        <v>192</v>
+      </c>
+      <c r="E163" s="11" t="s">
+        <v>283</v>
       </c>
       <c r="F163" s="3" t="s">
         <v>120</v>
@@ -7346,7 +7353,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75">
       <c r="A164" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B164" s="3" t="s">
         <v>15</v>
@@ -7355,13 +7362,13 @@
         <v>16</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="E164" s="12" t="s">
         <v>287</v>
       </c>
+      <c r="E164" s="11" t="s">
+        <v>288</v>
+      </c>
       <c r="F164" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G164" s="3" t="s">
         <v>80</v>
@@ -7386,7 +7393,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75">
       <c r="A165" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B165" s="3" t="s">
         <v>15</v>
@@ -7395,13 +7402,13 @@
         <v>16</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="E165" s="12" t="s">
-        <v>282</v>
+        <v>192</v>
+      </c>
+      <c r="E165" s="11" t="s">
+        <v>283</v>
       </c>
       <c r="F165" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G165" s="3" t="s">
         <v>80</v>
@@ -7426,7 +7433,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
       <c r="A166" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B166" s="3" t="s">
         <v>15</v>
@@ -7464,7 +7471,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
       <c r="A167" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B167" s="3" t="s">
         <v>15</v>
@@ -7473,13 +7480,13 @@
         <v>16</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E167" s="4">
         <v>2020</v>
       </c>
       <c r="F167" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G167" s="3" t="s">
         <v>80</v>
@@ -7502,7 +7509,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75">
       <c r="A168" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B168" s="3" t="s">
         <v>15</v>
@@ -7517,7 +7524,7 @@
         <v>2020</v>
       </c>
       <c r="F168" s="3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G168" s="3" t="s">
         <v>80</v>
@@ -7540,7 +7547,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18.75">
       <c r="A169" s="3" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B169" s="3" t="s">
         <v>15</v>
@@ -7549,7 +7556,7 @@
         <v>16</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E169" s="4">
         <v>2020</v>
@@ -7578,7 +7585,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75">
       <c r="A170" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B170" s="3" t="s">
         <v>15</v>
@@ -7587,7 +7594,7 @@
         <v>16</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E170" s="4">
         <v>2020</v>
@@ -7616,7 +7623,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75">
       <c r="A171" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B171" s="3" t="s">
         <v>15</v>
@@ -7625,13 +7632,13 @@
         <v>16</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E171" s="4">
         <v>2015</v>
       </c>
       <c r="F171" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G171" s="3"/>
       <c r="H171" s="5">
@@ -7649,12 +7656,12 @@
         <v>41</v>
       </c>
       <c r="N171" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18.75">
       <c r="A172" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B172" s="3" t="s">
         <v>15</v>
@@ -7663,7 +7670,7 @@
         <v>16</v>
       </c>
       <c r="D172" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E172" s="4">
         <v>2023</v>
@@ -7686,13 +7693,13 @@
         <v>1</v>
       </c>
       <c r="M172" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="N172" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75">
       <c r="A173" s="3" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B173" s="3" t="s">
         <v>15</v>
@@ -7701,13 +7708,13 @@
         <v>16</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E173" s="4">
         <v>2023</v>
       </c>
       <c r="F173" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G173" s="3"/>
       <c r="H173" s="5">
@@ -7722,13 +7729,13 @@
         <v>1</v>
       </c>
       <c r="M173" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="N173" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75">
       <c r="A174" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B174" s="3" t="s">
         <v>15</v>
@@ -7743,7 +7750,7 @@
         <v>2023</v>
       </c>
       <c r="F174" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G174" s="3" t="s">
         <v>80</v>
@@ -7760,13 +7767,13 @@
         <v>1</v>
       </c>
       <c r="M174" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="N174" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75">
       <c r="A175" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B175" s="3" t="s">
         <v>15</v>
@@ -7775,13 +7782,13 @@
         <v>16</v>
       </c>
       <c r="D175" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E175" s="4">
         <v>2023</v>
       </c>
       <c r="F175" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G175" s="3" t="s">
         <v>80</v>
@@ -7798,13 +7805,13 @@
         <v>1</v>
       </c>
       <c r="M175" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="N175" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75">
       <c r="A176" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B176" s="3" t="s">
         <v>15</v>
@@ -7819,7 +7826,7 @@
         <v>2023</v>
       </c>
       <c r="F176" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G176" s="3" t="s">
         <v>80</v>
@@ -7836,13 +7843,13 @@
         <v>1</v>
       </c>
       <c r="M176" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="N176" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18.75">
       <c r="A177" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B177" s="3" t="s">
         <v>15</v>
@@ -7857,7 +7864,7 @@
         <v>2023</v>
       </c>
       <c r="F177" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G177" s="3" t="s">
         <v>80</v>
@@ -7874,13 +7881,13 @@
         <v>1</v>
       </c>
       <c r="M177" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="N177" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75">
       <c r="A178" s="3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B178" s="3" t="s">
         <v>15</v>
@@ -7889,13 +7896,13 @@
         <v>16</v>
       </c>
       <c r="D178" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E178" s="4" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F178" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G178" s="3" t="s">
         <v>80</v>
@@ -7912,13 +7919,13 @@
         <v>1</v>
       </c>
       <c r="M178" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="N178" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75">
       <c r="A179" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B179" s="3" t="s">
         <v>15</v>
@@ -7927,13 +7934,13 @@
         <v>16</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E179" s="4">
         <v>2015</v>
       </c>
       <c r="F179" s="3" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="G179" s="3" t="s">
         <v>80</v>
@@ -7950,15 +7957,15 @@
         <v>1</v>
       </c>
       <c r="M179" s="6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="N179" s="3" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75">
       <c r="A180" s="3" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>82</v>
@@ -7967,9 +7974,9 @@
         <v>77</v>
       </c>
       <c r="D180" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="E180" s="12" t="s">
+        <v>324</v>
+      </c>
+      <c r="E180" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F180" s="3" t="s">
@@ -7978,11 +7985,11 @@
       <c r="G180" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H180" s="12"/>
+      <c r="H180" s="13"/>
       <c r="I180" s="3"/>
-      <c r="J180" s="12"/>
+      <c r="J180" s="13"/>
       <c r="K180" s="3"/>
-      <c r="L180" s="12"/>
+      <c r="L180" s="13"/>
       <c r="M180" s="3"/>
       <c r="N180" s="3" t="s">
         <v>100</v>
@@ -7990,16 +7997,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75">
       <c r="A181" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B181" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D181" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E181" s="4">
         <v>2020</v>
@@ -8010,28 +8017,28 @@
       <c r="G181" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H181" s="12"/>
+      <c r="H181" s="13"/>
       <c r="I181" s="3"/>
-      <c r="J181" s="12"/>
+      <c r="J181" s="13"/>
       <c r="K181" s="3"/>
-      <c r="L181" s="12"/>
+      <c r="L181" s="13"/>
       <c r="M181" s="3"/>
       <c r="N181" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75">
       <c r="A182" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B182" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D182" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E182" s="4">
         <v>2020</v>
@@ -8042,31 +8049,31 @@
       <c r="G182" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H182" s="12"/>
+      <c r="H182" s="13"/>
       <c r="I182" s="3"/>
-      <c r="J182" s="12"/>
+      <c r="J182" s="13"/>
       <c r="K182" s="3"/>
-      <c r="L182" s="12"/>
+      <c r="L182" s="13"/>
       <c r="M182" s="3"/>
       <c r="N182" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75">
       <c r="A183" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B183" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D183" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="E183" s="12" t="s">
-        <v>273</v>
+        <v>332</v>
+      </c>
+      <c r="E183" s="11" t="s">
+        <v>274</v>
       </c>
       <c r="F183" s="3" t="s">
         <v>79</v>
@@ -8074,31 +8081,31 @@
       <c r="G183" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H183" s="12"/>
+      <c r="H183" s="13"/>
       <c r="I183" s="3"/>
-      <c r="J183" s="12"/>
+      <c r="J183" s="13"/>
       <c r="K183" s="3"/>
-      <c r="L183" s="12"/>
+      <c r="L183" s="13"/>
       <c r="M183" s="3"/>
       <c r="N183" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75">
       <c r="A184" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B184" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D184" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="E184" s="12" t="s">
-        <v>333</v>
+        <v>332</v>
+      </c>
+      <c r="E184" s="11" t="s">
+        <v>334</v>
       </c>
       <c r="F184" s="3" t="s">
         <v>79</v>
@@ -8106,28 +8113,28 @@
       <c r="G184" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H184" s="12"/>
+      <c r="H184" s="13"/>
       <c r="I184" s="3"/>
-      <c r="J184" s="12"/>
+      <c r="J184" s="13"/>
       <c r="K184" s="3"/>
-      <c r="L184" s="12"/>
+      <c r="L184" s="13"/>
       <c r="M184" s="3"/>
       <c r="N184" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75">
       <c r="A185" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B185" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D185" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E185" s="4">
         <v>2020</v>
@@ -8138,28 +8145,28 @@
       <c r="G185" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H185" s="12"/>
+      <c r="H185" s="13"/>
       <c r="I185" s="3"/>
-      <c r="J185" s="12"/>
+      <c r="J185" s="13"/>
       <c r="K185" s="3"/>
-      <c r="L185" s="12"/>
+      <c r="L185" s="13"/>
       <c r="M185" s="3"/>
       <c r="N185" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75">
       <c r="A186" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B186" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D186" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E186" s="4">
         <v>2020</v>
@@ -8170,28 +8177,28 @@
       <c r="G186" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H186" s="12"/>
+      <c r="H186" s="13"/>
       <c r="I186" s="3"/>
-      <c r="J186" s="12"/>
+      <c r="J186" s="13"/>
       <c r="K186" s="3"/>
-      <c r="L186" s="12"/>
+      <c r="L186" s="13"/>
       <c r="M186" s="3"/>
       <c r="N186" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75">
       <c r="A187" s="3" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B187" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D187" s="3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E187" s="4">
         <v>2020</v>
@@ -8202,31 +8209,31 @@
       <c r="G187" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H187" s="12"/>
+      <c r="H187" s="13"/>
       <c r="I187" s="3"/>
-      <c r="J187" s="12"/>
+      <c r="J187" s="13"/>
       <c r="K187" s="3"/>
-      <c r="L187" s="12"/>
+      <c r="L187" s="13"/>
       <c r="M187" s="3"/>
       <c r="N187" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75">
       <c r="A188" s="3" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B188" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D188" s="3" t="s">
-        <v>339</v>
-      </c>
-      <c r="E188" s="12" t="s">
-        <v>333</v>
+        <v>340</v>
+      </c>
+      <c r="E188" s="11" t="s">
+        <v>334</v>
       </c>
       <c r="F188" s="3" t="s">
         <v>79</v>
@@ -8234,31 +8241,31 @@
       <c r="G188" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H188" s="12"/>
+      <c r="H188" s="13"/>
       <c r="I188" s="3"/>
-      <c r="J188" s="12"/>
+      <c r="J188" s="13"/>
       <c r="K188" s="3"/>
-      <c r="L188" s="12"/>
+      <c r="L188" s="13"/>
       <c r="M188" s="3"/>
       <c r="N188" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75">
       <c r="A189" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B189" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D189" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="E189" s="12" t="s">
-        <v>333</v>
+        <v>327</v>
+      </c>
+      <c r="E189" s="11" t="s">
+        <v>334</v>
       </c>
       <c r="F189" s="3" t="s">
         <v>79</v>
@@ -8266,31 +8273,31 @@
       <c r="G189" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H189" s="12"/>
+      <c r="H189" s="13"/>
       <c r="I189" s="3"/>
-      <c r="J189" s="12"/>
+      <c r="J189" s="13"/>
       <c r="K189" s="3"/>
-      <c r="L189" s="12"/>
+      <c r="L189" s="13"/>
       <c r="M189" s="3"/>
       <c r="N189" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
       <c r="A190" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B190" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D190" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="E190" s="12" t="s">
-        <v>333</v>
+        <v>344</v>
+      </c>
+      <c r="E190" s="11" t="s">
+        <v>334</v>
       </c>
       <c r="F190" s="3" t="s">
         <v>79</v>
@@ -8298,28 +8305,28 @@
       <c r="G190" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H190" s="12"/>
+      <c r="H190" s="13"/>
       <c r="I190" s="3"/>
-      <c r="J190" s="12"/>
+      <c r="J190" s="13"/>
       <c r="K190" s="3"/>
-      <c r="L190" s="12"/>
+      <c r="L190" s="13"/>
       <c r="M190" s="3"/>
       <c r="N190" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75">
       <c r="A191" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B191" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D191" s="3" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E191" s="4">
         <v>2015</v>
@@ -8330,30 +8337,30 @@
       <c r="G191" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H191" s="12"/>
+      <c r="H191" s="13"/>
       <c r="I191" s="3"/>
-      <c r="J191" s="12"/>
+      <c r="J191" s="13"/>
       <c r="K191" s="3"/>
-      <c r="L191" s="12"/>
+      <c r="L191" s="13"/>
       <c r="M191" s="3"/>
       <c r="N191" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18.75">
       <c r="A192" s="3" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B192" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D192" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="E192" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="E192" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F192" s="3" t="s">
@@ -8362,30 +8369,30 @@
       <c r="G192" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H192" s="12"/>
+      <c r="H192" s="13"/>
       <c r="I192" s="3"/>
-      <c r="J192" s="12"/>
+      <c r="J192" s="13"/>
       <c r="K192" s="3"/>
-      <c r="L192" s="12"/>
+      <c r="L192" s="13"/>
       <c r="M192" s="3"/>
       <c r="N192" s="3" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75">
       <c r="A193" s="3" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B193" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C193" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D193" s="3" t="s">
-        <v>351</v>
-      </c>
-      <c r="E193" s="12" t="s">
+        <v>352</v>
+      </c>
+      <c r="E193" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F193" s="3" t="s">
@@ -8394,30 +8401,30 @@
       <c r="G193" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H193" s="12"/>
+      <c r="H193" s="13"/>
       <c r="I193" s="3"/>
-      <c r="J193" s="12"/>
+      <c r="J193" s="13"/>
       <c r="K193" s="3"/>
-      <c r="L193" s="12"/>
+      <c r="L193" s="13"/>
       <c r="M193" s="3"/>
       <c r="N193" s="3" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="15">
       <c r="A194" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B194" s="3" t="s">
         <v>82</v>
       </c>
       <c r="C194" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D194" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="E194" s="12" t="s">
+        <v>355</v>
+      </c>
+      <c r="E194" s="11" t="s">
         <v>77</v>
       </c>
       <c r="F194" s="3" t="s">
@@ -8426,14 +8433,14 @@
       <c r="G194" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="H194" s="12"/>
+      <c r="H194" s="13"/>
       <c r="I194" s="3"/>
-      <c r="J194" s="12"/>
+      <c r="J194" s="13"/>
       <c r="K194" s="3"/>
-      <c r="L194" s="12"/>
+      <c r="L194" s="13"/>
       <c r="M194" s="3"/>
       <c r="N194" s="3" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
   </sheetData>
@@ -8449,20 +8456,20 @@
   <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -9042,7 +9049,7 @@
       <c r="D15" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="4" t="s">
         <v>47</v>
       </c>
       <c r="F15" s="3" t="s">
@@ -9082,7 +9089,7 @@
       <c r="D16" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="4" t="s">
         <v>51</v>
       </c>
       <c r="F16" s="3" t="s">
@@ -9122,7 +9129,7 @@
       <c r="D17" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="4" t="s">
         <v>54</v>
       </c>
       <c r="F17" s="3" t="s">
@@ -9162,7 +9169,7 @@
       <c r="D18" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="4" t="s">
         <v>54</v>
       </c>
       <c r="F18" s="3" t="s">

</xml_diff>

<commit_message>
updated doc for dataset
</commit_message>
<xml_diff>
--- a/whisp_columns.xlsx
+++ b/whisp_columns.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnell\Documents\GitHub\whisp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3CC688-2526-4953-8A57-48845E86BC7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73BD1CF-3F80-4868-A3BF-967D1406E478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1494" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1502" uniqueCount="364">
   <si>
     <t>Column name</t>
   </si>
@@ -1104,6 +1104,15 @@
   </si>
   <si>
     <t>Processing info in dictionary format: whisp_version (python package release), processing_timestamp_utc (in ISO 8601 standard and set to UTC)</t>
+  </si>
+  <si>
+    <t>DIST_after_2020</t>
+  </si>
+  <si>
+    <t>2023-2026</t>
+  </si>
+  <si>
+    <t>Pickens 2025</t>
   </si>
 </sst>
 </file>
@@ -1520,7 +1529,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:N195"/>
+  <dimension ref="A1:N196"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.7265625" bestFit="1" customWidth="1"/>
@@ -7012,7 +7021,7 @@
     </row>
     <row r="166" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>292</v>
+        <v>361</v>
       </c>
       <c r="B166" t="s">
         <v>15</v>
@@ -7021,35 +7030,33 @@
         <v>16</v>
       </c>
       <c r="D166" t="s">
-        <v>24</v>
-      </c>
-      <c r="E166" s="3">
-        <v>2020</v>
+        <v>194</v>
+      </c>
+      <c r="E166" s="9" t="s">
+        <v>362</v>
       </c>
       <c r="F166" t="s">
-        <v>114</v>
-      </c>
-      <c r="G166" t="s">
-        <v>82</v>
+        <v>363</v>
       </c>
       <c r="H166" s="4">
-        <v>0</v>
-      </c>
-      <c r="I166" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I166" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="J166" s="4">
-        <v>0</v>
-      </c>
-      <c r="K166" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="K166" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="L166" s="4">
-        <v>1</v>
-      </c>
-      <c r="M166" s="5" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B167" t="s">
         <v>15</v>
@@ -7058,13 +7065,13 @@
         <v>16</v>
       </c>
       <c r="D167" t="s">
-        <v>294</v>
+        <v>24</v>
       </c>
       <c r="E167" s="3">
         <v>2020</v>
       </c>
       <c r="F167" t="s">
-        <v>295</v>
+        <v>114</v>
       </c>
       <c r="G167" t="s">
         <v>82</v>
@@ -7086,7 +7093,7 @@
     </row>
     <row r="168" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B168" t="s">
         <v>15</v>
@@ -7095,13 +7102,13 @@
         <v>16</v>
       </c>
       <c r="D168" t="s">
-        <v>24</v>
+        <v>294</v>
       </c>
       <c r="E168" s="3">
         <v>2020</v>
       </c>
       <c r="F168" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="G168" t="s">
         <v>82</v>
@@ -7123,7 +7130,7 @@
     </row>
     <row r="169" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B169" t="s">
         <v>15</v>
@@ -7132,13 +7139,13 @@
         <v>16</v>
       </c>
       <c r="D169" t="s">
-        <v>299</v>
+        <v>24</v>
       </c>
       <c r="E169" s="3">
         <v>2020</v>
       </c>
       <c r="F169" t="s">
-        <v>114</v>
+        <v>297</v>
       </c>
       <c r="G169" t="s">
         <v>82</v>
@@ -7155,12 +7162,12 @@
         <v>1</v>
       </c>
       <c r="M169" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="170" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B170" t="s">
         <v>15</v>
@@ -7169,7 +7176,7 @@
         <v>16</v>
       </c>
       <c r="D170" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E170" s="3">
         <v>2020</v>
@@ -7192,12 +7199,12 @@
         <v>1</v>
       </c>
       <c r="M170" s="5" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
     </row>
     <row r="171" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B171" t="s">
         <v>15</v>
@@ -7206,13 +7213,16 @@
         <v>16</v>
       </c>
       <c r="D171" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E171" s="3">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="F171" t="s">
-        <v>304</v>
+        <v>114</v>
+      </c>
+      <c r="G171" t="s">
+        <v>82</v>
       </c>
       <c r="H171" s="4">
         <v>0</v>
@@ -7228,13 +7238,10 @@
       <c r="M171" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="N171" t="s">
-        <v>305</v>
-      </c>
     </row>
     <row r="172" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="B172" t="s">
         <v>15</v>
@@ -7243,16 +7250,13 @@
         <v>16</v>
       </c>
       <c r="D172" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="E172" s="3">
-        <v>2023</v>
+        <v>2015</v>
       </c>
       <c r="F172" t="s">
-        <v>120</v>
-      </c>
-      <c r="G172" t="s">
-        <v>82</v>
+        <v>304</v>
       </c>
       <c r="H172" s="4">
         <v>0</v>
@@ -7266,12 +7270,15 @@
         <v>1</v>
       </c>
       <c r="M172" s="5" t="s">
-        <v>308</v>
+        <v>41</v>
+      </c>
+      <c r="N172" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="173" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B173" t="s">
         <v>15</v>
@@ -7280,13 +7287,16 @@
         <v>16</v>
       </c>
       <c r="D173" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E173" s="3">
         <v>2023</v>
       </c>
       <c r="F173" t="s">
-        <v>311</v>
+        <v>120</v>
+      </c>
+      <c r="G173" t="s">
+        <v>82</v>
       </c>
       <c r="H173" s="4">
         <v>0</v>
@@ -7305,7 +7315,7 @@
     </row>
     <row r="174" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B174" t="s">
         <v>15</v>
@@ -7314,16 +7324,13 @@
         <v>16</v>
       </c>
       <c r="D174" t="s">
-        <v>62</v>
+        <v>310</v>
       </c>
       <c r="E174" s="3">
         <v>2023</v>
       </c>
       <c r="F174" t="s">
-        <v>126</v>
-      </c>
-      <c r="G174" t="s">
-        <v>82</v>
+        <v>311</v>
       </c>
       <c r="H174" s="4">
         <v>0</v>
@@ -7337,12 +7344,12 @@
         <v>1</v>
       </c>
       <c r="M174" s="5" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
     </row>
     <row r="175" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B175" t="s">
         <v>15</v>
@@ -7351,7 +7358,7 @@
         <v>16</v>
       </c>
       <c r="D175" t="s">
-        <v>138</v>
+        <v>62</v>
       </c>
       <c r="E175" s="3">
         <v>2023</v>
@@ -7379,7 +7386,7 @@
     </row>
     <row r="176" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B176" t="s">
         <v>15</v>
@@ -7388,7 +7395,7 @@
         <v>16</v>
       </c>
       <c r="D176" t="s">
-        <v>60</v>
+        <v>138</v>
       </c>
       <c r="E176" s="3">
         <v>2023</v>
@@ -7416,7 +7423,7 @@
     </row>
     <row r="177" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B177" t="s">
         <v>15</v>
@@ -7425,7 +7432,7 @@
         <v>16</v>
       </c>
       <c r="D177" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="E177" s="3">
         <v>2023</v>
@@ -7453,7 +7460,7 @@
     </row>
     <row r="178" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B178" t="s">
         <v>15</v>
@@ -7462,13 +7469,13 @@
         <v>16</v>
       </c>
       <c r="D178" t="s">
-        <v>318</v>
-      </c>
-      <c r="E178" s="3" t="s">
-        <v>319</v>
+        <v>74</v>
+      </c>
+      <c r="E178" s="3">
+        <v>2023</v>
       </c>
       <c r="F178" t="s">
-        <v>311</v>
+        <v>126</v>
       </c>
       <c r="G178" t="s">
         <v>82</v>
@@ -7490,7 +7497,7 @@
     </row>
     <row r="179" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="B179" t="s">
         <v>15</v>
@@ -7499,13 +7506,13 @@
         <v>16</v>
       </c>
       <c r="D179" t="s">
-        <v>321</v>
-      </c>
-      <c r="E179" s="3">
-        <v>2015</v>
+        <v>318</v>
+      </c>
+      <c r="E179" s="3" t="s">
+        <v>319</v>
       </c>
       <c r="F179" t="s">
-        <v>322</v>
+        <v>311</v>
       </c>
       <c r="G179" t="s">
         <v>82</v>
@@ -7522,44 +7529,52 @@
         <v>1</v>
       </c>
       <c r="M179" s="5" t="s">
-        <v>323</v>
-      </c>
-      <c r="N179" t="s">
-        <v>324</v>
+        <v>313</v>
       </c>
     </row>
     <row r="180" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B180" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C180" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="D180" t="s">
-        <v>326</v>
-      </c>
-      <c r="E180" s="9" t="s">
-        <v>79</v>
+        <v>321</v>
+      </c>
+      <c r="E180" s="3">
+        <v>2015</v>
       </c>
       <c r="F180" t="s">
-        <v>81</v>
+        <v>322</v>
       </c>
       <c r="G180" t="s">
         <v>82</v>
       </c>
-      <c r="H180" s="3"/>
-      <c r="J180" s="3"/>
-      <c r="L180" s="3"/>
+      <c r="H180" s="4">
+        <v>0</v>
+      </c>
+      <c r="I180" s="5"/>
+      <c r="J180" s="4">
+        <v>0</v>
+      </c>
+      <c r="K180" s="5"/>
+      <c r="L180" s="4">
+        <v>1</v>
+      </c>
+      <c r="M180" s="5" t="s">
+        <v>323</v>
+      </c>
       <c r="N180" t="s">
-        <v>102</v>
+        <v>324</v>
       </c>
     </row>
     <row r="181" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>359</v>
+        <v>325</v>
       </c>
       <c r="B181" t="s">
         <v>84</v>
@@ -7568,53 +7583,53 @@
         <v>79</v>
       </c>
       <c r="D181" t="s">
-        <v>360</v>
-      </c>
-      <c r="E181" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="E181" s="9" t="s">
         <v>79</v>
       </c>
       <c r="F181" t="s">
         <v>81</v>
       </c>
-      <c r="H181" s="4"/>
-      <c r="I181" s="5"/>
-      <c r="J181" s="4"/>
-      <c r="K181" s="5"/>
-      <c r="L181" s="4"/>
-      <c r="M181" s="5"/>
+      <c r="G181" t="s">
+        <v>82</v>
+      </c>
+      <c r="H181" s="3"/>
+      <c r="J181" s="3"/>
+      <c r="L181" s="3"/>
+      <c r="N181" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="182" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
-        <v>327</v>
+        <v>359</v>
       </c>
       <c r="B182" t="s">
         <v>84</v>
       </c>
       <c r="C182" t="s">
-        <v>328</v>
+        <v>79</v>
       </c>
       <c r="D182" t="s">
-        <v>329</v>
-      </c>
-      <c r="E182" s="3">
-        <v>2020</v>
+        <v>360</v>
+      </c>
+      <c r="E182" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="F182" t="s">
         <v>81</v>
       </c>
-      <c r="G182" t="s">
-        <v>82</v>
-      </c>
-      <c r="H182" s="3"/>
-      <c r="J182" s="3"/>
-      <c r="L182" s="3"/>
-      <c r="N182" t="s">
-        <v>330</v>
-      </c>
+      <c r="H182" s="4"/>
+      <c r="I182" s="5"/>
+      <c r="J182" s="4"/>
+      <c r="K182" s="5"/>
+      <c r="L182" s="4"/>
+      <c r="M182" s="5"/>
     </row>
     <row r="183" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="B183" t="s">
         <v>84</v>
@@ -7623,7 +7638,7 @@
         <v>328</v>
       </c>
       <c r="D183" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="E183" s="3">
         <v>2020</v>
@@ -7643,7 +7658,7 @@
     </row>
     <row r="184" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B184" t="s">
         <v>84</v>
@@ -7652,10 +7667,10 @@
         <v>328</v>
       </c>
       <c r="D184" t="s">
-        <v>334</v>
-      </c>
-      <c r="E184" s="9" t="s">
-        <v>276</v>
+        <v>332</v>
+      </c>
+      <c r="E184" s="3">
+        <v>2020</v>
       </c>
       <c r="F184" t="s">
         <v>81</v>
@@ -7672,7 +7687,7 @@
     </row>
     <row r="185" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B185" t="s">
         <v>84</v>
@@ -7684,7 +7699,7 @@
         <v>334</v>
       </c>
       <c r="E185" s="9" t="s">
-        <v>336</v>
+        <v>276</v>
       </c>
       <c r="F185" t="s">
         <v>81</v>
@@ -7701,7 +7716,7 @@
     </row>
     <row r="186" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B186" t="s">
         <v>84</v>
@@ -7710,10 +7725,10 @@
         <v>328</v>
       </c>
       <c r="D186" t="s">
-        <v>338</v>
-      </c>
-      <c r="E186" s="3">
-        <v>2020</v>
+        <v>334</v>
+      </c>
+      <c r="E186" s="9" t="s">
+        <v>336</v>
       </c>
       <c r="F186" t="s">
         <v>81</v>
@@ -7730,7 +7745,7 @@
     </row>
     <row r="187" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B187" t="s">
         <v>84</v>
@@ -7739,7 +7754,7 @@
         <v>328</v>
       </c>
       <c r="D187" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="E187" s="3">
         <v>2020</v>
@@ -7759,7 +7774,7 @@
     </row>
     <row r="188" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B188" t="s">
         <v>84</v>
@@ -7768,7 +7783,7 @@
         <v>328</v>
       </c>
       <c r="D188" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="E188" s="3">
         <v>2020</v>
@@ -7788,7 +7803,7 @@
     </row>
     <row r="189" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B189" t="s">
         <v>84</v>
@@ -7799,8 +7814,8 @@
       <c r="D189" t="s">
         <v>342</v>
       </c>
-      <c r="E189" s="9" t="s">
-        <v>336</v>
+      <c r="E189" s="3">
+        <v>2020</v>
       </c>
       <c r="F189" t="s">
         <v>81</v>
@@ -7817,7 +7832,7 @@
     </row>
     <row r="190" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B190" t="s">
         <v>84</v>
@@ -7826,7 +7841,7 @@
         <v>328</v>
       </c>
       <c r="D190" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="E190" s="9" t="s">
         <v>336</v>
@@ -7846,7 +7861,7 @@
     </row>
     <row r="191" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B191" t="s">
         <v>84</v>
@@ -7855,7 +7870,7 @@
         <v>328</v>
       </c>
       <c r="D191" t="s">
-        <v>346</v>
+        <v>329</v>
       </c>
       <c r="E191" s="9" t="s">
         <v>336</v>
@@ -7875,7 +7890,7 @@
     </row>
     <row r="192" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B192" t="s">
         <v>84</v>
@@ -7884,10 +7899,10 @@
         <v>328</v>
       </c>
       <c r="D192" t="s">
-        <v>348</v>
-      </c>
-      <c r="E192" s="3">
-        <v>2015</v>
+        <v>346</v>
+      </c>
+      <c r="E192" s="9" t="s">
+        <v>336</v>
       </c>
       <c r="F192" t="s">
         <v>81</v>
@@ -7904,19 +7919,19 @@
     </row>
     <row r="193" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B193" t="s">
         <v>84</v>
       </c>
       <c r="C193" t="s">
-        <v>350</v>
+        <v>328</v>
       </c>
       <c r="D193" t="s">
-        <v>351</v>
-      </c>
-      <c r="E193" s="9" t="s">
-        <v>79</v>
+        <v>348</v>
+      </c>
+      <c r="E193" s="3">
+        <v>2015</v>
       </c>
       <c r="F193" t="s">
         <v>81</v>
@@ -7928,12 +7943,12 @@
       <c r="J193" s="3"/>
       <c r="L193" s="3"/>
       <c r="N193" t="s">
-        <v>352</v>
+        <v>330</v>
       </c>
     </row>
     <row r="194" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="B194" t="s">
         <v>84</v>
@@ -7942,7 +7957,7 @@
         <v>350</v>
       </c>
       <c r="D194" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="E194" s="9" t="s">
         <v>79</v>
@@ -7957,12 +7972,12 @@
       <c r="J194" s="3"/>
       <c r="L194" s="3"/>
       <c r="N194" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="195" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="195" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="B195" t="s">
         <v>84</v>
@@ -7971,7 +7986,7 @@
         <v>350</v>
       </c>
       <c r="D195" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E195" s="9" t="s">
         <v>79</v>
@@ -7986,6 +8001,35 @@
       <c r="J195" s="3"/>
       <c r="L195" s="3"/>
       <c r="N195" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="196" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A196" t="s">
+        <v>356</v>
+      </c>
+      <c r="B196" t="s">
+        <v>84</v>
+      </c>
+      <c r="C196" t="s">
+        <v>350</v>
+      </c>
+      <c r="D196" t="s">
+        <v>357</v>
+      </c>
+      <c r="E196" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F196" t="s">
+        <v>81</v>
+      </c>
+      <c r="G196" t="s">
+        <v>82</v>
+      </c>
+      <c r="H196" s="3"/>
+      <c r="J196" s="3"/>
+      <c r="L196" s="3"/>
+      <c r="N196" t="s">
         <v>358</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added in GLAD Landsat (GLAD-L) alerts for after 2020 combined, and each annual time step; added in annual timesteps for DIST alerts for 2024-2026
</commit_message>
<xml_diff>
--- a/whisp_columns.xlsx
+++ b/whisp_columns.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnell\Documents\GitHub\whisp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73BD1CF-3F80-4868-A3BF-967D1406E478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2483E82-E14A-4683-A9FE-C0501ACEAFB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1502" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1555" uniqueCount="376">
   <si>
     <t>Column name</t>
   </si>
@@ -1109,17 +1109,53 @@
     <t>DIST_after_2020</t>
   </si>
   <si>
-    <t>2023-2026</t>
-  </si>
-  <si>
     <t>Pickens 2025</t>
+  </si>
+  <si>
+    <t>2024-2026</t>
+  </si>
+  <si>
+    <t>DIST_year_2024</t>
+  </si>
+  <si>
+    <t>DIST_year_2025</t>
+  </si>
+  <si>
+    <t>DIST_year_2026</t>
+  </si>
+  <si>
+    <t>GLAD-L_year_2001</t>
+  </si>
+  <si>
+    <t>GLAD-L_year_2002</t>
+  </si>
+  <si>
+    <t>GLAD-L_year_2003</t>
+  </si>
+  <si>
+    <t>GLAD-L_year_2004</t>
+  </si>
+  <si>
+    <t>GLAD-L_year_2005</t>
+  </si>
+  <si>
+    <t>GLAD-L_year_2006</t>
+  </si>
+  <si>
+    <t>Hansen 2016</t>
+  </si>
+  <si>
+    <t>GLAD-L_after_2020</t>
+  </si>
+  <si>
+    <t>2021-2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1137,6 +1173,18 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1192,7 +1240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1224,6 +1272,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1529,7 +1578,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:N196"/>
+  <dimension ref="A1:N206"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.7265625" bestFit="1" customWidth="1"/>
@@ -5189,7 +5238,7 @@
     </row>
     <row r="109" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>226</v>
+        <v>364</v>
       </c>
       <c r="B109" t="s">
         <v>15</v>
@@ -5198,13 +5247,13 @@
         <v>16</v>
       </c>
       <c r="D109" t="s">
-        <v>227</v>
-      </c>
-      <c r="E109" s="3">
-        <v>2001</v>
+        <v>194</v>
+      </c>
+      <c r="E109" s="9">
+        <v>2024</v>
       </c>
       <c r="F109" t="s">
-        <v>228</v>
+        <v>362</v>
       </c>
       <c r="H109" s="4">
         <v>0</v>
@@ -5220,7 +5269,7 @@
     </row>
     <row r="110" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>229</v>
+        <v>365</v>
       </c>
       <c r="B110" t="s">
         <v>15</v>
@@ -5229,13 +5278,13 @@
         <v>16</v>
       </c>
       <c r="D110" t="s">
-        <v>227</v>
-      </c>
-      <c r="E110" s="3">
-        <v>2002</v>
+        <v>194</v>
+      </c>
+      <c r="E110" s="9">
+        <v>2025</v>
       </c>
       <c r="F110" t="s">
-        <v>228</v>
+        <v>362</v>
       </c>
       <c r="H110" s="4">
         <v>0</v>
@@ -5251,7 +5300,7 @@
     </row>
     <row r="111" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>230</v>
+        <v>366</v>
       </c>
       <c r="B111" t="s">
         <v>15</v>
@@ -5260,13 +5309,13 @@
         <v>16</v>
       </c>
       <c r="D111" t="s">
-        <v>227</v>
-      </c>
-      <c r="E111" s="3">
-        <v>2003</v>
+        <v>194</v>
+      </c>
+      <c r="E111" s="9">
+        <v>2026</v>
       </c>
       <c r="F111" t="s">
-        <v>228</v>
+        <v>362</v>
       </c>
       <c r="H111" s="4">
         <v>0</v>
@@ -5282,7 +5331,7 @@
     </row>
     <row r="112" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>231</v>
+        <v>367</v>
       </c>
       <c r="B112" t="s">
         <v>15</v>
@@ -5291,14 +5340,15 @@
         <v>16</v>
       </c>
       <c r="D112" t="s">
-        <v>227</v>
-      </c>
-      <c r="E112" s="3">
-        <v>2004</v>
+        <v>194</v>
+      </c>
+      <c r="E112" s="9">
+        <v>2021</v>
       </c>
       <c r="F112" t="s">
-        <v>228</v>
-      </c>
+        <v>373</v>
+      </c>
+      <c r="G112" s="11"/>
       <c r="H112" s="4">
         <v>0</v>
       </c>
@@ -5313,7 +5363,7 @@
     </row>
     <row r="113" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>232</v>
+        <v>368</v>
       </c>
       <c r="B113" t="s">
         <v>15</v>
@@ -5322,13 +5372,13 @@
         <v>16</v>
       </c>
       <c r="D113" t="s">
-        <v>227</v>
-      </c>
-      <c r="E113" s="3">
-        <v>2005</v>
+        <v>194</v>
+      </c>
+      <c r="E113" s="9">
+        <v>2022</v>
       </c>
       <c r="F113" t="s">
-        <v>228</v>
+        <v>373</v>
       </c>
       <c r="H113" s="4">
         <v>0</v>
@@ -5344,7 +5394,7 @@
     </row>
     <row r="114" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>233</v>
+        <v>369</v>
       </c>
       <c r="B114" t="s">
         <v>15</v>
@@ -5353,13 +5403,13 @@
         <v>16</v>
       </c>
       <c r="D114" t="s">
-        <v>227</v>
-      </c>
-      <c r="E114" s="3">
-        <v>2006</v>
+        <v>194</v>
+      </c>
+      <c r="E114" s="9">
+        <v>2023</v>
       </c>
       <c r="F114" t="s">
-        <v>228</v>
+        <v>373</v>
       </c>
       <c r="H114" s="4">
         <v>0</v>
@@ -5375,7 +5425,7 @@
     </row>
     <row r="115" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>234</v>
+        <v>370</v>
       </c>
       <c r="B115" t="s">
         <v>15</v>
@@ -5384,13 +5434,13 @@
         <v>16</v>
       </c>
       <c r="D115" t="s">
-        <v>227</v>
-      </c>
-      <c r="E115" s="3">
-        <v>2007</v>
+        <v>194</v>
+      </c>
+      <c r="E115" s="9">
+        <v>2024</v>
       </c>
       <c r="F115" t="s">
-        <v>228</v>
+        <v>373</v>
       </c>
       <c r="H115" s="4">
         <v>0</v>
@@ -5406,7 +5456,7 @@
     </row>
     <row r="116" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>235</v>
+        <v>371</v>
       </c>
       <c r="B116" t="s">
         <v>15</v>
@@ -5415,13 +5465,13 @@
         <v>16</v>
       </c>
       <c r="D116" t="s">
-        <v>227</v>
-      </c>
-      <c r="E116" s="3">
-        <v>2008</v>
+        <v>194</v>
+      </c>
+      <c r="E116" s="9">
+        <v>2025</v>
       </c>
       <c r="F116" t="s">
-        <v>228</v>
+        <v>373</v>
       </c>
       <c r="H116" s="4">
         <v>0</v>
@@ -5437,7 +5487,7 @@
     </row>
     <row r="117" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>236</v>
+        <v>372</v>
       </c>
       <c r="B117" t="s">
         <v>15</v>
@@ -5446,13 +5496,13 @@
         <v>16</v>
       </c>
       <c r="D117" t="s">
-        <v>227</v>
-      </c>
-      <c r="E117" s="3">
-        <v>2009</v>
+        <v>194</v>
+      </c>
+      <c r="E117" s="9">
+        <v>2026</v>
       </c>
       <c r="F117" t="s">
-        <v>228</v>
+        <v>373</v>
       </c>
       <c r="H117" s="4">
         <v>0</v>
@@ -5468,7 +5518,7 @@
     </row>
     <row r="118" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="B118" t="s">
         <v>15</v>
@@ -5480,7 +5530,7 @@
         <v>227</v>
       </c>
       <c r="E118" s="3">
-        <v>2010</v>
+        <v>2001</v>
       </c>
       <c r="F118" t="s">
         <v>228</v>
@@ -5499,7 +5549,7 @@
     </row>
     <row r="119" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="B119" t="s">
         <v>15</v>
@@ -5511,7 +5561,7 @@
         <v>227</v>
       </c>
       <c r="E119" s="3">
-        <v>2011</v>
+        <v>2002</v>
       </c>
       <c r="F119" t="s">
         <v>228</v>
@@ -5530,7 +5580,7 @@
     </row>
     <row r="120" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="B120" t="s">
         <v>15</v>
@@ -5542,7 +5592,7 @@
         <v>227</v>
       </c>
       <c r="E120" s="3">
-        <v>2012</v>
+        <v>2003</v>
       </c>
       <c r="F120" t="s">
         <v>228</v>
@@ -5561,7 +5611,7 @@
     </row>
     <row r="121" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="B121" t="s">
         <v>15</v>
@@ -5573,7 +5623,7 @@
         <v>227</v>
       </c>
       <c r="E121" s="3">
-        <v>2013</v>
+        <v>2004</v>
       </c>
       <c r="F121" t="s">
         <v>228</v>
@@ -5592,7 +5642,7 @@
     </row>
     <row r="122" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="B122" t="s">
         <v>15</v>
@@ -5604,7 +5654,7 @@
         <v>227</v>
       </c>
       <c r="E122" s="3">
-        <v>2014</v>
+        <v>2005</v>
       </c>
       <c r="F122" t="s">
         <v>228</v>
@@ -5623,7 +5673,7 @@
     </row>
     <row r="123" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="B123" t="s">
         <v>15</v>
@@ -5635,7 +5685,7 @@
         <v>227</v>
       </c>
       <c r="E123" s="3">
-        <v>2015</v>
+        <v>2006</v>
       </c>
       <c r="F123" t="s">
         <v>228</v>
@@ -5654,7 +5704,7 @@
     </row>
     <row r="124" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="B124" t="s">
         <v>15</v>
@@ -5666,7 +5716,7 @@
         <v>227</v>
       </c>
       <c r="E124" s="3">
-        <v>2016</v>
+        <v>2007</v>
       </c>
       <c r="F124" t="s">
         <v>228</v>
@@ -5685,7 +5735,7 @@
     </row>
     <row r="125" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="B125" t="s">
         <v>15</v>
@@ -5697,7 +5747,7 @@
         <v>227</v>
       </c>
       <c r="E125" s="3">
-        <v>2017</v>
+        <v>2008</v>
       </c>
       <c r="F125" t="s">
         <v>228</v>
@@ -5716,7 +5766,7 @@
     </row>
     <row r="126" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="B126" t="s">
         <v>15</v>
@@ -5728,7 +5778,7 @@
         <v>227</v>
       </c>
       <c r="E126" s="3">
-        <v>2018</v>
+        <v>2009</v>
       </c>
       <c r="F126" t="s">
         <v>228</v>
@@ -5747,7 +5797,7 @@
     </row>
     <row r="127" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="B127" t="s">
         <v>15</v>
@@ -5759,7 +5809,7 @@
         <v>227</v>
       </c>
       <c r="E127" s="3">
-        <v>2019</v>
+        <v>2010</v>
       </c>
       <c r="F127" t="s">
         <v>228</v>
@@ -5778,7 +5828,7 @@
     </row>
     <row r="128" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="B128" t="s">
         <v>15</v>
@@ -5790,7 +5840,7 @@
         <v>227</v>
       </c>
       <c r="E128" s="3">
-        <v>2020</v>
+        <v>2011</v>
       </c>
       <c r="F128" t="s">
         <v>228</v>
@@ -5809,7 +5859,7 @@
     </row>
     <row r="129" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="B129" t="s">
         <v>15</v>
@@ -5821,10 +5871,10 @@
         <v>227</v>
       </c>
       <c r="E129" s="3">
-        <v>2000</v>
+        <v>2012</v>
       </c>
       <c r="F129" t="s">
-        <v>249</v>
+        <v>228</v>
       </c>
       <c r="H129" s="4">
         <v>0</v>
@@ -5840,7 +5890,7 @@
     </row>
     <row r="130" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="B130" t="s">
         <v>15</v>
@@ -5852,10 +5902,10 @@
         <v>227</v>
       </c>
       <c r="E130" s="3">
-        <v>2001</v>
+        <v>2013</v>
       </c>
       <c r="F130" t="s">
-        <v>249</v>
+        <v>228</v>
       </c>
       <c r="H130" s="4">
         <v>0</v>
@@ -5871,7 +5921,7 @@
     </row>
     <row r="131" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="B131" t="s">
         <v>15</v>
@@ -5883,10 +5933,10 @@
         <v>227</v>
       </c>
       <c r="E131" s="3">
-        <v>2002</v>
+        <v>2014</v>
       </c>
       <c r="F131" t="s">
-        <v>249</v>
+        <v>228</v>
       </c>
       <c r="H131" s="4">
         <v>0</v>
@@ -5902,7 +5952,7 @@
     </row>
     <row r="132" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="B132" t="s">
         <v>15</v>
@@ -5914,10 +5964,10 @@
         <v>227</v>
       </c>
       <c r="E132" s="3">
-        <v>2003</v>
+        <v>2015</v>
       </c>
       <c r="F132" t="s">
-        <v>249</v>
+        <v>228</v>
       </c>
       <c r="H132" s="4">
         <v>0</v>
@@ -5933,7 +5983,7 @@
     </row>
     <row r="133" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="B133" t="s">
         <v>15</v>
@@ -5945,10 +5995,10 @@
         <v>227</v>
       </c>
       <c r="E133" s="3">
-        <v>2004</v>
+        <v>2016</v>
       </c>
       <c r="F133" t="s">
-        <v>249</v>
+        <v>228</v>
       </c>
       <c r="H133" s="4">
         <v>0</v>
@@ -5964,7 +6014,7 @@
     </row>
     <row r="134" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="B134" t="s">
         <v>15</v>
@@ -5976,10 +6026,10 @@
         <v>227</v>
       </c>
       <c r="E134" s="3">
-        <v>2005</v>
+        <v>2017</v>
       </c>
       <c r="F134" t="s">
-        <v>249</v>
+        <v>228</v>
       </c>
       <c r="H134" s="4">
         <v>0</v>
@@ -5995,7 +6045,7 @@
     </row>
     <row r="135" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="B135" t="s">
         <v>15</v>
@@ -6007,10 +6057,10 @@
         <v>227</v>
       </c>
       <c r="E135" s="3">
-        <v>2006</v>
+        <v>2018</v>
       </c>
       <c r="F135" t="s">
-        <v>249</v>
+        <v>228</v>
       </c>
       <c r="H135" s="4">
         <v>0</v>
@@ -6026,7 +6076,7 @@
     </row>
     <row r="136" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="B136" t="s">
         <v>15</v>
@@ -6038,10 +6088,10 @@
         <v>227</v>
       </c>
       <c r="E136" s="3">
-        <v>2007</v>
+        <v>2019</v>
       </c>
       <c r="F136" t="s">
-        <v>249</v>
+        <v>228</v>
       </c>
       <c r="H136" s="4">
         <v>0</v>
@@ -6057,7 +6107,7 @@
     </row>
     <row r="137" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="B137" t="s">
         <v>15</v>
@@ -6069,10 +6119,10 @@
         <v>227</v>
       </c>
       <c r="E137" s="3">
-        <v>2008</v>
+        <v>2020</v>
       </c>
       <c r="F137" t="s">
-        <v>249</v>
+        <v>228</v>
       </c>
       <c r="H137" s="4">
         <v>0</v>
@@ -6088,7 +6138,7 @@
     </row>
     <row r="138" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="B138" t="s">
         <v>15</v>
@@ -6100,7 +6150,7 @@
         <v>227</v>
       </c>
       <c r="E138" s="3">
-        <v>2009</v>
+        <v>2000</v>
       </c>
       <c r="F138" t="s">
         <v>249</v>
@@ -6119,7 +6169,7 @@
     </row>
     <row r="139" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="B139" t="s">
         <v>15</v>
@@ -6131,7 +6181,7 @@
         <v>227</v>
       </c>
       <c r="E139" s="3">
-        <v>2010</v>
+        <v>2001</v>
       </c>
       <c r="F139" t="s">
         <v>249</v>
@@ -6150,7 +6200,7 @@
     </row>
     <row r="140" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="B140" t="s">
         <v>15</v>
@@ -6162,7 +6212,7 @@
         <v>227</v>
       </c>
       <c r="E140" s="3">
-        <v>2011</v>
+        <v>2002</v>
       </c>
       <c r="F140" t="s">
         <v>249</v>
@@ -6181,7 +6231,7 @@
     </row>
     <row r="141" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="B141" t="s">
         <v>15</v>
@@ -6193,7 +6243,7 @@
         <v>227</v>
       </c>
       <c r="E141" s="3">
-        <v>2012</v>
+        <v>2003</v>
       </c>
       <c r="F141" t="s">
         <v>249</v>
@@ -6212,7 +6262,7 @@
     </row>
     <row r="142" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="B142" t="s">
         <v>15</v>
@@ -6224,7 +6274,7 @@
         <v>227</v>
       </c>
       <c r="E142" s="3">
-        <v>2013</v>
+        <v>2004</v>
       </c>
       <c r="F142" t="s">
         <v>249</v>
@@ -6243,7 +6293,7 @@
     </row>
     <row r="143" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="B143" t="s">
         <v>15</v>
@@ -6255,7 +6305,7 @@
         <v>227</v>
       </c>
       <c r="E143" s="3">
-        <v>2014</v>
+        <v>2005</v>
       </c>
       <c r="F143" t="s">
         <v>249</v>
@@ -6274,7 +6324,7 @@
     </row>
     <row r="144" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="B144" t="s">
         <v>15</v>
@@ -6286,7 +6336,7 @@
         <v>227</v>
       </c>
       <c r="E144" s="3">
-        <v>2015</v>
+        <v>2006</v>
       </c>
       <c r="F144" t="s">
         <v>249</v>
@@ -6305,7 +6355,7 @@
     </row>
     <row r="145" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="B145" t="s">
         <v>15</v>
@@ -6317,7 +6367,7 @@
         <v>227</v>
       </c>
       <c r="E145" s="3">
-        <v>2016</v>
+        <v>2007</v>
       </c>
       <c r="F145" t="s">
         <v>249</v>
@@ -6336,7 +6386,7 @@
     </row>
     <row r="146" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="B146" t="s">
         <v>15</v>
@@ -6348,7 +6398,7 @@
         <v>227</v>
       </c>
       <c r="E146" s="3">
-        <v>2017</v>
+        <v>2008</v>
       </c>
       <c r="F146" t="s">
         <v>249</v>
@@ -6367,7 +6417,7 @@
     </row>
     <row r="147" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="B147" t="s">
         <v>15</v>
@@ -6379,7 +6429,7 @@
         <v>227</v>
       </c>
       <c r="E147" s="3">
-        <v>2018</v>
+        <v>2009</v>
       </c>
       <c r="F147" t="s">
         <v>249</v>
@@ -6398,7 +6448,7 @@
     </row>
     <row r="148" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="B148" t="s">
         <v>15</v>
@@ -6410,7 +6460,7 @@
         <v>227</v>
       </c>
       <c r="E148" s="3">
-        <v>2019</v>
+        <v>2010</v>
       </c>
       <c r="F148" t="s">
         <v>249</v>
@@ -6429,7 +6479,7 @@
     </row>
     <row r="149" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="B149" t="s">
         <v>15</v>
@@ -6441,7 +6491,7 @@
         <v>227</v>
       </c>
       <c r="E149" s="3">
-        <v>2020</v>
+        <v>2011</v>
       </c>
       <c r="F149" t="s">
         <v>249</v>
@@ -6460,7 +6510,7 @@
     </row>
     <row r="150" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="B150" t="s">
         <v>15</v>
@@ -6472,7 +6522,7 @@
         <v>227</v>
       </c>
       <c r="E150" s="3">
-        <v>2021</v>
+        <v>2012</v>
       </c>
       <c r="F150" t="s">
         <v>249</v>
@@ -6491,7 +6541,7 @@
     </row>
     <row r="151" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="B151" t="s">
         <v>15</v>
@@ -6503,7 +6553,7 @@
         <v>227</v>
       </c>
       <c r="E151" s="3">
-        <v>2022</v>
+        <v>2013</v>
       </c>
       <c r="F151" t="s">
         <v>249</v>
@@ -6522,7 +6572,7 @@
     </row>
     <row r="152" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="B152" t="s">
         <v>15</v>
@@ -6534,7 +6584,7 @@
         <v>227</v>
       </c>
       <c r="E152" s="3">
-        <v>2023</v>
+        <v>2014</v>
       </c>
       <c r="F152" t="s">
         <v>249</v>
@@ -6553,7 +6603,7 @@
     </row>
     <row r="153" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="B153" t="s">
         <v>15</v>
@@ -6565,7 +6615,7 @@
         <v>227</v>
       </c>
       <c r="E153" s="3">
-        <v>2024</v>
+        <v>2015</v>
       </c>
       <c r="F153" t="s">
         <v>249</v>
@@ -6584,7 +6634,7 @@
     </row>
     <row r="154" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="B154" t="s">
         <v>15</v>
@@ -6596,7 +6646,7 @@
         <v>227</v>
       </c>
       <c r="E154" s="3">
-        <v>2025</v>
+        <v>2016</v>
       </c>
       <c r="F154" t="s">
         <v>249</v>
@@ -6615,7 +6665,7 @@
     </row>
     <row r="155" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="B155" t="s">
         <v>15</v>
@@ -6624,23 +6674,18 @@
         <v>16</v>
       </c>
       <c r="D155" t="s">
-        <v>50</v>
-      </c>
-      <c r="E155" s="9" t="s">
-        <v>276</v>
+        <v>227</v>
+      </c>
+      <c r="E155" s="3">
+        <v>2017</v>
       </c>
       <c r="F155" t="s">
-        <v>120</v>
-      </c>
-      <c r="G155" t="s">
-        <v>82</v>
+        <v>249</v>
       </c>
       <c r="H155" s="4">
-        <v>1</v>
-      </c>
-      <c r="I155" s="5" t="s">
-        <v>48</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I155" s="5"/>
       <c r="J155" s="4">
         <v>0</v>
       </c>
@@ -6651,7 +6696,7 @@
     </row>
     <row r="156" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="B156" t="s">
         <v>15</v>
@@ -6660,23 +6705,18 @@
         <v>16</v>
       </c>
       <c r="D156" t="s">
-        <v>46</v>
-      </c>
-      <c r="E156" s="9" t="s">
-        <v>276</v>
+        <v>227</v>
+      </c>
+      <c r="E156" s="3">
+        <v>2018</v>
       </c>
       <c r="F156" t="s">
-        <v>120</v>
-      </c>
-      <c r="G156" t="s">
-        <v>82</v>
+        <v>249</v>
       </c>
       <c r="H156" s="4">
-        <v>1</v>
-      </c>
-      <c r="I156" s="5" t="s">
-        <v>48</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I156" s="5"/>
       <c r="J156" s="4">
         <v>0</v>
       </c>
@@ -6687,7 +6727,7 @@
     </row>
     <row r="157" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="B157" t="s">
         <v>15</v>
@@ -6696,23 +6736,18 @@
         <v>16</v>
       </c>
       <c r="D157" t="s">
-        <v>194</v>
-      </c>
-      <c r="E157" s="9" t="s">
-        <v>276</v>
+        <v>227</v>
+      </c>
+      <c r="E157" s="3">
+        <v>2019</v>
       </c>
       <c r="F157" t="s">
-        <v>122</v>
-      </c>
-      <c r="G157" t="s">
-        <v>82</v>
+        <v>249</v>
       </c>
       <c r="H157" s="4">
-        <v>1</v>
-      </c>
-      <c r="I157" s="5" t="s">
-        <v>48</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I157" s="5"/>
       <c r="J157" s="4">
         <v>0</v>
       </c>
@@ -6723,7 +6758,7 @@
     </row>
     <row r="158" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="B158" t="s">
         <v>15</v>
@@ -6732,23 +6767,18 @@
         <v>16</v>
       </c>
       <c r="D158" t="s">
-        <v>280</v>
-      </c>
-      <c r="E158" s="9" t="s">
-        <v>276</v>
+        <v>227</v>
+      </c>
+      <c r="E158" s="3">
+        <v>2020</v>
       </c>
       <c r="F158" t="s">
-        <v>228</v>
-      </c>
-      <c r="G158" t="s">
-        <v>82</v>
+        <v>249</v>
       </c>
       <c r="H158" s="4">
-        <v>1</v>
-      </c>
-      <c r="I158" s="5" t="s">
-        <v>48</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I158" s="5"/>
       <c r="J158" s="4">
         <v>0</v>
       </c>
@@ -6759,7 +6789,7 @@
     </row>
     <row r="159" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="B159" t="s">
         <v>15</v>
@@ -6768,23 +6798,18 @@
         <v>16</v>
       </c>
       <c r="D159" t="s">
-        <v>280</v>
-      </c>
-      <c r="E159" s="9" t="s">
-        <v>276</v>
+        <v>227</v>
+      </c>
+      <c r="E159" s="3">
+        <v>2021</v>
       </c>
       <c r="F159" t="s">
         <v>249</v>
       </c>
-      <c r="G159" t="s">
-        <v>82</v>
-      </c>
       <c r="H159" s="4">
-        <v>1</v>
-      </c>
-      <c r="I159" s="5" t="s">
-        <v>48</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I159" s="5"/>
       <c r="J159" s="4">
         <v>0</v>
       </c>
@@ -6795,7 +6820,7 @@
     </row>
     <row r="160" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="B160" t="s">
         <v>15</v>
@@ -6804,23 +6829,18 @@
         <v>16</v>
       </c>
       <c r="D160" t="s">
-        <v>194</v>
-      </c>
-      <c r="E160" s="9" t="s">
-        <v>283</v>
+        <v>227</v>
+      </c>
+      <c r="E160" s="3">
+        <v>2022</v>
       </c>
       <c r="F160" t="s">
-        <v>219</v>
-      </c>
-      <c r="G160" t="s">
-        <v>82</v>
+        <v>249</v>
       </c>
       <c r="H160" s="4">
-        <v>1</v>
-      </c>
-      <c r="I160" s="5" t="s">
-        <v>48</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I160" s="5"/>
       <c r="J160" s="4">
         <v>0</v>
       </c>
@@ -6829,9 +6849,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="B161" t="s">
         <v>15</v>
@@ -6840,127 +6860,106 @@
         <v>16</v>
       </c>
       <c r="D161" t="s">
+        <v>227</v>
+      </c>
+      <c r="E161" s="3">
+        <v>2023</v>
+      </c>
+      <c r="F161" t="s">
+        <v>249</v>
+      </c>
+      <c r="H161" s="4">
+        <v>0</v>
+      </c>
+      <c r="I161" s="5"/>
+      <c r="J161" s="4">
+        <v>0</v>
+      </c>
+      <c r="K161" s="5"/>
+      <c r="L161" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A162" t="s">
+        <v>273</v>
+      </c>
+      <c r="B162" t="s">
+        <v>15</v>
+      </c>
+      <c r="C162" t="s">
+        <v>16</v>
+      </c>
+      <c r="D162" t="s">
+        <v>227</v>
+      </c>
+      <c r="E162" s="3">
+        <v>2024</v>
+      </c>
+      <c r="F162" t="s">
+        <v>249</v>
+      </c>
+      <c r="H162" s="4">
+        <v>0</v>
+      </c>
+      <c r="I162" s="5"/>
+      <c r="J162" s="4">
+        <v>0</v>
+      </c>
+      <c r="K162" s="5"/>
+      <c r="L162" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A163" t="s">
+        <v>274</v>
+      </c>
+      <c r="B163" t="s">
+        <v>15</v>
+      </c>
+      <c r="C163" t="s">
+        <v>16</v>
+      </c>
+      <c r="D163" t="s">
+        <v>227</v>
+      </c>
+      <c r="E163" s="3">
+        <v>2025</v>
+      </c>
+      <c r="F163" t="s">
+        <v>249</v>
+      </c>
+      <c r="H163" s="4">
+        <v>0</v>
+      </c>
+      <c r="I163" s="5"/>
+      <c r="J163" s="4">
+        <v>0</v>
+      </c>
+      <c r="K163" s="5"/>
+      <c r="L163" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A164" t="s">
+        <v>275</v>
+      </c>
+      <c r="B164" t="s">
+        <v>15</v>
+      </c>
+      <c r="C164" t="s">
+        <v>16</v>
+      </c>
+      <c r="D164" t="s">
         <v>50</v>
       </c>
-      <c r="E161" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="F161" t="s">
+      <c r="E164" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="F164" t="s">
         <v>120</v>
-      </c>
-      <c r="G161" t="s">
-        <v>82</v>
-      </c>
-      <c r="H161" s="4">
-        <v>1</v>
-      </c>
-      <c r="I161" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="J161" s="4">
-        <v>1</v>
-      </c>
-      <c r="K161" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="L161" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="162" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A162" t="s">
-        <v>286</v>
-      </c>
-      <c r="B162" t="s">
-        <v>15</v>
-      </c>
-      <c r="C162" t="s">
-        <v>16</v>
-      </c>
-      <c r="D162" t="s">
-        <v>46</v>
-      </c>
-      <c r="E162" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="F162" t="s">
-        <v>120</v>
-      </c>
-      <c r="G162" t="s">
-        <v>82</v>
-      </c>
-      <c r="H162" s="4">
-        <v>1</v>
-      </c>
-      <c r="I162" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="J162" s="4">
-        <v>1</v>
-      </c>
-      <c r="K162" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="L162" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="163" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A163" t="s">
-        <v>287</v>
-      </c>
-      <c r="B163" t="s">
-        <v>15</v>
-      </c>
-      <c r="C163" t="s">
-        <v>16</v>
-      </c>
-      <c r="D163" t="s">
-        <v>194</v>
-      </c>
-      <c r="E163" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="F163" t="s">
-        <v>122</v>
-      </c>
-      <c r="G163" t="s">
-        <v>82</v>
-      </c>
-      <c r="H163" s="4">
-        <v>1</v>
-      </c>
-      <c r="I163" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="J163" s="4">
-        <v>1</v>
-      </c>
-      <c r="K163" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="L163" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="164" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A164" t="s">
-        <v>288</v>
-      </c>
-      <c r="B164" t="s">
-        <v>15</v>
-      </c>
-      <c r="C164" t="s">
-        <v>16</v>
-      </c>
-      <c r="D164" t="s">
-        <v>289</v>
-      </c>
-      <c r="E164" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="F164" t="s">
-        <v>228</v>
       </c>
       <c r="G164" t="s">
         <v>82</v>
@@ -6969,21 +6968,19 @@
         <v>1</v>
       </c>
       <c r="I164" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="J164" s="4">
-        <v>1</v>
-      </c>
-      <c r="K164" s="5" t="s">
-        <v>55</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K164" s="5"/>
       <c r="L164" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
-        <v>291</v>
+        <v>277</v>
       </c>
       <c r="B165" t="s">
         <v>15</v>
@@ -6992,13 +6989,13 @@
         <v>16</v>
       </c>
       <c r="D165" t="s">
-        <v>194</v>
+        <v>46</v>
       </c>
       <c r="E165" s="9" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="F165" t="s">
-        <v>249</v>
+        <v>120</v>
       </c>
       <c r="G165" t="s">
         <v>82</v>
@@ -7007,21 +7004,19 @@
         <v>1</v>
       </c>
       <c r="I165" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="J165" s="4">
-        <v>1</v>
-      </c>
-      <c r="K165" s="5" t="s">
-        <v>55</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K165" s="5"/>
       <c r="L165" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>361</v>
+        <v>278</v>
       </c>
       <c r="B166" t="s">
         <v>15</v>
@@ -7033,30 +7028,31 @@
         <v>194</v>
       </c>
       <c r="E166" s="9" t="s">
-        <v>362</v>
+        <v>276</v>
       </c>
       <c r="F166" t="s">
-        <v>363</v>
+        <v>122</v>
+      </c>
+      <c r="G166" t="s">
+        <v>82</v>
       </c>
       <c r="H166" s="4">
         <v>1</v>
       </c>
       <c r="I166" s="5" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="J166" s="4">
-        <v>1</v>
-      </c>
-      <c r="K166" s="5" t="s">
-        <v>55</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K166" s="5"/>
       <c r="L166" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
-        <v>292</v>
+        <v>279</v>
       </c>
       <c r="B167" t="s">
         <v>15</v>
@@ -7065,35 +7061,34 @@
         <v>16</v>
       </c>
       <c r="D167" t="s">
-        <v>24</v>
-      </c>
-      <c r="E167" s="3">
-        <v>2020</v>
+        <v>280</v>
+      </c>
+      <c r="E167" s="9" t="s">
+        <v>276</v>
       </c>
       <c r="F167" t="s">
-        <v>114</v>
+        <v>228</v>
       </c>
       <c r="G167" t="s">
         <v>82</v>
       </c>
       <c r="H167" s="4">
-        <v>0</v>
-      </c>
-      <c r="I167" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I167" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="J167" s="4">
         <v>0</v>
       </c>
       <c r="K167" s="5"/>
       <c r="L167" s="4">
-        <v>1</v>
-      </c>
-      <c r="M167" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="168" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="B168" t="s">
         <v>15</v>
@@ -7102,35 +7097,34 @@
         <v>16</v>
       </c>
       <c r="D168" t="s">
-        <v>294</v>
-      </c>
-      <c r="E168" s="3">
-        <v>2020</v>
+        <v>280</v>
+      </c>
+      <c r="E168" s="9" t="s">
+        <v>276</v>
       </c>
       <c r="F168" t="s">
-        <v>295</v>
+        <v>249</v>
       </c>
       <c r="G168" t="s">
         <v>82</v>
       </c>
       <c r="H168" s="4">
-        <v>0</v>
-      </c>
-      <c r="I168" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I168" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="J168" s="4">
         <v>0</v>
       </c>
       <c r="K168" s="5"/>
       <c r="L168" s="4">
-        <v>1</v>
-      </c>
-      <c r="M168" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="169" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
-        <v>296</v>
+        <v>282</v>
       </c>
       <c r="B169" t="s">
         <v>15</v>
@@ -7139,35 +7133,34 @@
         <v>16</v>
       </c>
       <c r="D169" t="s">
-        <v>24</v>
-      </c>
-      <c r="E169" s="3">
-        <v>2020</v>
+        <v>194</v>
+      </c>
+      <c r="E169" s="9" t="s">
+        <v>283</v>
       </c>
       <c r="F169" t="s">
-        <v>297</v>
+        <v>219</v>
       </c>
       <c r="G169" t="s">
         <v>82</v>
       </c>
       <c r="H169" s="4">
-        <v>0</v>
-      </c>
-      <c r="I169" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I169" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="J169" s="4">
         <v>0</v>
       </c>
       <c r="K169" s="5"/>
       <c r="L169" s="4">
-        <v>1</v>
-      </c>
-      <c r="M169" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="170" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
-        <v>298</v>
+        <v>284</v>
       </c>
       <c r="B170" t="s">
         <v>15</v>
@@ -7176,35 +7169,36 @@
         <v>16</v>
       </c>
       <c r="D170" t="s">
-        <v>299</v>
-      </c>
-      <c r="E170" s="3">
-        <v>2020</v>
+        <v>50</v>
+      </c>
+      <c r="E170" s="9" t="s">
+        <v>285</v>
       </c>
       <c r="F170" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="G170" t="s">
         <v>82</v>
       </c>
       <c r="H170" s="4">
-        <v>0</v>
-      </c>
-      <c r="I170" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I170" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="J170" s="4">
-        <v>0</v>
-      </c>
-      <c r="K170" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="K170" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="L170" s="4">
-        <v>1</v>
-      </c>
-      <c r="M170" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="171" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
-        <v>300</v>
+        <v>286</v>
       </c>
       <c r="B171" t="s">
         <v>15</v>
@@ -7213,35 +7207,36 @@
         <v>16</v>
       </c>
       <c r="D171" t="s">
-        <v>301</v>
-      </c>
-      <c r="E171" s="3">
-        <v>2020</v>
+        <v>46</v>
+      </c>
+      <c r="E171" s="9" t="s">
+        <v>285</v>
       </c>
       <c r="F171" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="G171" t="s">
         <v>82</v>
       </c>
       <c r="H171" s="4">
-        <v>0</v>
-      </c>
-      <c r="I171" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I171" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="J171" s="4">
-        <v>0</v>
-      </c>
-      <c r="K171" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="K171" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="L171" s="4">
-        <v>1</v>
-      </c>
-      <c r="M171" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="172" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
-        <v>302</v>
+        <v>287</v>
       </c>
       <c r="B172" t="s">
         <v>15</v>
@@ -7250,35 +7245,36 @@
         <v>16</v>
       </c>
       <c r="D172" t="s">
-        <v>303</v>
-      </c>
-      <c r="E172" s="3">
-        <v>2015</v>
+        <v>194</v>
+      </c>
+      <c r="E172" s="9" t="s">
+        <v>285</v>
       </c>
       <c r="F172" t="s">
-        <v>304</v>
+        <v>122</v>
+      </c>
+      <c r="G172" t="s">
+        <v>82</v>
       </c>
       <c r="H172" s="4">
-        <v>0</v>
-      </c>
-      <c r="I172" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I172" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="J172" s="4">
-        <v>0</v>
-      </c>
-      <c r="K172" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="K172" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="L172" s="4">
-        <v>1</v>
-      </c>
-      <c r="M172" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="N172" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="173" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
-        <v>306</v>
+        <v>288</v>
       </c>
       <c r="B173" t="s">
         <v>15</v>
@@ -7287,35 +7283,36 @@
         <v>16</v>
       </c>
       <c r="D173" t="s">
-        <v>307</v>
-      </c>
-      <c r="E173" s="3">
-        <v>2023</v>
+        <v>289</v>
+      </c>
+      <c r="E173" s="9" t="s">
+        <v>290</v>
       </c>
       <c r="F173" t="s">
-        <v>120</v>
+        <v>228</v>
       </c>
       <c r="G173" t="s">
         <v>82</v>
       </c>
       <c r="H173" s="4">
-        <v>0</v>
-      </c>
-      <c r="I173" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I173" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="J173" s="4">
-        <v>0</v>
-      </c>
-      <c r="K173" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="K173" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="L173" s="4">
-        <v>1</v>
-      </c>
-      <c r="M173" s="5" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="174" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
-        <v>309</v>
+        <v>291</v>
       </c>
       <c r="B174" t="s">
         <v>15</v>
@@ -7324,32 +7321,36 @@
         <v>16</v>
       </c>
       <c r="D174" t="s">
-        <v>310</v>
-      </c>
-      <c r="E174" s="3">
-        <v>2023</v>
+        <v>194</v>
+      </c>
+      <c r="E174" s="9" t="s">
+        <v>285</v>
       </c>
       <c r="F174" t="s">
-        <v>311</v>
+        <v>249</v>
+      </c>
+      <c r="G174" t="s">
+        <v>82</v>
       </c>
       <c r="H174" s="4">
-        <v>0</v>
-      </c>
-      <c r="I174" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I174" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="J174" s="4">
-        <v>0</v>
-      </c>
-      <c r="K174" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="K174" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="L174" s="4">
-        <v>1</v>
-      </c>
-      <c r="M174" s="5" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="175" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
-        <v>312</v>
+        <v>361</v>
       </c>
       <c r="B175" t="s">
         <v>15</v>
@@ -7358,35 +7359,33 @@
         <v>16</v>
       </c>
       <c r="D175" t="s">
-        <v>62</v>
-      </c>
-      <c r="E175" s="3">
-        <v>2023</v>
+        <v>194</v>
+      </c>
+      <c r="E175" s="9" t="s">
+        <v>363</v>
       </c>
       <c r="F175" t="s">
-        <v>126</v>
-      </c>
-      <c r="G175" t="s">
-        <v>82</v>
+        <v>362</v>
       </c>
       <c r="H175" s="4">
-        <v>0</v>
-      </c>
-      <c r="I175" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I175" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="J175" s="4">
-        <v>0</v>
-      </c>
-      <c r="K175" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="K175" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="L175" s="4">
-        <v>1</v>
-      </c>
-      <c r="M175" s="5" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="176" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
-        <v>314</v>
+        <v>374</v>
       </c>
       <c r="B176" t="s">
         <v>15</v>
@@ -7395,35 +7394,33 @@
         <v>16</v>
       </c>
       <c r="D176" t="s">
-        <v>138</v>
-      </c>
-      <c r="E176" s="3">
-        <v>2023</v>
+        <v>194</v>
+      </c>
+      <c r="E176" s="9" t="s">
+        <v>375</v>
       </c>
       <c r="F176" t="s">
-        <v>126</v>
-      </c>
-      <c r="G176" t="s">
-        <v>82</v>
+        <v>373</v>
       </c>
       <c r="H176" s="4">
-        <v>0</v>
-      </c>
-      <c r="I176" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="I176" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="J176" s="4">
-        <v>0</v>
-      </c>
-      <c r="K176" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="K176" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="L176" s="4">
-        <v>1</v>
-      </c>
-      <c r="M176" s="5" t="s">
-        <v>313</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
-        <v>315</v>
+        <v>292</v>
       </c>
       <c r="B177" t="s">
         <v>15</v>
@@ -7432,13 +7429,13 @@
         <v>16</v>
       </c>
       <c r="D177" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="E177" s="3">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="F177" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="G177" t="s">
         <v>82</v>
@@ -7455,12 +7452,12 @@
         <v>1</v>
       </c>
       <c r="M177" s="5" t="s">
-        <v>313</v>
+        <v>26</v>
       </c>
     </row>
     <row r="178" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
-        <v>316</v>
+        <v>293</v>
       </c>
       <c r="B178" t="s">
         <v>15</v>
@@ -7469,13 +7466,13 @@
         <v>16</v>
       </c>
       <c r="D178" t="s">
-        <v>74</v>
+        <v>294</v>
       </c>
       <c r="E178" s="3">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="F178" t="s">
-        <v>126</v>
+        <v>295</v>
       </c>
       <c r="G178" t="s">
         <v>82</v>
@@ -7492,12 +7489,12 @@
         <v>1</v>
       </c>
       <c r="M178" s="5" t="s">
-        <v>313</v>
+        <v>26</v>
       </c>
     </row>
     <row r="179" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
-        <v>317</v>
+        <v>296</v>
       </c>
       <c r="B179" t="s">
         <v>15</v>
@@ -7506,13 +7503,13 @@
         <v>16</v>
       </c>
       <c r="D179" t="s">
-        <v>318</v>
-      </c>
-      <c r="E179" s="3" t="s">
-        <v>319</v>
+        <v>24</v>
+      </c>
+      <c r="E179" s="3">
+        <v>2020</v>
       </c>
       <c r="F179" t="s">
-        <v>311</v>
+        <v>297</v>
       </c>
       <c r="G179" t="s">
         <v>82</v>
@@ -7529,12 +7526,12 @@
         <v>1</v>
       </c>
       <c r="M179" s="5" t="s">
-        <v>313</v>
+        <v>26</v>
       </c>
     </row>
     <row r="180" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>320</v>
+        <v>298</v>
       </c>
       <c r="B180" t="s">
         <v>15</v>
@@ -7543,13 +7540,13 @@
         <v>16</v>
       </c>
       <c r="D180" t="s">
-        <v>321</v>
+        <v>299</v>
       </c>
       <c r="E180" s="3">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="F180" t="s">
-        <v>322</v>
+        <v>114</v>
       </c>
       <c r="G180" t="s">
         <v>82</v>
@@ -7566,314 +7563,394 @@
         <v>1</v>
       </c>
       <c r="M180" s="5" t="s">
-        <v>323</v>
-      </c>
-      <c r="N180" t="s">
-        <v>324</v>
+        <v>28</v>
       </c>
     </row>
     <row r="181" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>325</v>
+        <v>300</v>
       </c>
       <c r="B181" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C181" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="D181" t="s">
-        <v>326</v>
-      </c>
-      <c r="E181" s="9" t="s">
-        <v>79</v>
+        <v>301</v>
+      </c>
+      <c r="E181" s="3">
+        <v>2020</v>
       </c>
       <c r="F181" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="G181" t="s">
         <v>82</v>
       </c>
-      <c r="H181" s="3"/>
-      <c r="J181" s="3"/>
-      <c r="L181" s="3"/>
-      <c r="N181" t="s">
-        <v>102</v>
+      <c r="H181" s="4">
+        <v>0</v>
+      </c>
+      <c r="I181" s="5"/>
+      <c r="J181" s="4">
+        <v>0</v>
+      </c>
+      <c r="K181" s="5"/>
+      <c r="L181" s="4">
+        <v>1</v>
+      </c>
+      <c r="M181" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="182" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
-        <v>359</v>
+        <v>302</v>
       </c>
       <c r="B182" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C182" t="s">
-        <v>79</v>
+        <v>16</v>
       </c>
       <c r="D182" t="s">
-        <v>360</v>
-      </c>
-      <c r="E182" s="3" t="s">
-        <v>79</v>
+        <v>303</v>
+      </c>
+      <c r="E182" s="3">
+        <v>2015</v>
       </c>
       <c r="F182" t="s">
-        <v>81</v>
-      </c>
-      <c r="H182" s="4"/>
+        <v>304</v>
+      </c>
+      <c r="H182" s="4">
+        <v>0</v>
+      </c>
       <c r="I182" s="5"/>
-      <c r="J182" s="4"/>
+      <c r="J182" s="4">
+        <v>0</v>
+      </c>
       <c r="K182" s="5"/>
-      <c r="L182" s="4"/>
-      <c r="M182" s="5"/>
+      <c r="L182" s="4">
+        <v>1</v>
+      </c>
+      <c r="M182" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="N182" t="s">
+        <v>305</v>
+      </c>
     </row>
     <row r="183" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
-        <v>327</v>
+        <v>306</v>
       </c>
       <c r="B183" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C183" t="s">
-        <v>328</v>
+        <v>16</v>
       </c>
       <c r="D183" t="s">
-        <v>329</v>
+        <v>307</v>
       </c>
       <c r="E183" s="3">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="F183" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="G183" t="s">
         <v>82</v>
       </c>
-      <c r="H183" s="3"/>
-      <c r="J183" s="3"/>
-      <c r="L183" s="3"/>
-      <c r="N183" t="s">
-        <v>330</v>
+      <c r="H183" s="4">
+        <v>0</v>
+      </c>
+      <c r="I183" s="5"/>
+      <c r="J183" s="4">
+        <v>0</v>
+      </c>
+      <c r="K183" s="5"/>
+      <c r="L183" s="4">
+        <v>1</v>
+      </c>
+      <c r="M183" s="5" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="184" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
-        <v>331</v>
+        <v>309</v>
       </c>
       <c r="B184" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C184" t="s">
-        <v>328</v>
+        <v>16</v>
       </c>
       <c r="D184" t="s">
-        <v>332</v>
+        <v>310</v>
       </c>
       <c r="E184" s="3">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="F184" t="s">
-        <v>81</v>
-      </c>
-      <c r="G184" t="s">
-        <v>82</v>
-      </c>
-      <c r="H184" s="3"/>
-      <c r="J184" s="3"/>
-      <c r="L184" s="3"/>
-      <c r="N184" t="s">
-        <v>330</v>
+        <v>311</v>
+      </c>
+      <c r="H184" s="4">
+        <v>0</v>
+      </c>
+      <c r="I184" s="5"/>
+      <c r="J184" s="4">
+        <v>0</v>
+      </c>
+      <c r="K184" s="5"/>
+      <c r="L184" s="4">
+        <v>1</v>
+      </c>
+      <c r="M184" s="5" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="185" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
-        <v>333</v>
+        <v>312</v>
       </c>
       <c r="B185" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C185" t="s">
-        <v>328</v>
+        <v>16</v>
       </c>
       <c r="D185" t="s">
-        <v>334</v>
-      </c>
-      <c r="E185" s="9" t="s">
-        <v>276</v>
+        <v>62</v>
+      </c>
+      <c r="E185" s="3">
+        <v>2023</v>
       </c>
       <c r="F185" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G185" t="s">
         <v>82</v>
       </c>
-      <c r="H185" s="3"/>
-      <c r="J185" s="3"/>
-      <c r="L185" s="3"/>
-      <c r="N185" t="s">
-        <v>330</v>
+      <c r="H185" s="4">
+        <v>0</v>
+      </c>
+      <c r="I185" s="5"/>
+      <c r="J185" s="4">
+        <v>0</v>
+      </c>
+      <c r="K185" s="5"/>
+      <c r="L185" s="4">
+        <v>1</v>
+      </c>
+      <c r="M185" s="5" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="186" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>335</v>
+        <v>314</v>
       </c>
       <c r="B186" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C186" t="s">
-        <v>328</v>
+        <v>16</v>
       </c>
       <c r="D186" t="s">
-        <v>334</v>
-      </c>
-      <c r="E186" s="9" t="s">
-        <v>336</v>
+        <v>138</v>
+      </c>
+      <c r="E186" s="3">
+        <v>2023</v>
       </c>
       <c r="F186" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G186" t="s">
         <v>82</v>
       </c>
-      <c r="H186" s="3"/>
-      <c r="J186" s="3"/>
-      <c r="L186" s="3"/>
-      <c r="N186" t="s">
-        <v>330</v>
+      <c r="H186" s="4">
+        <v>0</v>
+      </c>
+      <c r="I186" s="5"/>
+      <c r="J186" s="4">
+        <v>0</v>
+      </c>
+      <c r="K186" s="5"/>
+      <c r="L186" s="4">
+        <v>1</v>
+      </c>
+      <c r="M186" s="5" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="187" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>337</v>
+        <v>315</v>
       </c>
       <c r="B187" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C187" t="s">
-        <v>328</v>
+        <v>16</v>
       </c>
       <c r="D187" t="s">
-        <v>338</v>
+        <v>60</v>
       </c>
       <c r="E187" s="3">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="F187" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G187" t="s">
         <v>82</v>
       </c>
-      <c r="H187" s="3"/>
-      <c r="J187" s="3"/>
-      <c r="L187" s="3"/>
-      <c r="N187" t="s">
-        <v>330</v>
+      <c r="H187" s="4">
+        <v>0</v>
+      </c>
+      <c r="I187" s="5"/>
+      <c r="J187" s="4">
+        <v>0</v>
+      </c>
+      <c r="K187" s="5"/>
+      <c r="L187" s="4">
+        <v>1</v>
+      </c>
+      <c r="M187" s="5" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="188" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>339</v>
+        <v>316</v>
       </c>
       <c r="B188" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C188" t="s">
-        <v>328</v>
+        <v>16</v>
       </c>
       <c r="D188" t="s">
-        <v>340</v>
+        <v>74</v>
       </c>
       <c r="E188" s="3">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="F188" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="G188" t="s">
         <v>82</v>
       </c>
-      <c r="H188" s="3"/>
-      <c r="J188" s="3"/>
-      <c r="L188" s="3"/>
-      <c r="N188" t="s">
-        <v>330</v>
+      <c r="H188" s="4">
+        <v>0</v>
+      </c>
+      <c r="I188" s="5"/>
+      <c r="J188" s="4">
+        <v>0</v>
+      </c>
+      <c r="K188" s="5"/>
+      <c r="L188" s="4">
+        <v>1</v>
+      </c>
+      <c r="M188" s="5" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="189" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>341</v>
+        <v>317</v>
       </c>
       <c r="B189" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C189" t="s">
-        <v>328</v>
+        <v>16</v>
       </c>
       <c r="D189" t="s">
-        <v>342</v>
-      </c>
-      <c r="E189" s="3">
-        <v>2020</v>
+        <v>318</v>
+      </c>
+      <c r="E189" s="3" t="s">
+        <v>319</v>
       </c>
       <c r="F189" t="s">
-        <v>81</v>
+        <v>311</v>
       </c>
       <c r="G189" t="s">
         <v>82</v>
       </c>
-      <c r="H189" s="3"/>
-      <c r="J189" s="3"/>
-      <c r="L189" s="3"/>
-      <c r="N189" t="s">
-        <v>330</v>
+      <c r="H189" s="4">
+        <v>0</v>
+      </c>
+      <c r="I189" s="5"/>
+      <c r="J189" s="4">
+        <v>0</v>
+      </c>
+      <c r="K189" s="5"/>
+      <c r="L189" s="4">
+        <v>1</v>
+      </c>
+      <c r="M189" s="5" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="190" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>343</v>
+        <v>320</v>
       </c>
       <c r="B190" t="s">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C190" t="s">
-        <v>328</v>
+        <v>16</v>
       </c>
       <c r="D190" t="s">
-        <v>342</v>
-      </c>
-      <c r="E190" s="9" t="s">
-        <v>336</v>
+        <v>321</v>
+      </c>
+      <c r="E190" s="3">
+        <v>2015</v>
       </c>
       <c r="F190" t="s">
-        <v>81</v>
+        <v>322</v>
       </c>
       <c r="G190" t="s">
         <v>82</v>
       </c>
-      <c r="H190" s="3"/>
-      <c r="J190" s="3"/>
-      <c r="L190" s="3"/>
+      <c r="H190" s="4">
+        <v>0</v>
+      </c>
+      <c r="I190" s="5"/>
+      <c r="J190" s="4">
+        <v>0</v>
+      </c>
+      <c r="K190" s="5"/>
+      <c r="L190" s="4">
+        <v>1</v>
+      </c>
+      <c r="M190" s="5" t="s">
+        <v>323</v>
+      </c>
       <c r="N190" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
     </row>
     <row r="191" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>344</v>
+        <v>325</v>
       </c>
       <c r="B191" t="s">
         <v>84</v>
       </c>
       <c r="C191" t="s">
-        <v>328</v>
+        <v>79</v>
       </c>
       <c r="D191" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="E191" s="9" t="s">
-        <v>336</v>
+        <v>79</v>
       </c>
       <c r="F191" t="s">
         <v>81</v>
@@ -7885,41 +7962,38 @@
       <c r="J191" s="3"/>
       <c r="L191" s="3"/>
       <c r="N191" t="s">
-        <v>330</v>
+        <v>102</v>
       </c>
     </row>
     <row r="192" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
-        <v>345</v>
+        <v>359</v>
       </c>
       <c r="B192" t="s">
         <v>84</v>
       </c>
       <c r="C192" t="s">
-        <v>328</v>
+        <v>79</v>
       </c>
       <c r="D192" t="s">
-        <v>346</v>
-      </c>
-      <c r="E192" s="9" t="s">
-        <v>336</v>
+        <v>360</v>
+      </c>
+      <c r="E192" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="F192" t="s">
         <v>81</v>
       </c>
-      <c r="G192" t="s">
-        <v>82</v>
-      </c>
-      <c r="H192" s="3"/>
-      <c r="J192" s="3"/>
-      <c r="L192" s="3"/>
-      <c r="N192" t="s">
-        <v>330</v>
-      </c>
+      <c r="H192" s="4"/>
+      <c r="I192" s="5"/>
+      <c r="J192" s="4"/>
+      <c r="K192" s="5"/>
+      <c r="L192" s="4"/>
+      <c r="M192" s="5"/>
     </row>
     <row r="193" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
-        <v>347</v>
+        <v>327</v>
       </c>
       <c r="B193" t="s">
         <v>84</v>
@@ -7928,10 +8002,10 @@
         <v>328</v>
       </c>
       <c r="D193" t="s">
-        <v>348</v>
+        <v>329</v>
       </c>
       <c r="E193" s="3">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="F193" t="s">
         <v>81</v>
@@ -7948,19 +8022,19 @@
     </row>
     <row r="194" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
-        <v>349</v>
+        <v>331</v>
       </c>
       <c r="B194" t="s">
         <v>84</v>
       </c>
       <c r="C194" t="s">
-        <v>350</v>
+        <v>328</v>
       </c>
       <c r="D194" t="s">
-        <v>351</v>
-      </c>
-      <c r="E194" s="9" t="s">
-        <v>79</v>
+        <v>332</v>
+      </c>
+      <c r="E194" s="3">
+        <v>2020</v>
       </c>
       <c r="F194" t="s">
         <v>81</v>
@@ -7972,24 +8046,24 @@
       <c r="J194" s="3"/>
       <c r="L194" s="3"/>
       <c r="N194" t="s">
-        <v>352</v>
+        <v>330</v>
       </c>
     </row>
     <row r="195" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
-        <v>353</v>
+        <v>333</v>
       </c>
       <c r="B195" t="s">
         <v>84</v>
       </c>
       <c r="C195" t="s">
-        <v>350</v>
+        <v>328</v>
       </c>
       <c r="D195" t="s">
-        <v>354</v>
+        <v>334</v>
       </c>
       <c r="E195" s="9" t="s">
-        <v>79</v>
+        <v>276</v>
       </c>
       <c r="F195" t="s">
         <v>81</v>
@@ -8001,24 +8075,24 @@
       <c r="J195" s="3"/>
       <c r="L195" s="3"/>
       <c r="N195" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="196" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="196" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
-        <v>356</v>
+        <v>335</v>
       </c>
       <c r="B196" t="s">
         <v>84</v>
       </c>
       <c r="C196" t="s">
-        <v>350</v>
+        <v>328</v>
       </c>
       <c r="D196" t="s">
-        <v>357</v>
+        <v>334</v>
       </c>
       <c r="E196" s="9" t="s">
-        <v>79</v>
+        <v>336</v>
       </c>
       <c r="F196" t="s">
         <v>81</v>
@@ -8030,11 +8104,303 @@
       <c r="J196" s="3"/>
       <c r="L196" s="3"/>
       <c r="N196" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="197" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A197" t="s">
+        <v>337</v>
+      </c>
+      <c r="B197" t="s">
+        <v>84</v>
+      </c>
+      <c r="C197" t="s">
+        <v>328</v>
+      </c>
+      <c r="D197" t="s">
+        <v>338</v>
+      </c>
+      <c r="E197" s="3">
+        <v>2020</v>
+      </c>
+      <c r="F197" t="s">
+        <v>81</v>
+      </c>
+      <c r="G197" t="s">
+        <v>82</v>
+      </c>
+      <c r="H197" s="3"/>
+      <c r="J197" s="3"/>
+      <c r="L197" s="3"/>
+      <c r="N197" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="198" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A198" t="s">
+        <v>339</v>
+      </c>
+      <c r="B198" t="s">
+        <v>84</v>
+      </c>
+      <c r="C198" t="s">
+        <v>328</v>
+      </c>
+      <c r="D198" t="s">
+        <v>340</v>
+      </c>
+      <c r="E198" s="3">
+        <v>2020</v>
+      </c>
+      <c r="F198" t="s">
+        <v>81</v>
+      </c>
+      <c r="G198" t="s">
+        <v>82</v>
+      </c>
+      <c r="H198" s="3"/>
+      <c r="J198" s="3"/>
+      <c r="L198" s="3"/>
+      <c r="N198" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="199" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A199" t="s">
+        <v>341</v>
+      </c>
+      <c r="B199" t="s">
+        <v>84</v>
+      </c>
+      <c r="C199" t="s">
+        <v>328</v>
+      </c>
+      <c r="D199" t="s">
+        <v>342</v>
+      </c>
+      <c r="E199" s="3">
+        <v>2020</v>
+      </c>
+      <c r="F199" t="s">
+        <v>81</v>
+      </c>
+      <c r="G199" t="s">
+        <v>82</v>
+      </c>
+      <c r="H199" s="3"/>
+      <c r="J199" s="3"/>
+      <c r="L199" s="3"/>
+      <c r="N199" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="200" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A200" t="s">
+        <v>343</v>
+      </c>
+      <c r="B200" t="s">
+        <v>84</v>
+      </c>
+      <c r="C200" t="s">
+        <v>328</v>
+      </c>
+      <c r="D200" t="s">
+        <v>342</v>
+      </c>
+      <c r="E200" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="F200" t="s">
+        <v>81</v>
+      </c>
+      <c r="G200" t="s">
+        <v>82</v>
+      </c>
+      <c r="H200" s="3"/>
+      <c r="J200" s="3"/>
+      <c r="L200" s="3"/>
+      <c r="N200" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="201" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A201" t="s">
+        <v>344</v>
+      </c>
+      <c r="B201" t="s">
+        <v>84</v>
+      </c>
+      <c r="C201" t="s">
+        <v>328</v>
+      </c>
+      <c r="D201" t="s">
+        <v>329</v>
+      </c>
+      <c r="E201" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="F201" t="s">
+        <v>81</v>
+      </c>
+      <c r="G201" t="s">
+        <v>82</v>
+      </c>
+      <c r="H201" s="3"/>
+      <c r="J201" s="3"/>
+      <c r="L201" s="3"/>
+      <c r="N201" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="202" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A202" t="s">
+        <v>345</v>
+      </c>
+      <c r="B202" t="s">
+        <v>84</v>
+      </c>
+      <c r="C202" t="s">
+        <v>328</v>
+      </c>
+      <c r="D202" t="s">
+        <v>346</v>
+      </c>
+      <c r="E202" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="F202" t="s">
+        <v>81</v>
+      </c>
+      <c r="G202" t="s">
+        <v>82</v>
+      </c>
+      <c r="H202" s="3"/>
+      <c r="J202" s="3"/>
+      <c r="L202" s="3"/>
+      <c r="N202" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="203" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A203" t="s">
+        <v>347</v>
+      </c>
+      <c r="B203" t="s">
+        <v>84</v>
+      </c>
+      <c r="C203" t="s">
+        <v>328</v>
+      </c>
+      <c r="D203" t="s">
+        <v>348</v>
+      </c>
+      <c r="E203" s="3">
+        <v>2015</v>
+      </c>
+      <c r="F203" t="s">
+        <v>81</v>
+      </c>
+      <c r="G203" t="s">
+        <v>82</v>
+      </c>
+      <c r="H203" s="3"/>
+      <c r="J203" s="3"/>
+      <c r="L203" s="3"/>
+      <c r="N203" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="204" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A204" t="s">
+        <v>349</v>
+      </c>
+      <c r="B204" t="s">
+        <v>84</v>
+      </c>
+      <c r="C204" t="s">
+        <v>350</v>
+      </c>
+      <c r="D204" t="s">
+        <v>351</v>
+      </c>
+      <c r="E204" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F204" t="s">
+        <v>81</v>
+      </c>
+      <c r="G204" t="s">
+        <v>82</v>
+      </c>
+      <c r="H204" s="3"/>
+      <c r="J204" s="3"/>
+      <c r="L204" s="3"/>
+      <c r="N204" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="205" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A205" t="s">
+        <v>353</v>
+      </c>
+      <c r="B205" t="s">
+        <v>84</v>
+      </c>
+      <c r="C205" t="s">
+        <v>350</v>
+      </c>
+      <c r="D205" t="s">
+        <v>354</v>
+      </c>
+      <c r="E205" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F205" t="s">
+        <v>81</v>
+      </c>
+      <c r="G205" t="s">
+        <v>82</v>
+      </c>
+      <c r="H205" s="3"/>
+      <c r="J205" s="3"/>
+      <c r="L205" s="3"/>
+      <c r="N205" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="206" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A206" t="s">
+        <v>356</v>
+      </c>
+      <c r="B206" t="s">
+        <v>84</v>
+      </c>
+      <c r="C206" t="s">
+        <v>350</v>
+      </c>
+      <c r="D206" t="s">
+        <v>357</v>
+      </c>
+      <c r="E206" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F206" t="s">
+        <v>81</v>
+      </c>
+      <c r="G206" t="s">
+        <v>82</v>
+      </c>
+      <c r="H206" s="3"/>
+      <c r="J206" s="3"/>
+      <c r="L206" s="3"/>
+      <c r="N206" t="s">
         <v>358</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
updated missing cameroon dataset from whisp_columns.xlsx
</commit_message>
<xml_diff>
--- a/whisp_columns.xlsx
+++ b/whisp_columns.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnell\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0CAFD05-62BA-4718-B43D-46F81171967B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DDF8C9-FFFF-4F96-A986-405CD27793AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="whisp outputs global" sheetId="1" r:id="rId1"/>
+    <sheet name="whisp outputs standard" sheetId="1" r:id="rId1"/>
     <sheet name="whisp outputs national" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1549" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1558" uniqueCount="399">
   <si>
     <t>Column name</t>
   </si>
@@ -1094,9 +1094,6 @@
     <t>nCO_ideam_eufo_commission_2020</t>
   </si>
   <si>
-    <t>Area of Treecover outside EUFO</t>
-  </si>
-  <si>
     <t>nBR_INPE_TC_primary_forest_Amazon_2020</t>
   </si>
   <si>
@@ -1212,6 +1209,15 @@
   </si>
   <si>
     <t>BNETD 2020.</t>
+  </si>
+  <si>
+    <t>Area of Tree cover outside EUFO</t>
+  </si>
+  <si>
+    <t>nCM_Treecover_2020</t>
+  </si>
+  <si>
+    <t>Area of Treecover</t>
   </si>
 </sst>
 </file>
@@ -1233,14 +1239,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1309,26 +1315,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8306,1112 +8310,1197 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06C9A24C-67E0-477E-A2C1-2524EF892E56}">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="N1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="5">
         <v>2020</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="H2" s="5">
-        <v>1</v>
-      </c>
-      <c r="I2" s="6" t="s">
+      <c r="G2" s="2"/>
+      <c r="H2" s="6">
+        <v>1</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J2" s="6">
+        <v>1</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L2" s="6">
+        <v>1</v>
+      </c>
+      <c r="M2" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="J2" s="5">
-        <v>1</v>
-      </c>
-      <c r="K2" s="6" t="s">
+      <c r="N2" s="2"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="E3" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="6">
+        <v>1</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="L2" s="5">
-        <v>1</v>
-      </c>
-      <c r="M2" s="6" t="s">
+      <c r="J3" s="6">
+        <v>1</v>
+      </c>
+      <c r="K3" s="7" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>356</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="L3" s="6">
+        <v>1</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="N3" s="2"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="E3" s="4">
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="5">
         <v>2020</v>
       </c>
-      <c r="F3" t="s">
-        <v>355</v>
-      </c>
-      <c r="H3" s="5">
-        <v>1</v>
-      </c>
-      <c r="I3" s="6" t="s">
+      <c r="F4" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="6">
+        <v>1</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J4" s="6">
+        <v>1</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L4" s="6">
+        <v>1</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N4" s="2"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="6">
+        <v>1</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J5" s="6">
+        <v>1</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L5" s="6">
+        <v>1</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="N5" s="2"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="6">
+        <v>1</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J6" s="6">
+        <v>1</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L6" s="6">
+        <v>1</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N6" s="2"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="6">
+        <v>1</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J7" s="6">
+        <v>1</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L7" s="6">
+        <v>1</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N7" s="2"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="6">
+        <v>1</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J8" s="6">
+        <v>1</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L8" s="6">
+        <v>1</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N8" s="2"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="G9" s="2"/>
+      <c r="H9" s="6">
+        <v>1</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J9" s="6">
+        <v>1</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L9" s="6">
+        <v>1</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N9" s="2"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="6">
+        <v>1</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J10" s="6">
+        <v>1</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L10" s="6">
+        <v>1</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="N10" s="2"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="6">
+        <v>1</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J11" s="6">
+        <v>1</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L11" s="6">
+        <v>1</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="N11" s="2"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="G12" s="2"/>
+      <c r="H12" s="6">
+        <v>1</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J12" s="6">
+        <v>1</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" s="6">
+        <v>1</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="N12" s="2"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="6">
+        <v>1</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" s="6">
+        <v>1</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L13" s="6">
+        <v>1</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="N13" s="2"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="6">
+        <v>1</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J14" s="6">
+        <v>1</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L14" s="6">
+        <v>1</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="N14" s="2"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="G15" s="2"/>
+      <c r="H15" s="6">
+        <v>1</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="J15" s="6">
+        <v>1</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="L15" s="6">
+        <v>1</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="N15" s="2"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="6">
+        <v>1</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="J16" s="6">
+        <v>1</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="L16" s="6">
+        <v>1</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="N16" s="2"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="G17" s="2"/>
+      <c r="H17" s="6">
+        <v>1</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="J17" s="6">
+        <v>1</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="L17" s="6">
+        <v>1</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="G18" s="2"/>
+      <c r="H18" s="6">
+        <v>1</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="J18" s="6">
+        <v>1</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="L18" s="6">
+        <v>1</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="E19" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" s="6">
+        <v>1</v>
+      </c>
+      <c r="I19" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="J3" s="5">
-        <v>1</v>
-      </c>
-      <c r="K3" s="6" t="s">
+      <c r="J19" s="6">
+        <v>1</v>
+      </c>
+      <c r="K19" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="L3" s="5">
-        <v>1</v>
-      </c>
-      <c r="M3" s="6" t="s">
+      <c r="L19" s="6">
+        <v>1</v>
+      </c>
+      <c r="M19" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>358</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" s="4">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E20" s="5">
         <v>2020</v>
       </c>
-      <c r="F4" t="s">
-        <v>359</v>
-      </c>
-      <c r="H4" s="5">
-        <v>1</v>
-      </c>
-      <c r="I4" s="6" t="s">
+      <c r="F20" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G20" s="2"/>
+      <c r="H20" s="6">
+        <v>1</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J20" s="6">
+        <v>1</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L20" s="6">
+        <v>1</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E21" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="6">
+        <v>1</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J21" s="6">
+        <v>1</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L21" s="6">
+        <v>1</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="E22" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G22" s="2"/>
+      <c r="H22" s="6">
+        <v>1</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J22" s="6">
+        <v>1</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L22" s="6">
+        <v>1</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="G23" s="2"/>
+      <c r="H23" s="6">
+        <v>1</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J23" s="6">
+        <v>1</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L23" s="6">
+        <v>1</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E24" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="6">
+        <v>1</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J24" s="6">
+        <v>1</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L24" s="6">
+        <v>1</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="E25" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="H25" s="6">
+        <v>1</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J25" s="6">
+        <v>1</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L25" s="6">
+        <v>1</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E26" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="6">
+        <v>1</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J26" s="6">
+        <v>1</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L26" s="6">
+        <v>1</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E27" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="G27" s="2"/>
+      <c r="H27" s="6">
+        <v>1</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J27" s="6">
+        <v>1</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L27" s="6">
+        <v>1</v>
+      </c>
+      <c r="M27" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E28" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="G28" s="2"/>
+      <c r="H28" s="6">
+        <v>1</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J28" s="6">
+        <v>1</v>
+      </c>
+      <c r="K28" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L28" s="6">
+        <v>1</v>
+      </c>
+      <c r="M28" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E29" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="G29" s="2"/>
+      <c r="H29" s="6">
+        <v>1</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="J29" s="6">
+        <v>1</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L29" s="6">
+        <v>1</v>
+      </c>
+      <c r="M29" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="E30" s="5">
+        <v>2020</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="G30" s="2"/>
+      <c r="H30" s="6">
+        <v>1</v>
+      </c>
+      <c r="I30" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="J4" s="5">
-        <v>1</v>
-      </c>
-      <c r="K4" s="6" t="s">
+      <c r="J30" s="6">
+        <v>1</v>
+      </c>
+      <c r="K30" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="L4" s="5">
-        <v>1</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>360</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F5" t="s">
-        <v>359</v>
-      </c>
-      <c r="H5" s="5">
-        <v>1</v>
-      </c>
-      <c r="I5" s="6" t="s">
+      <c r="L30" s="6">
+        <v>1</v>
+      </c>
+      <c r="M30" s="7" t="s">
         <v>53</v>
-      </c>
-      <c r="J5" s="5">
-        <v>1</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L5" s="5">
-        <v>1</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>361</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E6" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F6" t="s">
-        <v>362</v>
-      </c>
-      <c r="H6" s="5">
-        <v>1</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J6" s="5">
-        <v>1</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L6" s="5">
-        <v>1</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>363</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" t="s">
-        <v>51</v>
-      </c>
-      <c r="E7" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F7" t="s">
-        <v>362</v>
-      </c>
-      <c r="H7" s="5">
-        <v>1</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J7" s="5">
-        <v>1</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L7" s="5">
-        <v>1</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>364</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" t="s">
-        <v>51</v>
-      </c>
-      <c r="E8" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F8" t="s">
-        <v>362</v>
-      </c>
-      <c r="H8" s="5">
-        <v>1</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J8" s="5">
-        <v>1</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L8" s="5">
-        <v>1</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>365</v>
-      </c>
-      <c r="B9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E9" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F9" t="s">
-        <v>362</v>
-      </c>
-      <c r="H9" s="5">
-        <v>1</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J9" s="5">
-        <v>1</v>
-      </c>
-      <c r="K9" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L9" s="5">
-        <v>1</v>
-      </c>
-      <c r="M9" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>366</v>
-      </c>
-      <c r="B10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D10" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F10" t="s">
-        <v>362</v>
-      </c>
-      <c r="H10" s="5">
-        <v>1</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J10" s="5">
-        <v>1</v>
-      </c>
-      <c r="K10" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L10" s="5">
-        <v>1</v>
-      </c>
-      <c r="M10" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>367</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" t="s">
-        <v>64</v>
-      </c>
-      <c r="E11" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F11" t="s">
-        <v>368</v>
-      </c>
-      <c r="H11" s="5">
-        <v>1</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J11" s="5">
-        <v>1</v>
-      </c>
-      <c r="K11" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L11" s="5">
-        <v>1</v>
-      </c>
-      <c r="M11" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>369</v>
-      </c>
-      <c r="B12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E12" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F12" t="s">
-        <v>370</v>
-      </c>
-      <c r="H12" s="5">
-        <v>1</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J12" s="5">
-        <v>1</v>
-      </c>
-      <c r="K12" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L12" s="5">
-        <v>1</v>
-      </c>
-      <c r="M12" s="6" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>371</v>
-      </c>
-      <c r="B13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" t="s">
-        <v>50</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F13" t="s">
-        <v>372</v>
-      </c>
-      <c r="H13" s="5">
-        <v>1</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J13" s="5">
-        <v>1</v>
-      </c>
-      <c r="K13" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L13" s="5">
-        <v>1</v>
-      </c>
-      <c r="M13" s="6" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>373</v>
-      </c>
-      <c r="B14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E14" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F14" t="s">
-        <v>368</v>
-      </c>
-      <c r="H14" s="5">
-        <v>1</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="J14" s="5">
-        <v>1</v>
-      </c>
-      <c r="K14" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="L14" s="5">
-        <v>1</v>
-      </c>
-      <c r="M14" s="6" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>374</v>
-      </c>
-      <c r="B15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" t="s">
-        <v>50</v>
-      </c>
-      <c r="D15" t="s">
-        <v>93</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>375</v>
-      </c>
-      <c r="F15" t="s">
-        <v>359</v>
-      </c>
-      <c r="H15" s="5">
-        <v>1</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="J15" s="5">
-        <v>1</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="L15" s="5">
-        <v>1</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>376</v>
-      </c>
-      <c r="B16" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" t="s">
-        <v>119</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>377</v>
-      </c>
-      <c r="F16" t="s">
-        <v>378</v>
-      </c>
-      <c r="H16" s="5">
-        <v>1</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="J16" s="5">
-        <v>1</v>
-      </c>
-      <c r="K16" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="L16" s="5">
-        <v>1</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>379</v>
-      </c>
-      <c r="B17" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" t="s">
-        <v>50</v>
-      </c>
-      <c r="D17" t="s">
-        <v>93</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="F17" t="s">
-        <v>359</v>
-      </c>
-      <c r="H17" s="5">
-        <v>1</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="J17" s="5">
-        <v>1</v>
-      </c>
-      <c r="K17" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="L17" s="5">
-        <v>1</v>
-      </c>
-      <c r="M17" s="6" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>381</v>
-      </c>
-      <c r="B18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" t="s">
-        <v>50</v>
-      </c>
-      <c r="D18" t="s">
-        <v>119</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="F18" t="s">
-        <v>378</v>
-      </c>
-      <c r="H18" s="5">
-        <v>1</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="J18" s="5">
-        <v>1</v>
-      </c>
-      <c r="K18" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="L18" s="5">
-        <v>1</v>
-      </c>
-      <c r="M18" s="6" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>382</v>
-      </c>
-      <c r="B19" t="s">
-        <v>15</v>
-      </c>
-      <c r="C19" t="s">
-        <v>50</v>
-      </c>
-      <c r="D19" t="s">
-        <v>383</v>
-      </c>
-      <c r="E19" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F19" t="s">
-        <v>370</v>
-      </c>
-      <c r="H19" s="5">
-        <v>1</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J19" s="5">
-        <v>1</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L19" s="5">
-        <v>1</v>
-      </c>
-      <c r="M19" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>384</v>
-      </c>
-      <c r="B20" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" t="s">
-        <v>80</v>
-      </c>
-      <c r="E20" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F20" t="s">
-        <v>368</v>
-      </c>
-      <c r="H20" s="5">
-        <v>1</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J20" s="5">
-        <v>1</v>
-      </c>
-      <c r="K20" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L20" s="5">
-        <v>1</v>
-      </c>
-      <c r="M20" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>385</v>
-      </c>
-      <c r="B21" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" t="s">
-        <v>50</v>
-      </c>
-      <c r="D21" t="s">
-        <v>76</v>
-      </c>
-      <c r="E21" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F21" t="s">
-        <v>368</v>
-      </c>
-      <c r="H21" s="5">
-        <v>1</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J21" s="5">
-        <v>1</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L21" s="5">
-        <v>1</v>
-      </c>
-      <c r="M21" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>386</v>
-      </c>
-      <c r="B22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" t="s">
-        <v>50</v>
-      </c>
-      <c r="D22" t="s">
-        <v>383</v>
-      </c>
-      <c r="E22" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F22" t="s">
-        <v>368</v>
-      </c>
-      <c r="H22" s="5">
-        <v>1</v>
-      </c>
-      <c r="I22" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J22" s="5">
-        <v>1</v>
-      </c>
-      <c r="K22" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L22" s="5">
-        <v>1</v>
-      </c>
-      <c r="M22" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>387</v>
-      </c>
-      <c r="B23" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" t="s">
-        <v>50</v>
-      </c>
-      <c r="D23" t="s">
-        <v>388</v>
-      </c>
-      <c r="E23" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F23" t="s">
-        <v>370</v>
-      </c>
-      <c r="H23" s="5">
-        <v>1</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J23" s="5">
-        <v>1</v>
-      </c>
-      <c r="K23" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L23" s="5">
-        <v>1</v>
-      </c>
-      <c r="M23" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>389</v>
-      </c>
-      <c r="B24" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" t="s">
-        <v>50</v>
-      </c>
-      <c r="D24" t="s">
-        <v>90</v>
-      </c>
-      <c r="E24" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F24" t="s">
-        <v>368</v>
-      </c>
-      <c r="H24" s="5">
-        <v>1</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J24" s="5">
-        <v>1</v>
-      </c>
-      <c r="K24" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L24" s="5">
-        <v>1</v>
-      </c>
-      <c r="M24" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>390</v>
-      </c>
-      <c r="B25" t="s">
-        <v>15</v>
-      </c>
-      <c r="C25" t="s">
-        <v>50</v>
-      </c>
-      <c r="D25" t="s">
-        <v>388</v>
-      </c>
-      <c r="E25" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F25" t="s">
-        <v>368</v>
-      </c>
-      <c r="H25" s="5">
-        <v>1</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J25" s="5">
-        <v>1</v>
-      </c>
-      <c r="K25" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L25" s="5">
-        <v>1</v>
-      </c>
-      <c r="M25" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>391</v>
-      </c>
-      <c r="B26" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" t="s">
-        <v>50</v>
-      </c>
-      <c r="D26" t="s">
-        <v>392</v>
-      </c>
-      <c r="E26" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F26" t="s">
-        <v>370</v>
-      </c>
-      <c r="H26" s="5">
-        <v>1</v>
-      </c>
-      <c r="I26" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J26" s="5">
-        <v>1</v>
-      </c>
-      <c r="K26" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L26" s="5">
-        <v>1</v>
-      </c>
-      <c r="M26" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>393</v>
-      </c>
-      <c r="B27" t="s">
-        <v>15</v>
-      </c>
-      <c r="C27" t="s">
-        <v>50</v>
-      </c>
-      <c r="D27" t="s">
-        <v>392</v>
-      </c>
-      <c r="E27" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F27" t="s">
-        <v>372</v>
-      </c>
-      <c r="H27" s="5">
-        <v>1</v>
-      </c>
-      <c r="I27" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J27" s="5">
-        <v>1</v>
-      </c>
-      <c r="K27" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L27" s="5">
-        <v>1</v>
-      </c>
-      <c r="M27" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>394</v>
-      </c>
-      <c r="B28" t="s">
-        <v>15</v>
-      </c>
-      <c r="C28" t="s">
-        <v>50</v>
-      </c>
-      <c r="D28" t="s">
-        <v>392</v>
-      </c>
-      <c r="E28" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F28" t="s">
-        <v>368</v>
-      </c>
-      <c r="H28" s="5">
-        <v>1</v>
-      </c>
-      <c r="I28" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J28" s="5">
-        <v>1</v>
-      </c>
-      <c r="K28" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L28" s="5">
-        <v>1</v>
-      </c>
-      <c r="M28" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>395</v>
-      </c>
-      <c r="B29" t="s">
-        <v>15</v>
-      </c>
-      <c r="C29" t="s">
-        <v>50</v>
-      </c>
-      <c r="D29" t="s">
-        <v>82</v>
-      </c>
-      <c r="E29" s="4">
-        <v>2020</v>
-      </c>
-      <c r="F29" t="s">
-        <v>396</v>
-      </c>
-      <c r="H29" s="5">
-        <v>1</v>
-      </c>
-      <c r="I29" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J29" s="5">
-        <v>1</v>
-      </c>
-      <c r="K29" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="L29" s="5">
-        <v>1</v>
-      </c>
-      <c r="M29" s="6" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync docs and comments to the 2024 dataset refresh; refresh README timber decision tree; add caveat that diagram datasets are examples; fix two LUT corresponding_variable entries
Follow-up to #200. Updates leftover 2023 vintage references to 2024 in datasets.py and risk.py comments, the README timber categories, and the renamed rows in whisp_columns.xlsx, and swaps the timber decision tree image for the 2024 version. Also corrects the corresponding_variable for Coffee_FDaP and GFW_logging_before_2020 (a metadata field, not used at runtime). No change to risk outputs.
</commit_message>
<xml_diff>
--- a/whisp_columns.xlsx
+++ b/whisp_columns.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnell\Documents\GitHub\whisp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D95A118C-1FBF-48D2-B9F7-1C3A73A32E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61D0EBD5-1733-49F6-88F7-50B81C5557CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -899,48 +899,24 @@
     <t>Assumes management continues to 2020</t>
   </si>
   <si>
-    <t>TMF_regrowth_2023</t>
-  </si>
-  <si>
     <t>Area of Regrowth</t>
   </si>
   <si>
     <t>treecover_after_2020</t>
   </si>
   <si>
-    <t>ESRI_2023_TC</t>
-  </si>
-  <si>
     <t>Area of Tree cover</t>
   </si>
   <si>
     <t>Karra 2021</t>
   </si>
   <si>
-    <t>Oil_palm_2023_FDaP</t>
-  </si>
-  <si>
     <t>agri_after_2020</t>
   </si>
   <si>
-    <t>Rubber_2023_FDaP</t>
-  </si>
-  <si>
-    <t>Coffee_FDaP_2023</t>
-  </si>
-  <si>
-    <t>Cocoa_2023_FDaP</t>
-  </si>
-  <si>
-    <t>ESRI_crop_gain_2020_2023</t>
-  </si>
-  <si>
     <t>Area of Crop</t>
   </si>
   <si>
-    <t>2020 and 2023</t>
-  </si>
-  <si>
     <t>GFW_logging_before_2020</t>
   </si>
   <si>
@@ -1197,6 +1173,30 @@
   </si>
   <si>
     <t>Area of Treecover</t>
+  </si>
+  <si>
+    <t>TMF_regrowth_2024</t>
+  </si>
+  <si>
+    <t>ESRI_2024_TC</t>
+  </si>
+  <si>
+    <t>Oil_palm_2024_FDaP</t>
+  </si>
+  <si>
+    <t>Rubber_2024_FDaP</t>
+  </si>
+  <si>
+    <t>Coffee_FDaP_2024</t>
+  </si>
+  <si>
+    <t>Cocoa_2024_FDaP</t>
+  </si>
+  <si>
+    <t>ESRI_crop_gain_2020_2024</t>
+  </si>
+  <si>
+    <t>2020 and 2024</t>
   </si>
 </sst>
 </file>
@@ -7492,19 +7492,19 @@
     </row>
     <row r="197" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
+        <v>384</v>
+      </c>
+      <c r="B197" t="s">
+        <v>15</v>
+      </c>
+      <c r="C197" t="s">
+        <v>50</v>
+      </c>
+      <c r="D197" t="s">
         <v>292</v>
       </c>
-      <c r="B197" t="s">
-        <v>15</v>
-      </c>
-      <c r="C197" t="s">
-        <v>50</v>
-      </c>
-      <c r="D197" t="s">
-        <v>293</v>
-      </c>
       <c r="E197">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F197" t="s">
         <v>62</v>
@@ -7522,28 +7522,28 @@
         <v>1</v>
       </c>
       <c r="M197" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="198" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
+        <v>385</v>
+      </c>
+      <c r="B198" t="s">
+        <v>15</v>
+      </c>
+      <c r="C198" t="s">
+        <v>50</v>
+      </c>
+      <c r="D198" t="s">
+        <v>294</v>
+      </c>
+      <c r="E198">
+        <v>2024</v>
+      </c>
+      <c r="F198" t="s">
         <v>295</v>
       </c>
-      <c r="B198" t="s">
-        <v>15</v>
-      </c>
-      <c r="C198" t="s">
-        <v>50</v>
-      </c>
-      <c r="D198" t="s">
-        <v>296</v>
-      </c>
-      <c r="E198">
-        <v>2023</v>
-      </c>
-      <c r="F198" t="s">
-        <v>297</v>
-      </c>
       <c r="H198">
         <v>0</v>
       </c>
@@ -7554,12 +7554,12 @@
         <v>1</v>
       </c>
       <c r="M198" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="199" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
-        <v>298</v>
+        <v>386</v>
       </c>
       <c r="B199" t="s">
         <v>15</v>
@@ -7571,7 +7571,7 @@
         <v>75</v>
       </c>
       <c r="E199">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F199" t="s">
         <v>68</v>
@@ -7589,12 +7589,12 @@
         <v>1</v>
       </c>
       <c r="M199" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="200" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
-        <v>300</v>
+        <v>387</v>
       </c>
       <c r="B200" t="s">
         <v>15</v>
@@ -7606,7 +7606,7 @@
         <v>85</v>
       </c>
       <c r="E200">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F200" t="s">
         <v>68</v>
@@ -7624,12 +7624,12 @@
         <v>1</v>
       </c>
       <c r="M200" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="201" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
-        <v>301</v>
+        <v>388</v>
       </c>
       <c r="B201" t="s">
         <v>15</v>
@@ -7641,7 +7641,7 @@
         <v>79</v>
       </c>
       <c r="E201">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F201" t="s">
         <v>68</v>
@@ -7659,12 +7659,12 @@
         <v>1</v>
       </c>
       <c r="M201" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="202" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
-        <v>302</v>
+        <v>389</v>
       </c>
       <c r="B202" t="s">
         <v>15</v>
@@ -7676,7 +7676,7 @@
         <v>81</v>
       </c>
       <c r="E202">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F202" t="s">
         <v>68</v>
@@ -7694,12 +7694,12 @@
         <v>1</v>
       </c>
       <c r="M202" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="203" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
-        <v>303</v>
+        <v>390</v>
       </c>
       <c r="B203" t="s">
         <v>15</v>
@@ -7708,13 +7708,13 @@
         <v>50</v>
       </c>
       <c r="D203" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="E203" t="s">
-        <v>305</v>
+        <v>391</v>
       </c>
       <c r="F203" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="G203" t="s">
         <v>18</v>
@@ -7729,12 +7729,12 @@
         <v>1</v>
       </c>
       <c r="M203" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="204" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="B204" t="s">
         <v>15</v>
@@ -7743,13 +7743,13 @@
         <v>50</v>
       </c>
       <c r="D204" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="E204">
         <v>2015</v>
       </c>
       <c r="F204" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="G204" t="s">
         <v>18</v>
@@ -7764,21 +7764,21 @@
         <v>1</v>
       </c>
       <c r="M204" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="N204" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
     </row>
     <row r="205" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="B205" t="s">
         <v>20</v>
       </c>
       <c r="D205" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="F205" t="s">
         <v>17</v>
@@ -7792,13 +7792,13 @@
     </row>
     <row r="206" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="B206" t="s">
         <v>20</v>
       </c>
       <c r="D206" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="F206" t="s">
         <v>17</v>
@@ -7806,16 +7806,16 @@
     </row>
     <row r="207" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="B207" t="s">
         <v>20</v>
       </c>
       <c r="C207" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D207" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="E207">
         <v>2020</v>
@@ -7827,21 +7827,21 @@
         <v>18</v>
       </c>
       <c r="N207" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="208" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="B208" t="s">
         <v>20</v>
       </c>
       <c r="C208" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D208" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="E208">
         <v>2020</v>
@@ -7853,21 +7853,21 @@
         <v>18</v>
       </c>
       <c r="N208" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="209" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="B209" t="s">
         <v>20</v>
       </c>
       <c r="C209" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D209" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="E209" t="s">
         <v>259</v>
@@ -7879,24 +7879,24 @@
         <v>18</v>
       </c>
       <c r="N209" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="210" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="B210" t="s">
         <v>20</v>
       </c>
       <c r="C210" t="s">
+        <v>308</v>
+      </c>
+      <c r="D210" t="s">
+        <v>314</v>
+      </c>
+      <c r="E210" t="s">
         <v>316</v>
-      </c>
-      <c r="D210" t="s">
-        <v>322</v>
-      </c>
-      <c r="E210" t="s">
-        <v>324</v>
       </c>
       <c r="F210" t="s">
         <v>17</v>
@@ -7905,21 +7905,21 @@
         <v>18</v>
       </c>
       <c r="N210" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="211" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="B211" t="s">
         <v>20</v>
       </c>
       <c r="C211" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D211" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="E211">
         <v>2020</v>
@@ -7931,21 +7931,21 @@
         <v>18</v>
       </c>
       <c r="N211" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="212" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="B212" t="s">
         <v>20</v>
       </c>
       <c r="C212" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D212" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="E212">
         <v>2020</v>
@@ -7957,21 +7957,21 @@
         <v>18</v>
       </c>
       <c r="N212" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="213" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="B213" t="s">
         <v>20</v>
       </c>
       <c r="C213" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D213" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="E213">
         <v>2020</v>
@@ -7983,24 +7983,24 @@
         <v>18</v>
       </c>
       <c r="N213" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="214" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="B214" t="s">
         <v>20</v>
       </c>
       <c r="C214" t="s">
+        <v>308</v>
+      </c>
+      <c r="D214" t="s">
+        <v>322</v>
+      </c>
+      <c r="E214" t="s">
         <v>316</v>
-      </c>
-      <c r="D214" t="s">
-        <v>330</v>
-      </c>
-      <c r="E214" t="s">
-        <v>324</v>
       </c>
       <c r="F214" t="s">
         <v>17</v>
@@ -8009,24 +8009,24 @@
         <v>18</v>
       </c>
       <c r="N214" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="215" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="B215" t="s">
         <v>20</v>
       </c>
       <c r="C215" t="s">
+        <v>308</v>
+      </c>
+      <c r="D215" t="s">
+        <v>309</v>
+      </c>
+      <c r="E215" t="s">
         <v>316</v>
-      </c>
-      <c r="D215" t="s">
-        <v>317</v>
-      </c>
-      <c r="E215" t="s">
-        <v>324</v>
       </c>
       <c r="F215" t="s">
         <v>17</v>
@@ -8035,24 +8035,24 @@
         <v>18</v>
       </c>
       <c r="N215" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="216" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="B216" t="s">
         <v>20</v>
       </c>
       <c r="C216" t="s">
+        <v>308</v>
+      </c>
+      <c r="D216" t="s">
+        <v>326</v>
+      </c>
+      <c r="E216" t="s">
         <v>316</v>
-      </c>
-      <c r="D216" t="s">
-        <v>334</v>
-      </c>
-      <c r="E216" t="s">
-        <v>324</v>
       </c>
       <c r="F216" t="s">
         <v>17</v>
@@ -8061,21 +8061,21 @@
         <v>18</v>
       </c>
       <c r="N216" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="217" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="B217" t="s">
         <v>20</v>
       </c>
       <c r="C217" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D217" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="E217">
         <v>2015</v>
@@ -8087,21 +8087,21 @@
         <v>18</v>
       </c>
       <c r="N217" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="218" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="B218" t="s">
         <v>20</v>
       </c>
       <c r="C218" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="D218" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="F218" t="s">
         <v>17</v>
@@ -8110,21 +8110,21 @@
         <v>18</v>
       </c>
       <c r="N218" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
     </row>
     <row r="219" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="B219" t="s">
         <v>20</v>
       </c>
       <c r="C219" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="D219" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="F219" t="s">
         <v>17</v>
@@ -8133,21 +8133,21 @@
         <v>18</v>
       </c>
       <c r="N219" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
     </row>
     <row r="220" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="B220" t="s">
         <v>20</v>
       </c>
       <c r="C220" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="D220" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="F220" t="s">
         <v>17</v>
@@ -8156,7 +8156,7 @@
         <v>18</v>
       </c>
       <c r="N220" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -8215,7 +8215,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="B2" t="s">
         <v>15</v>
@@ -8230,7 +8230,7 @@
         <v>2020</v>
       </c>
       <c r="F2" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="H2" s="5">
         <v>1</v>
@@ -8253,7 +8253,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -8262,13 +8262,13 @@
         <v>50</v>
       </c>
       <c r="D3" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="E3" s="4">
         <v>2020</v>
       </c>
       <c r="F3" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="H3" s="5">
         <v>1</v>
@@ -8291,7 +8291,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="B4" t="s">
         <v>15</v>
@@ -8306,7 +8306,7 @@
         <v>2020</v>
       </c>
       <c r="F4" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="H4" s="5">
         <v>1</v>
@@ -8329,7 +8329,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="B5" t="s">
         <v>15</v>
@@ -8344,7 +8344,7 @@
         <v>2020</v>
       </c>
       <c r="F5" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="H5" s="5">
         <v>1</v>
@@ -8367,7 +8367,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="B6" t="s">
         <v>15</v>
@@ -8382,7 +8382,7 @@
         <v>2020</v>
       </c>
       <c r="F6" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="H6" s="5">
         <v>1</v>
@@ -8405,7 +8405,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="B7" t="s">
         <v>15</v>
@@ -8420,7 +8420,7 @@
         <v>2020</v>
       </c>
       <c r="F7" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="H7" s="5">
         <v>1</v>
@@ -8443,7 +8443,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
@@ -8458,7 +8458,7 @@
         <v>2020</v>
       </c>
       <c r="F8" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="H8" s="5">
         <v>1</v>
@@ -8481,7 +8481,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
@@ -8496,7 +8496,7 @@
         <v>2020</v>
       </c>
       <c r="F9" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="H9" s="5">
         <v>1</v>
@@ -8519,7 +8519,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="B10" t="s">
         <v>15</v>
@@ -8534,7 +8534,7 @@
         <v>2020</v>
       </c>
       <c r="F10" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="H10" s="5">
         <v>1</v>
@@ -8557,7 +8557,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="B11" t="s">
         <v>15</v>
@@ -8572,7 +8572,7 @@
         <v>2020</v>
       </c>
       <c r="F11" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="H11" s="5">
         <v>1</v>
@@ -8595,7 +8595,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="B12" t="s">
         <v>15</v>
@@ -8610,7 +8610,7 @@
         <v>2020</v>
       </c>
       <c r="F12" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="H12" s="5">
         <v>1</v>
@@ -8633,7 +8633,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
@@ -8648,7 +8648,7 @@
         <v>2020</v>
       </c>
       <c r="F13" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="H13" s="5">
         <v>1</v>
@@ -8671,7 +8671,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="B14" t="s">
         <v>15</v>
@@ -8686,7 +8686,7 @@
         <v>2020</v>
       </c>
       <c r="F14" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="H14" s="5">
         <v>1</v>
@@ -8709,7 +8709,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="B15" t="s">
         <v>15</v>
@@ -8721,10 +8721,10 @@
         <v>92</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="F15" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="H15" s="5">
         <v>1</v>
@@ -8747,7 +8747,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="B16" t="s">
         <v>15</v>
@@ -8759,10 +8759,10 @@
         <v>118</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="F16" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="H16" s="5">
         <v>1</v>
@@ -8785,7 +8785,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="B17" t="s">
         <v>15</v>
@@ -8797,10 +8797,10 @@
         <v>92</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="F17" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="H17" s="5">
         <v>1</v>
@@ -8823,7 +8823,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="B18" t="s">
         <v>15</v>
@@ -8835,10 +8835,10 @@
         <v>118</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="F18" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="H18" s="5">
         <v>1</v>
@@ -8861,7 +8861,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="B19" t="s">
         <v>15</v>
@@ -8870,13 +8870,13 @@
         <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="E19" s="4">
         <v>2020</v>
       </c>
       <c r="F19" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="H19" s="5">
         <v>1</v>
@@ -8899,7 +8899,7 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="B20" t="s">
         <v>15</v>
@@ -8914,7 +8914,7 @@
         <v>2020</v>
       </c>
       <c r="F20" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="H20" s="5">
         <v>1</v>
@@ -8937,7 +8937,7 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
       <c r="B21" t="s">
         <v>15</v>
@@ -8952,7 +8952,7 @@
         <v>2020</v>
       </c>
       <c r="F21" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="H21" s="5">
         <v>1</v>
@@ -8975,7 +8975,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>379</v>
+        <v>371</v>
       </c>
       <c r="B22" t="s">
         <v>15</v>
@@ -8984,13 +8984,13 @@
         <v>50</v>
       </c>
       <c r="D22" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="E22" s="4">
         <v>2020</v>
       </c>
       <c r="F22" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="H22" s="5">
         <v>1</v>
@@ -9013,7 +9013,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>380</v>
+        <v>372</v>
       </c>
       <c r="B23" t="s">
         <v>15</v>
@@ -9022,13 +9022,13 @@
         <v>50</v>
       </c>
       <c r="D23" t="s">
-        <v>381</v>
+        <v>373</v>
       </c>
       <c r="E23" s="4">
         <v>2020</v>
       </c>
       <c r="F23" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="H23" s="5">
         <v>1</v>
@@ -9051,7 +9051,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
       <c r="B24" t="s">
         <v>15</v>
@@ -9066,7 +9066,7 @@
         <v>2020</v>
       </c>
       <c r="F24" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="H24" s="5">
         <v>1</v>
@@ -9089,7 +9089,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>383</v>
+        <v>375</v>
       </c>
       <c r="B25" t="s">
         <v>15</v>
@@ -9098,13 +9098,13 @@
         <v>50</v>
       </c>
       <c r="D25" t="s">
-        <v>381</v>
+        <v>373</v>
       </c>
       <c r="E25" s="4">
         <v>2020</v>
       </c>
       <c r="F25" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="H25" s="5">
         <v>1</v>
@@ -9127,7 +9127,7 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="B26" t="s">
         <v>15</v>
@@ -9136,13 +9136,13 @@
         <v>50</v>
       </c>
       <c r="D26" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="E26" s="4">
         <v>2020</v>
       </c>
       <c r="F26" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="H26" s="5">
         <v>1</v>
@@ -9165,7 +9165,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>386</v>
+        <v>378</v>
       </c>
       <c r="B27" t="s">
         <v>15</v>
@@ -9174,13 +9174,13 @@
         <v>50</v>
       </c>
       <c r="D27" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="E27" s="4">
         <v>2020</v>
       </c>
       <c r="F27" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="H27" s="5">
         <v>1</v>
@@ -9203,7 +9203,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="B28" t="s">
         <v>15</v>
@@ -9212,13 +9212,13 @@
         <v>50</v>
       </c>
       <c r="D28" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="E28" s="4">
         <v>2020</v>
       </c>
       <c r="F28" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="H28" s="5">
         <v>1</v>
@@ -9241,7 +9241,7 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="B29" t="s">
         <v>15</v>
@@ -9256,7 +9256,7 @@
         <v>2020</v>
       </c>
       <c r="F29" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="H29" s="5">
         <v>1</v>
@@ -9279,7 +9279,7 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="B30" t="s">
         <v>15</v>
@@ -9288,13 +9288,13 @@
         <v>50</v>
       </c>
       <c r="D30" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="E30" s="4">
         <v>2020</v>
       </c>
       <c r="F30" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="H30" s="5">
         <v>1</v>

</xml_diff>